<commit_message>
F2.2: verificar en navegador y documentar la 0.2.0 (S-01, S-07, S-08, G-07)
- V-02: lista de F1.1 en Chromium con el reproductor nuevo, ninguna
  petición externa, y 22 notas grabadas a la salida de audio, todas a
  menos de 1 cent de su nota en los dos timbres.
- La herramienta de navegador sirve para la 0.2.0 y para versiones
  anteriores, y graba cuerdas al aire y 1ª cuerda en los dos timbres.
- Requisitos v1.5: S-08 validado; S-01, S-07 y G-07 modificados (G-07
  anota que con doble clic suena el sintetizador hasta F2.3).
- Matriz 1.3, roadmap 3.3 (F1 cerrada con v0.1.5), CHANGELOG 0.2.0,
  créditos, compatibilidad y README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.2. Base: requisitos.md v1.4 · app 0.1.4 · roadmap 3.2 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.3. Base: requisitos.md v1.5 · app 0.2.0 · roadmap 3.3 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.4</t>
+          <t>Cambio en v1.5</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       <c r="P10" s="6" t="n"/>
       <c r="Q10" s="5" t="inlineStr"/>
     </row>
-    <row r="11" ht="78" customHeight="1">
+    <row r="11" ht="120" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>G-07</t>
@@ -1215,11 +1215,15 @@
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>Hoy funciona sin conexión pero con sonido sintetizado, porque los samples se descargan de internet. Se completa al incrustar el audio en el archivo (F2.3). En iPhone puede no ser viable: ver PL-03.</t>
+          <t>Se completa al incrustar el audio en el archivo (F2.3). Retroceso temporal desde la 0.2.0: al abrir con doble clic suena el sintetizador, porque los navegadores no dejan a una página local leer otros archivos; antes, con conexión, sonaban las grabaciones descargadas. Con Live Server y en la web suena la guitarra. En iPhone puede no ser viable: ver PL-03.</t>
         </is>
       </c>
       <c r="P11" s="6" t="n"/>
-      <c r="Q11" s="5" t="inlineStr"/>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="78" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -1693,11 +1697,7 @@
         </is>
       </c>
       <c r="P17" s="6" t="n"/>
-      <c r="Q17" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q17" s="5" t="inlineStr"/>
     </row>
     <row r="18" ht="120" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -1855,11 +1855,7 @@
         </is>
       </c>
       <c r="P19" s="6" t="n"/>
-      <c r="Q19" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="Q19" s="5" t="inlineStr"/>
     </row>
     <row r="20" ht="33" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
@@ -2785,7 +2781,7 @@
       <c r="P31" s="6" t="n"/>
       <c r="Q31" s="5" t="inlineStr"/>
     </row>
-    <row r="32" ht="93" customHeight="1">
+    <row r="32" ht="120" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>S-01</t>
@@ -2858,11 +2854,15 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>Hoy con Tone.js y samples de un tercero, ya copiados en samples/ (F2.1). En F2 se sustituye por un reproductor propio que los usa (S-07). La 0.1.3 corrige el registro agudo de la guitarra clásica, que sonaba medio tono alto (S-08).</t>
+          <t>Desde la 0.2.0 suena con un reproductor propio y las grabaciones de samples/, sin Tone.js (F2.2). Grabado en el navegador, de la 6ª al aire al traste 24 de la 1ª y en los dos timbres, cada nota suena a menos de 1 cent de su frecuencia. La 0.1.3 corrigió el registro agudo de la guitarra clásica, que sonaba medio tono alto (S-08).</t>
         </is>
       </c>
       <c r="P32" s="6" t="n"/>
-      <c r="Q32" s="5" t="inlineStr"/>
+      <c r="Q32" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="63" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -3309,7 +3309,7 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>CREDITOS.md y samples/ (F2.1). La app aún descarga el audio de fuera</t>
+          <t>CREDITOS.md y samples/ (F2.1) · Banco (node --test): ninguna dirección externa (0.2.0)</t>
         </is>
       </c>
       <c r="M38" s="5" t="inlineStr">
@@ -3324,11 +3324,15 @@
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>Opción A, decidida el 14/10. Hecho en F2.1: licencias verificadas y los 16 archivos en samples/, con CREDITOS.md. Falta que la app los use en lugar de descargarlos (F2.2), meterlos en el archivo (F2.3) y confirmar, antes de F2.3, que todos los sonidos del pack de nylon comparten la licencia comprobada en uno de ellos.</t>
+          <t>Opción A, decidida el 14/10. Hecho: licencias verificadas y los 16 archivos en samples/, con CREDITOS.md (F2.1); desde la 0.2.0 la app los usa y no descarga nada de otros servidores (F2.2). Falta meterlos en el archivo (F2.3) y confirmar, antes de F2.3, que todos los sonidos del pack de nylon comparten la licencia comprobada en uno de ellos.</t>
         </is>
       </c>
       <c r="P38" s="6" t="n"/>
-      <c r="Q38" s="5" t="inlineStr"/>
+      <c r="Q38" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="120" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -3388,12 +3392,12 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>samples/afinacion.json · Banco (node --test): muestras. Falta que la app use samples/ (F2.2)</t>
+          <t>samples/afinacion.json · Banco (node --test): muestras y todas las notas · V-02: 22 notas grabadas en el navegador, a menos de 1 cent</t>
         </is>
       </c>
       <c r="M39" s="5" t="inlineStr">
         <is>
-          <t>Verificado parcialmente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N39" s="5" t="inlineStr">
@@ -3403,11 +3407,15 @@
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>Origen: la medición de F2.1 encontró que el D5.mp3 de nylon suena en Re♯5 (+101 cents); con la 0.1.2, todo el registro agudo de la guitarra clásica sonaba medio tono alto. Sostiene también la precisión del afinador por referencia (A-01). Hoy lo demuestran la medición de las copias de samples/ y una prueba del banco; queda validado cuando la app use esas copias (F2.2). F2.4 lo aplica a cada muestra nueva.</t>
+          <t>Origen: la medición de F2.1 encontró que el D5.mp3 de nylon suena en Re♯5 (+101 cents); con la 0.1.2, todo el registro agudo de la guitarra clásica sonaba medio tono alto. Sostiene también la precisión del afinador por referencia (A-01). Validado en la 0.2.0: la app usa las copias medidas de samples/ y corrige su desviación; el banco lo comprueba para todas las notas posibles y la grabación en el navegador lo confirma (V-02). F2.4 lo aplica a cada muestra nueva.</t>
         </is>
       </c>
       <c r="P39" s="6" t="n"/>
-      <c r="Q39" s="5" t="inlineStr"/>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="78" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
@@ -7767,11 +7775,7 @@
         </is>
       </c>
       <c r="P95" s="6" t="n"/>
-      <c r="Q95" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q95" s="5" t="inlineStr"/>
     </row>
     <row r="96" ht="33" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
@@ -8581,7 +8585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8621,34 +8625,34 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -8658,7 +8662,7 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
@@ -8668,32 +8672,59 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F2.4: añadir la grabación aguda de nylon y reformular S-08 (S-01, S-08)
- samples/nylon/As5.mp3 (−10 cents medidos, corregidos al reproducir).
  En afinación estándar la clásica ya no transporta más de 6 semitonos
  (antes 12 en el traste 24); la acústica sigue en 14 por falta de
  grabaciones agudas en la fuente elegida. Versión 0.2.2.
- S-08 con la redacción aprobada por el cliente el 19/10: ±5 cents en la
  nota que suena tras la corrección; cada grabación es su nota y está
  medida. La prueba de grabaciones exige ahora menos de medio semitono, y
  la de todas las notas añade los límites de transporte de F2.4.
- dist/trasteando.html regenerado (1,46 MB). V-04: desde disco y sin
  conexión, notas a menos de 1 cent.
- Requisitos v1.7, matriz 1.5, roadmap 3.5, CHANGELOG y créditos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.4. Base: requisitos.md v1.6 · app 0.2.1 · roadmap 3.4 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.5. Base: requisitos.md v1.7 · app 0.2.2 · roadmap 3.5 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.6</t>
+          <t>Cambio en v1.7</t>
         </is>
       </c>
     </row>
@@ -1219,11 +1219,7 @@
         </is>
       </c>
       <c r="P11" s="6" t="n"/>
-      <c r="Q11" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -1302,11 +1298,7 @@
         </is>
       </c>
       <c r="P12" s="6" t="n"/>
-      <c r="Q12" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="63" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -2858,11 +2850,15 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>Desde la 0.2.0 suena con un reproductor propio y las grabaciones de samples/, sin Tone.js (F2.2). Grabado en el navegador, de la 6ª al aire al traste 24 de la 1ª y en los dos timbres, cada nota suena a menos de 1 cent de su frecuencia. La 0.1.3 corrigió el registro agudo de la guitarra clásica, que sonaba medio tono alto (S-08).</t>
+          <t>Reproductor propio con las grabaciones de samples/ desde la 0.2.0. Desde la 0.2.2 la guitarra clásica tiene también la grabación de La♯5: en afinación estándar ninguna nota se transporta más de 6 semitonos, y el traste 24 suena menos artificial. La acústica no tiene grabaciones por encima del Re5 y llega a 14. La 0.1.3 corrigió el registro agudo de nylon, que sonaba medio tono alto.</t>
         </is>
       </c>
       <c r="P32" s="6" t="n"/>
-      <c r="Q32" s="5" t="inlineStr"/>
+      <c r="Q32" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="63" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -3328,11 +3324,7 @@
         </is>
       </c>
       <c r="P38" s="6" t="n"/>
-      <c r="Q38" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q38" s="5" t="inlineStr"/>
     </row>
     <row r="39" ht="120" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -3347,7 +3339,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Cada muestra que usa la app suena en la nota a la que está asignada, con una desviación máxima de ±5 cents.</t>
+          <t>Cada nota suena a menos de 5 cents de su frecuencia, una vez corregida la desviación medida de su grabación. Cada grabación que usa la app es la nota a la que está asignada y tiene su desviación medida.</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -3377,7 +3369,7 @@
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>Medida con herramientas/medir-afinacion.py, cada muestra que usa la app suena a ±5 cents de la nota a la que está asignada; el banco lo comprueba contra la frecuencia medida y la huella sha256 de cada archivo.</t>
+          <t>Cada nota posible, en los dos timbres, suena a ±5 cents de su frecuencia una vez aplicada la corrección de su grabación; cada grabación es la nota asignada (a menos de 50 cents) y su desviación coincide con samples/afinacion.json.</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
@@ -3392,7 +3384,7 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>samples/afinacion.json · Banco (node --test): muestras y todas las notas · V-02: 22 notas grabadas en el navegador, a menos de 1 cent</t>
+          <t>samples/afinacion.json · Banco (node --test): grabaciones y todas las notas (±0,5 cents) · V-02, V-03 y V-04: notas grabadas en el navegador, a menos de 1 cent</t>
         </is>
       </c>
       <c r="M39" s="5" t="inlineStr">
@@ -3407,11 +3399,15 @@
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>Origen: la medición de F2.1 encontró que el D5.mp3 de nylon suena en Re♯5 (+101 cents); con la 0.1.2, todo el registro agudo de la guitarra clásica sonaba medio tono alto. Sostiene también la precisión del afinador por referencia (A-01). Validado en la 0.2.0: la app usa las copias medidas de samples/ y corrige su desviación; el banco lo comprueba para todas las notas posibles y la grabación en el navegador lo confirma (V-02). F2.4 lo aplica a cada muestra nueva.</t>
+          <t>Reformulado el 19/10, con tu aprobación: antes exigía ±5 cents a la grabación sin corregir; desde la 0.2.0 la app corrige cada grabación con su medida, así que lo que importa y se comprueba es la nota que suena. Origen: el D5.mp3 de nylon sonaba en Re♯5. Validado: el banco comprueba todas las notas posibles (±0,5 cents) y la grabación en el navegador lo confirma (V-02, V-03, V-04).</t>
         </is>
       </c>
       <c r="P39" s="6" t="n"/>
-      <c r="Q39" s="5" t="inlineStr"/>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="78" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
@@ -8581,7 +8577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8621,7 +8617,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -8631,24 +8627,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -8658,51 +8654,51 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -8712,7 +8708,7 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
@@ -8722,32 +8718,59 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
CP-2: guardar las auditorías AR-03 y AT-03 y aplicar sus cambios en documentos
- AR-03 y AT-03 con la respuesta a cada hallazgo.
- V-05: la escucha del cliente en su iPhone con la 0.2.0 (19/10).
- Requisitos v1.8: G-07 limitado a Windows y Android, con los límites
  de peso revisados; X-01 cumple; S-07 (licencia del pack de nylon, como
  tarde al cerrar F3); S-01 (escucha y agudo de la acústica). Dos
  decisiones nuevas: Service Worker y agudo de la acústica.
- Matriz 1.6, roadmap 3.6 (F2.1 y F2.4 cerradas, criterios de F2.3 y
  F2.5, despliegue de pruebas activo, Sesión 1 ampliada), CHANGELOG
  0.2.3, compatibilidad 1.1 y créditos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.5. Base: requisitos.md v1.7 · app 0.2.2 · roadmap 3.5 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.6. Base: requisitos.md v1.8 · app 0.2.3 · roadmap 3.6 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.7</t>
+          <t>Cambio en v1.8</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Modo archivo autónomo: la app funciona completa —salvo el afinador por micrófono— abriendo el archivo directamente (file://), sin servidor y sin conexión.</t>
+          <t>Modo archivo autónomo en Windows y Android: la app funciona completa —salvo el afinador por micrófono— abriendo el archivo directamente (file://), sin servidor y sin conexión. En iPhone, donde no se pueden abrir páginas desde Archivos, la autonomía llega por G-03.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Con el ordenador en modo avión, abrir el archivo con doble clic: suenan las muestras reales y funcionan Libre, Adivinar y el afinador por referencia.</t>
+          <t>En Windows (y Android cuando lo haya), con el ordenador en modo avión, dist/trasteando.html abre con doble clic en ≤ 3 s, suenan las grabaciones y funcionan Libre, Adivinar y el afinador por referencia. Audio ≤ 1,45 MB y archivo ≤ 2 MB.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>V-03: dist/trasteando.html desde disco y sin conexión en Chromium, abre en 0,6 s y suena a menos de 1 cent · Banco (node --test): autónomo al día y sin descargas</t>
+          <t>V-03 y V-04: desde disco y sin conexión en Chromium, abre en 0,3 s y suena a menos de 1 cent · Banco (node --test): autónomo al día, con su audio, huellas y límites</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
@@ -1215,11 +1215,15 @@
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>Desde la 0.2.1 es dist/trasteando.html: la app con sus 16 grabaciones dentro, recortadas a 4,5 s (1,42 MB). Abierto desde disco y sin conexión en Chromium abre en 0,6 s, suena con la guitarra real y no intenta ninguna conexión (V-03). index.html no lleva el audio dentro: con doble clic suena el sintetizador. Falta probarlo en cada plataforma (F2.5). En iPhone no es viable: ver PL-03.</t>
+          <t>dist/trasteando.html: la app con sus 17 grabaciones dentro (1,46 MB). Límites revisados en CP-2: el audio no pasa de 1,45 MB, y bajar su calidad exige tu escucha; el archivo entero no pasa de 2 MB, para dejar sitio al código de F3 a F6. Lo que cuenta para ti es que abra en ≤ 3 s en Windows: en Chromium tarda 0,3 s, y en tu PC se mide en la Sesión 1 (F2.5). Redacción limitada a Windows y Android tras AR-03.</t>
         </is>
       </c>
       <c r="P11" s="6" t="n"/>
-      <c r="Q11" s="5" t="inlineStr"/>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -2835,12 +2839,12 @@
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14 y #15</t>
+          <t>F1.1 #14 y #15 · V-05: escucha del cliente en su iPhone (0.2.0, 19/10)</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
@@ -2850,7 +2854,7 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>Reproductor propio con las grabaciones de samples/ desde la 0.2.0. Desde la 0.2.2 la guitarra clásica tiene también la grabación de La♯5: en afinación estándar ninguna nota se transporta más de 6 semitonos, y el traste 24 suena menos artificial. La acústica no tiene grabaciones por encima del Re5 y llega a 14. La 0.1.3 corrigió el registro agudo de nylon, que sonaba medio tono alto.</t>
+          <t>Reproductor propio con las grabaciones de samples/ desde la 0.2.0. Desde la 0.2.2 la guitarra clásica tiene también la grabación de La♯5: en afinación estándar ninguna nota se transporta más de 6 semitonos, y el traste 24 suena menos artificial. La acústica no tiene grabaciones por encima del Re5 y llega a 14: limitación conocida, pendiente de que la aceptes. Escuchada por ti en el iPhone con la 0.2.0 el 19/10 (V-05). La 0.1.3 corrigió el registro agudo de nylon, que sonaba medio tono alto.</t>
         </is>
       </c>
       <c r="P32" s="6" t="n"/>
@@ -3320,11 +3324,15 @@
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>Opción A, decidida el 14/10. Hecho: licencias verificadas y los 16 archivos en samples/, con CREDITOS.md (F2.1); desde la 0.2.0 la app los usa y no descarga nada de otros servidores (F2.2). Desde la 0.2.1 van también dentro del archivo autónomo (F2.3). Falta confirmar que todos los sonidos del pack de nylon comparten la licencia comprobada en uno de ellos: estaba previsto antes de F2.3 y pasa a ser condición antes de publicar (F7).</t>
+          <t>Opción A, decidida el 14/10. Hecho: licencias verificadas y los 16 archivos en samples/, con CREDITOS.md (F2.1); desde la 0.2.0 la app los usa y no descarga nada de otros servidores (F2.2). Desde la 0.2.1 van también dentro del archivo autónomo (F2.3). Falta confirmar que todos los sonidos del pack de nylon comparten la licencia comprobada en uno de ellos. El repositorio y la web de pruebas ya son públicos, así que se hace lo antes posible y como tarde al cerrar F3 (AR-03); si algún sonido no fuera CC BY, se sustituye su grabación.</t>
         </is>
       </c>
       <c r="P38" s="6" t="n"/>
-      <c r="Q38" s="5" t="inlineStr"/>
+      <c r="Q38" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="120" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -3403,11 +3411,7 @@
         </is>
       </c>
       <c r="P39" s="6" t="n"/>
-      <c r="Q39" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q39" s="5" t="inlineStr"/>
     </row>
     <row r="40" ht="78" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
@@ -7611,7 +7615,7 @@
       <c r="P93" s="6" t="n"/>
       <c r="Q93" s="5" t="inlineStr"/>
     </row>
-    <row r="94" ht="120" customHeight="1">
+    <row r="94" ht="78" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
         <is>
           <t>X-01</t>
@@ -7654,27 +7658,27 @@
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>GitHub muestra la última versión y la etiqueta de cierre de fase.</t>
+          <t>GitHub muestra la última versión en main, entrada por pull request aprobado, y la etiqueta de cierre de fase.</t>
         </is>
       </c>
       <c r="J94" s="5" t="inlineStr">
         <is>
-          <t>Cumple parcialmente</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
-          <t>0.0.1</t>
+          <t>0.1.4</t>
         </is>
       </c>
       <c r="L94" s="5" t="inlineStr">
         <is>
-          <t>Rama local auto/F1-iteracion-0, sin subir</t>
+          <t>PR #1 a #5 fusionados · etiqueta v0.1.5</t>
         </is>
       </c>
       <c r="M94" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N94" s="5" t="inlineStr">
@@ -7684,11 +7688,15 @@
       </c>
       <c r="O94" s="5" t="inlineStr">
         <is>
-          <t>El repositorio existe con la versión 0.0.1. Reorganizado en local el 14/10 (rama auto/F1-iteracion-0): docs/, tests/, samples/, CLAUDE.md y la app 0.1.3. Falta subirlo, para lo que hay que vincular GitHub a Claude o abrir la conversación desde el ordenador. Parada antes de F2.2 (CP-1): no se construye F2 sobre trabajo sin copia.</t>
+          <t>Desde el 15/10 todo el proyecto está en pdigue/guitarra; cada versión entra por pull request aprobado (del #1 al #5) y F1 se cerró con la etiqueta v0.1.5. El repositorio es público.</t>
         </is>
       </c>
       <c r="P94" s="6" t="n"/>
-      <c r="Q94" s="5" t="inlineStr"/>
+      <c r="Q94" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="120" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
@@ -8577,7 +8585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8617,7 +8625,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -8627,24 +8635,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -8654,24 +8662,24 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -8681,51 +8689,51 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -8735,7 +8743,7 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
@@ -8745,32 +8753,59 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F3.1: registrar las decisiones del 20/10 y la licencia de nylon en tres sonidos (G-03, S-01, S-07)
Requisitos v1.9, matriz 1.7 y roadmap 3.7. Service Worker en F6.2; agudo
de la acústica aceptado como limitación conocida.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.6. Base: requisitos.md v1.8 · app 0.2.3 · roadmap 3.6 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.7. Base: requisitos.md v1.9 · app 0.2.3 · roadmap 3.7 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.8</t>
+          <t>Cambio en v1.9</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       <c r="P6" s="6" t="n"/>
       <c r="Q6" s="5" t="inlineStr"/>
     </row>
-    <row r="7" ht="78" customHeight="1">
+    <row r="7" ht="108" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>G-03</t>
@@ -899,11 +899,15 @@
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>Service Worker. Depende de S-07. Se valida en dos pasos: en localhost en F6.2 y desde la web publicada en F7.2 (CP-1). En modo archivo (G-07) la autonomía se consigue de otra forma: el audio va dentro del archivo.</t>
+          <t>Service Worker en F6.2, decidido el 20/10: en la Sesión 1 el iPhone no prueba la app sin conexión. Depende de S-07. Se valida en dos pasos: en localhost en F6.2 y desde la web publicada en F7.2 (CP-1). En modo archivo (G-07) la autonomía se consigue de otra forma: el audio va dentro del archivo.</t>
         </is>
       </c>
       <c r="P7" s="6" t="n"/>
-      <c r="Q7" s="5" t="inlineStr"/>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -1219,11 +1223,7 @@
         </is>
       </c>
       <c r="P11" s="6" t="n"/>
-      <c r="Q11" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -2854,7 +2854,7 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>Reproductor propio con las grabaciones de samples/ desde la 0.2.0. Desde la 0.2.2 la guitarra clásica tiene también la grabación de La♯5: en afinación estándar ninguna nota se transporta más de 6 semitonos, y el traste 24 suena menos artificial. La acústica no tiene grabaciones por encima del Re5 y llega a 14: limitación conocida, pendiente de que la aceptes. Escuchada por ti en el iPhone con la 0.2.0 el 19/10 (V-05). La 0.1.3 corrigió el registro agudo de nylon, que sonaba medio tono alto.</t>
+          <t>Reproductor propio con las grabaciones de samples/ desde la 0.2.0. Desde la 0.2.2 la guitarra clásica tiene también la grabación de La♯5: en afinación estándar ninguna nota se transporta más de 6 semitonos, y el traste 24 suena menos artificial. La acústica no tiene grabaciones por encima del Re5 y llega a 14: limitación conocida, aceptada por ti el 20/10; se comprueba de oído en la Sesión 1 (trastes 15 a 24 de la 1ª cuerda). Escuchada por ti en el iPhone con la 0.2.0 el 19/10 (V-05). La 0.1.3 corrigió el registro agudo de nylon, que sonaba medio tono alto.</t>
         </is>
       </c>
       <c r="P32" s="6" t="n"/>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>CREDITOS.md y samples/ (F2.1) · Banco (node --test): ninguna dirección externa (0.2.0)</t>
+          <t>CREDITOS.md y samples/ (F2.1) · Banco (node --test): ninguna dirección externa (0.2.0) · licencia de nylon comprobada en 3 sonidos del pack (20/10)</t>
         </is>
       </c>
       <c r="M38" s="5" t="inlineStr">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>Opción A, decidida el 14/10. Hecho: licencias verificadas y los 16 archivos en samples/, con CREDITOS.md (F2.1); desde la 0.2.0 la app los usa y no descarga nada de otros servidores (F2.2). Desde la 0.2.1 van también dentro del archivo autónomo (F2.3). Falta confirmar que todos los sonidos del pack de nylon comparten la licencia comprobada en uno de ellos. El repositorio y la web de pruebas ya son públicos, así que se hace lo antes posible y como tarde al cerrar F3 (AR-03); si algún sonido no fuera CC BY, se sustituye su grabación.</t>
+          <t>Opción A, decidida el 14/10. Hecho: licencias verificadas y los 16 archivos en samples/, con CREDITOS.md (F2.1); desde la 0.2.0 la app los usa y no descarga nada de otros servidores (F2.2). Desde la 0.2.1 van también dentro del archivo autónomo (F2.3). El 20/10 se comprobaron tres sonidos del pack de nylon, de cuerdas distintas (183078, 183083 y 183089): los tres «Attribution 4.0». Falta confirmar el pack entero, que solo se ve en la búsqueda de Freesound, cerrada a los agentes: lo miras tú en un minuto. El repositorio y la web de pruebas ya son públicos, así que se hace lo antes posible y como tarde al cerrar F3 (AR-03); si algún sonido no fuera CC BY, se sustituye su grabación.</t>
         </is>
       </c>
       <c r="P38" s="6" t="n"/>
@@ -7692,11 +7692,7 @@
         </is>
       </c>
       <c r="P94" s="6" t="n"/>
-      <c r="Q94" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q94" s="5" t="inlineStr"/>
     </row>
     <row r="95" ht="120" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
@@ -8585,7 +8581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8625,17 +8621,17 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
@@ -8645,14 +8641,14 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -8662,24 +8658,24 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -8689,24 +8685,24 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -8716,51 +8712,51 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -8770,7 +8766,7 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
@@ -8780,32 +8776,59 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F3.1: cerrar la licencia del pack de nylon, 161 sonidos CC BY (S-07)
Requisitos v1.10 (S-07 implementado y validado), matriz 1.8 y roadmap 3.8.
Comprobación hecha por el cliente en la búsqueda de Freesound, con dos
filtros de control a 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.7. Base: requisitos.md v1.9 · app 0.2.3 · roadmap 3.7 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.8. Base: requisitos.md v1.10 · app 0.2.3 · roadmap 3.8 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.9</t>
+          <t>Cambio en v1.10</t>
         </is>
       </c>
     </row>
@@ -903,11 +903,7 @@
         </is>
       </c>
       <c r="P7" s="6" t="n"/>
-      <c r="Q7" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -2858,11 +2854,7 @@
         </is>
       </c>
       <c r="P32" s="6" t="n"/>
-      <c r="Q32" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q32" s="5" t="inlineStr"/>
     </row>
     <row r="33" ht="63" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -3299,22 +3291,22 @@
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>Cumple parcialmente</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>CREDITOS.md y samples/ (F2.1) · Banco (node --test): ninguna dirección externa (0.2.0) · licencia de nylon comprobada en 3 sonidos del pack (20/10)</t>
+          <t>CREDITOS.md y samples/ (F2.1) · Banco (node --test): ninguna dirección externa (0.2.0) · licencia de los 161 sonidos del pack de nylon: CC BY, con filtros de control a 0 (20/10)</t>
         </is>
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>Verificado parcialmente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N38" s="5" t="inlineStr">
@@ -3324,7 +3316,7 @@
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>Opción A, decidida el 14/10. Hecho: licencias verificadas y los 16 archivos en samples/, con CREDITOS.md (F2.1); desde la 0.2.0 la app los usa y no descarga nada de otros servidores (F2.2). Desde la 0.2.1 van también dentro del archivo autónomo (F2.3). El 20/10 se comprobaron tres sonidos del pack de nylon, de cuerdas distintas (183078, 183083 y 183089): los tres «Attribution 4.0». Falta confirmar el pack entero, que solo se ve en la búsqueda de Freesound, cerrada a los agentes: lo miras tú en un minuto. El repositorio y la web de pruebas ya son públicos, así que se hace lo antes posible y como tarde al cerrar F3 (AR-03); si algún sonido no fuera CC BY, se sustituye su grabación.</t>
+          <t>Opción A, decidida el 14/10. Hecho: licencias verificadas y los 16 archivos en samples/, con CREDITOS.md (F2.1); desde la 0.2.0 la app los usa y no descarga nada de otros servidores (F2.2). Desde la 0.2.1 van también dentro del archivo autónomo (F2.3). El 20/10 se completó la licencia del pack de nylon: en la búsqueda de Freesound, el pack tiene 161 sonidos y el filtro de licencia «Attribution» (CC BY) devuelve los 161; dos filtros de control («Attribution 4.0» y «Creative Commons 0») devuelven 0, lo que prueba que el filtro se aplica. Tres sonidos revisados uno a uno (183078, 183083 y 183089) son «Attribution 4.0». La búsqueda la hiciste tú en tu iPhone, porque está cerrada a los agentes. Validado por inspección: ninguna petición de audio sale del dominio propio (banco) y CREDITOS.md documenta origen y licencia de los 17 archivos.</t>
         </is>
       </c>
       <c r="P38" s="6" t="n"/>
@@ -8581,7 +8573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8621,7 +8613,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -8631,7 +8623,7 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
@@ -8641,24 +8633,24 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
@@ -8668,14 +8660,14 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -8685,24 +8677,24 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -8712,24 +8704,24 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -8739,51 +8731,51 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -8793,7 +8785,7 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
@@ -8803,32 +8795,59 @@
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F3.1: aprobar la interfaz, interfaz.md v1.0 (C-06, C-07, V-01, V-04, G-05)
Requisitos v1.11 (C-07 nuevo; C-06 validado; criterios de V-01, V-04 y
G-05; notas de C-01 a C-04), matriz 1.9 y roadmap 3.9.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control de cambios" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz'!$A$4:$Q$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz'!$A$4:$Q$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q96"/>
+  <dimension ref="A1:Q97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.8. Base: requisitos.md v1.10 · app 0.2.3 · roadmap 3.8 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.9. Base: requisitos.md v1.11 · app 0.2.3 · roadmap 3.9 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.10</t>
+          <t>Cambio en v1.11</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       <c r="P8" s="6" t="n"/>
       <c r="Q8" s="5" t="inlineStr"/>
     </row>
-    <row r="9" ht="93" customHeight="1">
+    <row r="9" ht="120" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>G-05</t>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Desarrollo · v1.1</t>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Todo control es alcanzable con teclado y muestra el foco; contrastes ≥ 4,5:1 medidos; el movimiento se reduce con prefers-reduced-motion.</t>
+          <t>Todo control es alcanzable con teclado y muestra el foco; contrastes ≥ 4,5:1 medidos; el movimiento se reduce con prefers-reduced-motion; en pantallas táctiles, todo control y toda casilla del mástil mide al menos 40 × 40 px.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -1057,11 +1057,15 @@
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>Hecho: foco visible, movimiento reducido, interruptores con role="switch" (0.1.1), aria-pressed en los selectores y aviso del reto para lectores de pantalla (0.1.2). Falta: recorrer el mástil con teclado y auditar el contraste.</t>
+          <t>Hecho: foco visible, movimiento reducido, interruptores con role="switch" (0.1.1), aria-pressed en los selectores y aviso del reto para lectores de pantalla (0.1.2). Falta: recorrer el mástil con teclado y auditar el contraste. Añadido al criterio el 20/10 (interfaz.md v1.0, aprobada el 20/10): en pantallas táctiles, todo control y toda casilla del mástil mide al menos 40 × 40 px.</t>
         </is>
       </c>
       <c r="P9" s="6" t="n"/>
-      <c r="Q9" s="5" t="inlineStr"/>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="78" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -3320,11 +3324,7 @@
         </is>
       </c>
       <c r="P38" s="6" t="n"/>
-      <c r="Q38" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q38" s="5" t="inlineStr"/>
     </row>
     <row r="39" ht="120" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -6438,7 +6438,7 @@
       <c r="P78" s="6" t="n"/>
       <c r="Q78" s="5" t="inlineStr"/>
     </row>
-    <row r="79" ht="63" customHeight="1">
+    <row r="79" ht="120" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
           <t>V-01</t>
@@ -6461,7 +6461,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
@@ -6481,7 +6481,7 @@
       </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>En un móvil apaisado cada cuerda mide al menos 40 px, y en vertical aparece el aviso para girar.</t>
+          <t>En horizontal, con un alto útil de 268 px o más, cada cuerda mide al menos 40 px (iPhone en Safari e instalada; simulador de Android). En vertical, en pantallas táctiles de menos de 600 px y en Libre, Adivinar y Escalas, aparece el aviso para girar; nunca en el Afinador; cerrado, no vuelve y «Restablecer» lo recupera.</t>
         </is>
       </c>
       <c r="J79" s="5" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="L79" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>interfaz.md §7: bocetos medidos (52 px en el iPhone, 42 px en Android)</t>
         </is>
       </c>
       <c r="M79" s="5" t="inlineStr">
@@ -6511,11 +6511,15 @@
       </c>
       <c r="O79" s="5" t="inlineStr">
         <is>
-          <t>El bloqueo de orientación tiene mal soporte en iOS. Menos trastes visibles en vertical es la solución adoptada. Falta el aviso y un diseño apaisado que dé altura a las cuerdas.</t>
+          <t>Criterio concreto el 20/10 (interfaz.md v1.0, aprobada el 20/10): el aviso sale solo en pantallas táctiles (pointer: coarse) en vertical de menos de 600 px de ancho, en Libre, Adivinar y Escalas, y nunca en el Afinador; si lo cierras, no vuelve (se guarda con los ajustes) y «Restablecer» lo recupera. En horizontal, raíl, mástil a todo el alto y panel: los bocetos dan 52 px por cuerda en el iPhone y 42 en un Android de 280 px de alto; los 40 px se exigen con un alto útil de 268 px o más. El bloqueo de orientación tiene mal soporte en iOS, así que no se fuerza.</t>
         </is>
       </c>
       <c r="P79" s="6" t="n"/>
-      <c r="Q79" s="5" t="inlineStr"/>
+      <c r="Q79" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="33" customHeight="1">
       <c r="A80" s="4" t="inlineStr">
@@ -6671,7 +6675,7 @@
       <c r="P81" s="6" t="n"/>
       <c r="Q81" s="5" t="inlineStr"/>
     </row>
-    <row r="82" ht="63" customHeight="1">
+    <row r="82" ht="120" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
         <is>
           <t>V-04</t>
@@ -6694,17 +6698,17 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 · F3</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>F1.1</t>
+          <t>F1.1 · F3.2</t>
         </is>
       </c>
       <c r="H82" s="5" t="inlineStr">
@@ -6714,12 +6718,12 @@
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>El zoom cambia los trastes visibles entre 3 y el máximo que cabe, y la etiqueta dice la cifra real.</t>
+          <t>El zoom cambia los trastes visibles entre 3 y el máximo que cabe, y la etiqueta dice la cifra real. Con pointer: coarse, un traste mide al menos 40 px y el zoom guardado se ajusta a ese límite.</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
-          <t>Cumple</t>
+          <t>Cumple parcialmente</t>
         </is>
       </c>
       <c r="K82" s="5" t="inlineStr">
@@ -6734,7 +6738,7 @@
       </c>
       <c r="M82" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N82" s="5" t="inlineStr">
@@ -6744,11 +6748,15 @@
       </c>
       <c r="O82" s="5" t="inlineStr">
         <is>
-          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando.</t>
+          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Añadido el 20/10 (interfaz.md v1.0, aprobada el 20/10): con pointer: coarse, un traste mide al menos 40 px y el zoom guardado se ajusta a ese límite; en el iPhone en vertical quedan como mucho 8 trastes a la vista. Se hace en F3.2.</t>
         </is>
       </c>
       <c r="P82" s="6" t="n"/>
-      <c r="Q82" s="5" t="inlineStr"/>
+      <c r="Q82" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="33" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
@@ -7133,7 +7141,7 @@
       <c r="P87" s="6" t="n"/>
       <c r="Q87" s="5" t="inlineStr"/>
     </row>
-    <row r="88" ht="33" customHeight="1">
+    <row r="88" ht="48" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
         <is>
           <t>C-01</t>
@@ -7206,13 +7214,17 @@
       </c>
       <c r="O88" s="5" t="inlineStr">
         <is>
-          <t>Panel deslizante desde la cabecera.</t>
+          <t>Hoja que sube desde abajo en vertical; panel lateral en horizontal y en pantallas amplias (interfaz.md v1.0, aprobada el 20/10).</t>
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
-      <c r="Q88" s="5" t="inlineStr"/>
-    </row>
-    <row r="89" ht="63" customHeight="1">
+      <c r="Q88" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="78" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
         <is>
           <t>C-02</t>
@@ -7285,13 +7297,17 @@
       </c>
       <c r="O89" s="5" t="inlineStr">
         <is>
-          <t>Ampliado en 0.1.2 con la numeración en tres modos y la versión (G-10).</t>
+          <t>Ampliado en 0.1.2 con la numeración en tres modos y la versión (G-10). En F6.4 se añade el grupo «Acerca de», con los créditos (G-06) y la privacidad (G-11) (interfaz.md v1.0, aprobada el 20/10).</t>
         </is>
       </c>
       <c r="P89" s="6" t="n"/>
-      <c r="Q89" s="5" t="inlineStr"/>
-    </row>
-    <row r="90" ht="33" customHeight="1">
+      <c r="Q89" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="78" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
         <is>
           <t>C-03</t>
@@ -7364,13 +7380,17 @@
       </c>
       <c r="O90" s="5" t="inlineStr">
         <is>
-          <t>Nomenclatura, pentagrama y las dos pistas del juego.</t>
+          <t>Nomenclatura y pentagrama en chips bajo la cabecera, o en el panel en horizontal; las dos pistas del juego, en la tarjeta del reto desde F3.2 (interfaz.md v1.0, aprobada el 20/10).</t>
         </is>
       </c>
       <c r="P90" s="6" t="n"/>
-      <c r="Q90" s="5" t="inlineStr"/>
-    </row>
-    <row r="91" ht="33" customHeight="1">
+      <c r="Q90" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="63" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
         <is>
           <t>C-04</t>
@@ -7393,7 +7413,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
@@ -7413,7 +7433,7 @@
       </c>
       <c r="I91" s="5" t="inlineStr">
         <is>
-          <t>La barra inferior lleva a cada área con un toque.</t>
+          <t>La navegación (barra inferior, raíl o pestañas en la cabecera, según la disposición) lleva a cada área con un toque.</t>
         </is>
       </c>
       <c r="J91" s="5" t="inlineStr">
@@ -7443,11 +7463,15 @@
       </c>
       <c r="O91" s="5" t="inlineStr">
         <is>
-          <t>Barra inferior con cuatro destinos.</t>
+          <t>Barra inferior con cuatro destinos en vertical, raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (interfaz.md v1.0, aprobada el 20/10).</t>
         </is>
       </c>
       <c r="P91" s="6" t="n"/>
-      <c r="Q91" s="5" t="inlineStr"/>
+      <c r="Q91" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="33" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
@@ -7528,7 +7552,7 @@
       <c r="P92" s="6" t="n"/>
       <c r="Q92" s="5" t="inlineStr"/>
     </row>
-    <row r="93" ht="48" customHeight="1">
+    <row r="93" ht="93" customHeight="1">
       <c r="A93" s="4" t="inlineStr">
         <is>
           <t>C-06</t>
@@ -7576,22 +7600,22 @@
       </c>
       <c r="J93" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K93" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="L93" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>interfaz.md v1.0 · AR-04 · aprobación del cliente el 20/10</t>
         </is>
       </c>
       <c r="M93" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N93" s="5" t="inlineStr">
@@ -7601,174 +7625,182 @@
       </c>
       <c r="O93" s="5" t="inlineStr">
         <is>
-          <t>Bloqueante de F3.2 y de toda F5. Requiere sesión dedicada.</t>
+          <t>docs/interfaz.md v1.0, aprobada por ti el 20/10 tras la auditoría AR-04 (10 hallazgos resueltos). Bocetos al tamaño real de cada pantalla en docs/interfaz/, comprobados por herramientas/capturar-wireframes.js. Los cambios posteriores suben su versión.</t>
         </is>
       </c>
       <c r="P93" s="6" t="n"/>
-      <c r="Q93" s="5" t="inlineStr"/>
+      <c r="Q93" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="78" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
         <is>
+          <t>C-07</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Configuración y navegación</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Botón «atrás» del sistema: mientras haya un paso anterior en la sesión, el botón o gesto «atrás» cierra Ajustes o vuelve al área anterior; desde la primera área actúa el sistema. Al abrir la app se entra en Libre.</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>F3.2</t>
+        </is>
+      </c>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>Con un paso anterior en la sesión, «atrás» cierra Ajustes o vuelve al área anterior; desde la primera área actúa el sistema; al abrir o recargar se entra en Libre. Prueba manual en Windows y en el simulador de Android de Chrome.</t>
+        </is>
+      </c>
+      <c r="J94" s="5" t="inlineStr">
+        <is>
+          <t>No cumple</t>
+        </is>
+      </c>
+      <c r="K94" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L94" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M94" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="N94" s="5" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="O94" s="5" t="inlineStr">
+        <is>
+          <t>Aprobado el 20/10 con interfaz.md v1.0. Usa el historial del navegador (history), estándar en todos los sistemas. En el iPhone instalado no hay botón atrás.</t>
+        </is>
+      </c>
+      <c r="P94" s="6" t="n"/>
+      <c r="Q94" s="5" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="78" customHeight="1">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
           <t>X-01</t>
         </is>
       </c>
-      <c r="B94" s="5" t="inlineStr">
+      <c r="B95" s="5" t="inlineStr">
         <is>
           <t>Respaldo y publicación</t>
         </is>
       </c>
-      <c r="C94" s="5" t="inlineStr">
+      <c r="C95" s="5" t="inlineStr">
         <is>
           <t>El código y la documentación están respaldados en el repositorio remoto (GitHub). Respaldar no es publicar.</t>
         </is>
       </c>
-      <c r="D94" s="5" t="inlineStr">
+      <c r="D95" s="5" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="E94" s="5" t="inlineStr">
+      <c r="E95" s="5" t="inlineStr">
         <is>
           <t>Desarrollo · v1.1</t>
         </is>
       </c>
-      <c r="F94" s="5" t="inlineStr">
+      <c r="F95" s="5" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="G94" s="5" t="inlineStr">
+      <c r="G95" s="5" t="inlineStr">
         <is>
           <t>F1.2 · F1.4</t>
         </is>
       </c>
-      <c r="H94" s="5" t="inlineStr">
+      <c r="H95" s="5" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="I94" s="5" t="inlineStr">
+      <c r="I95" s="5" t="inlineStr">
         <is>
           <t>GitHub muestra la última versión en main, entrada por pull request aprobado, y la etiqueta de cierre de fase.</t>
         </is>
       </c>
-      <c r="J94" s="5" t="inlineStr">
+      <c r="J95" s="5" t="inlineStr">
         <is>
           <t>Cumple</t>
         </is>
       </c>
-      <c r="K94" s="5" t="inlineStr">
+      <c r="K95" s="5" t="inlineStr">
         <is>
           <t>0.1.4</t>
         </is>
       </c>
-      <c r="L94" s="5" t="inlineStr">
+      <c r="L95" s="5" t="inlineStr">
         <is>
           <t>PR #1 a #5 fusionados · etiqueta v0.1.5</t>
         </is>
       </c>
-      <c r="M94" s="5" t="inlineStr">
+      <c r="M95" s="5" t="inlineStr">
         <is>
           <t>Verificado parcialmente</t>
         </is>
       </c>
-      <c r="N94" s="5" t="inlineStr">
+      <c r="N95" s="5" t="inlineStr">
         <is>
           <t>Auditor de requisitos</t>
         </is>
       </c>
-      <c r="O94" s="5" t="inlineStr">
+      <c r="O95" s="5" t="inlineStr">
         <is>
           <t>Desde el 15/10 todo el proyecto está en pdigue/guitarra; cada versión entra por pull request aprobado (del #1 al #5) y F1 se cerró con la etiqueta v0.1.5. El repositorio es público.</t>
-        </is>
-      </c>
-      <c r="P94" s="6" t="n"/>
-      <c r="Q94" s="5" t="inlineStr"/>
-    </row>
-    <row r="95" ht="120" customHeight="1">
-      <c r="A95" s="4" t="inlineStr">
-        <is>
-          <t>X-02</t>
-        </is>
-      </c>
-      <c r="B95" s="5" t="inlineStr">
-        <is>
-          <t>Respaldo y publicación</t>
-        </is>
-      </c>
-      <c r="C95" s="5" t="inlineStr">
-        <is>
-          <t>La app está publicada en una URL pública (GitHub Pages).</t>
-        </is>
-      </c>
-      <c r="D95" s="5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="E95" s="5" t="inlineStr">
-        <is>
-          <t>Desarrollo · v1.1</t>
-        </is>
-      </c>
-      <c r="F95" s="5" t="inlineStr">
-        <is>
-          <t>F7</t>
-        </is>
-      </c>
-      <c r="G95" s="5" t="inlineStr">
-        <is>
-          <t>F7.1</t>
-        </is>
-      </c>
-      <c r="H95" s="5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="I95" s="5" t="inlineStr">
-        <is>
-          <t>La URL pública carga la app desde un dispositivo ajeno al proyecto.</t>
-        </is>
-      </c>
-      <c r="J95" s="5" t="inlineStr">
-        <is>
-          <t>No cumple</t>
-        </is>
-      </c>
-      <c r="K95" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L95" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M95" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="N95" s="5" t="inlineStr">
-        <is>
-          <t>Cliente</t>
-        </is>
-      </c>
-      <c r="O95" s="5" t="inlineStr">
-        <is>
-          <t>Antes en V1; pasa a la última fase por decisión del 15/09: desarrollo local de principio a fin. Despliegue de pruebas (decisión del 15/10): antes de la Sesión 1 se publica una versión de pruebas en GitHub Pages, sin anunciar, para probar en el iPhone con https la instalación, el modo sin conexión y el micrófono. X-02 sigue siendo la publicación oficial.</t>
         </is>
       </c>
       <c r="P95" s="6" t="n"/>
       <c r="Q95" s="5" t="inlineStr"/>
     </row>
-    <row r="96" ht="33" customHeight="1">
+    <row r="96" ht="120" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>X-03</t>
+          <t>X-02</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
@@ -7778,7 +7810,7 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>La app está verificada en móviles reales, instalada como icono desde la web publicada.</t>
+          <t>La app está publicada en una URL pública (GitHub Pages).</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
@@ -7798,7 +7830,7 @@
       </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
-          <t>F7.2</t>
+          <t>F7.1</t>
         </is>
       </c>
       <c r="H96" s="5" t="inlineStr">
@@ -7808,7 +7840,7 @@
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>La app instalada desde la web funciona en un Android, un iPhone y un Windows reales.</t>
+          <t>La URL pública carga la app desde un dispositivo ajeno al proyecto.</t>
         </is>
       </c>
       <c r="J96" s="5" t="inlineStr">
@@ -7838,15 +7870,94 @@
       </c>
       <c r="O96" s="5" t="inlineStr">
         <is>
-          <t>Cierra G-04 y PL-01 a PL-03 en su modo web.</t>
+          <t>Antes en V1; pasa a la última fase por decisión del 15/09: desarrollo local de principio a fin. Despliegue de pruebas (decisión del 15/10): antes de la Sesión 1 se publica una versión de pruebas en GitHub Pages, sin anunciar, para probar en el iPhone con https la instalación, el modo sin conexión y el micrófono. X-02 sigue siendo la publicación oficial.</t>
         </is>
       </c>
       <c r="P96" s="6" t="n"/>
       <c r="Q96" s="5" t="inlineStr"/>
     </row>
+    <row r="97" ht="33" customHeight="1">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>X-03</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Respaldo y publicación</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>La app está verificada en móviles reales, instalada como icono desde la web publicada.</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>Desarrollo · v1.1</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>F7.2</t>
+        </is>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>La app instalada desde la web funciona en un Android, un iPhone y un Windows reales.</t>
+        </is>
+      </c>
+      <c r="J97" s="5" t="inlineStr">
+        <is>
+          <t>No cumple</t>
+        </is>
+      </c>
+      <c r="K97" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L97" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M97" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="N97" s="5" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="O97" s="5" t="inlineStr">
+        <is>
+          <t>Cierra G-04 y PL-01 a PL-03 en su modo web.</t>
+        </is>
+      </c>
+      <c r="P97" s="6" t="n"/>
+      <c r="Q97" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q96"/>
-  <conditionalFormatting sqref="J5:J96">
+  <autoFilter ref="A4:Q97"/>
+  <conditionalFormatting sqref="J5:J97">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>J5="Cumple"</formula>
     </cfRule>
@@ -7863,7 +7974,7 @@
       <formula>J5="No aplica"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M96">
+  <conditionalFormatting sqref="M5:M97">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>M5="Cumple"</formula>
     </cfRule>
@@ -7881,13 +7992,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="J5:J96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
+    <dataValidation sqref="J5:J97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
       <formula1>"Cumple,Cumple parcialmente,No cumple,No aplica"</formula1>
     </dataValidation>
-    <dataValidation sqref="M5:M96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
+    <dataValidation sqref="M5:M97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
       <formula1>"Verificado,Verificado parcialmente,Pendiente,No aplica"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
+    <dataValidation sqref="H5:H97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
       <formula1>"I,A,D,T,I+T,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7983,23 +8094,23 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$96,"*F1*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$97,"*F1*")</f>
         <v/>
       </c>
       <c r="C5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F1*",Matriz!$J$5:$J$96,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F1*",Matriz!$J$5:$J$97,"Cumple")</f>
         <v/>
       </c>
       <c r="D5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F1*",Matriz!$J$5:$J$96,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F1*",Matriz!$J$5:$J$97,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F1*",Matriz!$J$5:$J$96,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F1*",Matriz!$J$5:$J$97,"No cumple")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F1*",Matriz!$J$5:$J$96,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F1*",Matriz!$J$5:$J$97,"No aplica")</f>
         <v/>
       </c>
       <c r="G5" s="8">
@@ -8007,11 +8118,11 @@
         <v/>
       </c>
       <c r="H5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F1*",Matriz!$M$5:$M$96,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F1*",Matriz!$M$5:$M$97,"Verificado")</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F1*",Matriz!$M$5:$M$96,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F1*",Matriz!$M$5:$M$97,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -8022,23 +8133,23 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$96,"*F2*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$97,"*F2*")</f>
         <v/>
       </c>
       <c r="C6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F2*",Matriz!$J$5:$J$96,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F2*",Matriz!$J$5:$J$97,"Cumple")</f>
         <v/>
       </c>
       <c r="D6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F2*",Matriz!$J$5:$J$96,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F2*",Matriz!$J$5:$J$97,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F2*",Matriz!$J$5:$J$96,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F2*",Matriz!$J$5:$J$97,"No cumple")</f>
         <v/>
       </c>
       <c r="F6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F2*",Matriz!$J$5:$J$96,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F2*",Matriz!$J$5:$J$97,"No aplica")</f>
         <v/>
       </c>
       <c r="G6" s="8">
@@ -8046,11 +8157,11 @@
         <v/>
       </c>
       <c r="H6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F2*",Matriz!$M$5:$M$96,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F2*",Matriz!$M$5:$M$97,"Verificado")</f>
         <v/>
       </c>
       <c r="I6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F2*",Matriz!$M$5:$M$96,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F2*",Matriz!$M$5:$M$97,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -8061,23 +8172,23 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$96,"*F3*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$97,"*F3*")</f>
         <v/>
       </c>
       <c r="C7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F3*",Matriz!$J$5:$J$96,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F3*",Matriz!$J$5:$J$97,"Cumple")</f>
         <v/>
       </c>
       <c r="D7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F3*",Matriz!$J$5:$J$96,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F3*",Matriz!$J$5:$J$97,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F3*",Matriz!$J$5:$J$96,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F3*",Matriz!$J$5:$J$97,"No cumple")</f>
         <v/>
       </c>
       <c r="F7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F3*",Matriz!$J$5:$J$96,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F3*",Matriz!$J$5:$J$97,"No aplica")</f>
         <v/>
       </c>
       <c r="G7" s="8">
@@ -8085,11 +8196,11 @@
         <v/>
       </c>
       <c r="H7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F3*",Matriz!$M$5:$M$96,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F3*",Matriz!$M$5:$M$97,"Verificado")</f>
         <v/>
       </c>
       <c r="I7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F3*",Matriz!$M$5:$M$96,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F3*",Matriz!$M$5:$M$97,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -8100,23 +8211,23 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$96,"*F4*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$97,"*F4*")</f>
         <v/>
       </c>
       <c r="C8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F4*",Matriz!$J$5:$J$96,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F4*",Matriz!$J$5:$J$97,"Cumple")</f>
         <v/>
       </c>
       <c r="D8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F4*",Matriz!$J$5:$J$96,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F4*",Matriz!$J$5:$J$97,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F4*",Matriz!$J$5:$J$96,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F4*",Matriz!$J$5:$J$97,"No cumple")</f>
         <v/>
       </c>
       <c r="F8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F4*",Matriz!$J$5:$J$96,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F4*",Matriz!$J$5:$J$97,"No aplica")</f>
         <v/>
       </c>
       <c r="G8" s="8">
@@ -8124,11 +8235,11 @@
         <v/>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F4*",Matriz!$M$5:$M$96,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F4*",Matriz!$M$5:$M$97,"Verificado")</f>
         <v/>
       </c>
       <c r="I8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F4*",Matriz!$M$5:$M$96,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F4*",Matriz!$M$5:$M$97,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -8139,23 +8250,23 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$96,"*F5*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$97,"*F5*")</f>
         <v/>
       </c>
       <c r="C9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F5*",Matriz!$J$5:$J$96,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F5*",Matriz!$J$5:$J$97,"Cumple")</f>
         <v/>
       </c>
       <c r="D9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F5*",Matriz!$J$5:$J$96,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F5*",Matriz!$J$5:$J$97,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F5*",Matriz!$J$5:$J$96,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F5*",Matriz!$J$5:$J$97,"No cumple")</f>
         <v/>
       </c>
       <c r="F9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F5*",Matriz!$J$5:$J$96,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F5*",Matriz!$J$5:$J$97,"No aplica")</f>
         <v/>
       </c>
       <c r="G9" s="8">
@@ -8163,11 +8274,11 @@
         <v/>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F5*",Matriz!$M$5:$M$96,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F5*",Matriz!$M$5:$M$97,"Verificado")</f>
         <v/>
       </c>
       <c r="I9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F5*",Matriz!$M$5:$M$96,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F5*",Matriz!$M$5:$M$97,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -8178,23 +8289,23 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$96,"*F6*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$97,"*F6*")</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F6*",Matriz!$J$5:$J$96,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F6*",Matriz!$J$5:$J$97,"Cumple")</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F6*",Matriz!$J$5:$J$96,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F6*",Matriz!$J$5:$J$97,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F6*",Matriz!$J$5:$J$96,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F6*",Matriz!$J$5:$J$97,"No cumple")</f>
         <v/>
       </c>
       <c r="F10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F6*",Matriz!$J$5:$J$96,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F6*",Matriz!$J$5:$J$97,"No aplica")</f>
         <v/>
       </c>
       <c r="G10" s="8">
@@ -8202,11 +8313,11 @@
         <v/>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F6*",Matriz!$M$5:$M$96,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F6*",Matriz!$M$5:$M$97,"Verificado")</f>
         <v/>
       </c>
       <c r="I10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F6*",Matriz!$M$5:$M$96,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F6*",Matriz!$M$5:$M$97,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -8217,23 +8328,23 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$96,"*F7*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$97,"*F7*")</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F7*",Matriz!$J$5:$J$96,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F7*",Matriz!$J$5:$J$97,"Cumple")</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F7*",Matriz!$J$5:$J$96,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F7*",Matriz!$J$5:$J$97,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F7*",Matriz!$J$5:$J$96,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F7*",Matriz!$J$5:$J$97,"No cumple")</f>
         <v/>
       </c>
       <c r="F11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F7*",Matriz!$J$5:$J$96,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F7*",Matriz!$J$5:$J$97,"No aplica")</f>
         <v/>
       </c>
       <c r="G11" s="8">
@@ -8241,11 +8352,11 @@
         <v/>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F7*",Matriz!$M$5:$M$96,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F7*",Matriz!$M$5:$M$97,"Verificado")</f>
         <v/>
       </c>
       <c r="I11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*F7*",Matriz!$M$5:$M$96,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*F7*",Matriz!$M$5:$M$97,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -8256,23 +8367,23 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$96,"*Posterior*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$97,"*Posterior*")</f>
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*Posterior*",Matriz!$J$5:$J$96,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*Posterior*",Matriz!$J$5:$J$97,"Cumple")</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*Posterior*",Matriz!$J$5:$J$96,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*Posterior*",Matriz!$J$5:$J$97,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*Posterior*",Matriz!$J$5:$J$96,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*Posterior*",Matriz!$J$5:$J$97,"No cumple")</f>
         <v/>
       </c>
       <c r="F12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*Posterior*",Matriz!$J$5:$J$96,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*Posterior*",Matriz!$J$5:$J$97,"No aplica")</f>
         <v/>
       </c>
       <c r="G12" s="8">
@@ -8280,11 +8391,11 @@
         <v/>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*Posterior*",Matriz!$M$5:$M$96,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*Posterior*",Matriz!$M$5:$M$97,"Verificado")</f>
         <v/>
       </c>
       <c r="I12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$96,"*Posterior*",Matriz!$M$5:$M$96,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$97,"*Posterior*",Matriz!$M$5:$M$97,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -8295,23 +8406,23 @@
         </is>
       </c>
       <c r="B13" s="9">
-        <f>COUNTA(Matriz!$A$5:$A$96)</f>
+        <f>COUNTA(Matriz!$A$5:$A$97)</f>
         <v/>
       </c>
       <c r="C13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$96,"Cumple")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$97,"Cumple")</f>
         <v/>
       </c>
       <c r="D13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$96,"Cumple parcialmente")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$97,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$96,"No cumple")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$97,"No cumple")</f>
         <v/>
       </c>
       <c r="F13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$96,"No aplica")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$97,"No aplica")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -8319,11 +8430,11 @@
         <v/>
       </c>
       <c r="H13" s="9">
-        <f>COUNTIF(Matriz!$M$5:$M$96,"Verificado")</f>
+        <f>COUNTIF(Matriz!$M$5:$M$97,"Verificado")</f>
         <v/>
       </c>
       <c r="I13" s="9">
-        <f>COUNTIF(Matriz!$M$5:$M$96,"Verificado parcialmente")</f>
+        <f>COUNTIF(Matriz!$M$5:$M$97,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -8341,7 +8452,7 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$96,"I")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$97,"I")</f>
         <v/>
       </c>
     </row>
@@ -8352,7 +8463,7 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$96,"A")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$97,"A")</f>
         <v/>
       </c>
     </row>
@@ -8363,7 +8474,7 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$96,"D")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$97,"D")</f>
         <v/>
       </c>
     </row>
@@ -8374,7 +8485,7 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$96,"T")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$97,"T")</f>
         <v/>
       </c>
     </row>
@@ -8385,7 +8496,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$96,"I+T")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$97,"I+T")</f>
         <v/>
       </c>
     </row>
@@ -8396,7 +8507,7 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$96,"N/A")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$97,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -8573,7 +8684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8613,7 +8724,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -8623,7 +8734,7 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
@@ -8633,14 +8744,14 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -8650,7 +8761,7 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
@@ -8660,24 +8771,24 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
@@ -8687,14 +8798,14 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -8704,24 +8815,24 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -8731,24 +8842,24 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -8758,51 +8869,51 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -8812,7 +8923,7 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
@@ -8822,32 +8933,59 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F3.2: resolver AR-05 y AT-04 y documentar la etapa (V-01, V-04, C-07, G-05, PL-04)
La navegación nunca se sale en pantallas bajas; pentagrama de al menos
60 px; controles de Ajustes a 40 px; Ajustes como diálogo modal; orden
del foco igual al visual; «atrás» sin pasos huérfanos. Requisitos v1.12,
matriz 1.10, roadmap 3.10, interfaz 1.2 y verificación V-06.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.9. Base: requisitos.md v1.11 · app 0.2.3 · roadmap 3.9 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.10. Base: requisitos.md v1.12 · app 0.3.0 · roadmap 3.10 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.11</t>
+          <t>Cambio en v1.12</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Todo control es alcanzable con teclado y muestra el foco; contrastes ≥ 4,5:1 medidos; el movimiento se reduce con prefers-reduced-motion; en pantallas táctiles, todo control y toda casilla del mástil mide al menos 40 × 40 px.</t>
+          <t>Todo control es alcanzable con teclado y muestra el foco; contrastes ≥ 4,5:1 medidos; el movimiento se reduce con prefers-reduced-motion; en pantallas táctiles, todo control y toda casilla del mástil mide al menos 40 × 40 px, salvo las cuerdas en vertical con menos de 660 px de alto, donde manda que la navegación no se salga.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>V-06: comprobar-disposicion.js en 14 pantallas (40 × 40 px, también con Ajustes abierto) · Banco (node --test): Ajustes inerte</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>Hecho: foco visible, movimiento reducido, interruptores con role="switch" (0.1.1), aria-pressed en los selectores y aviso del reto para lectores de pantalla (0.1.2). Falta: recorrer el mástil con teclado y auditar el contraste. Añadido al criterio el 20/10 (interfaz.md v1.0, aprobada el 20/10): en pantallas táctiles, todo control y toda casilla del mástil mide al menos 40 × 40 px.</t>
+          <t>Hecho: foco visible, movimiento reducido, interruptores con role="switch" (0.1.1), aria-pressed en los selectores y aviso del reto para lectores de pantalla (0.1.2). Desde la 0.3.0, con el dedo todo botón, desplegable e interruptor mide al menos 40 × 40 px, también en Ajustes, y las casillas del mástil también; Ajustes es un diálogo que deja inerte el resto, y el orden del tabulador sigue al visual (V-06). Excepción (AR-05): en vertical, en pantallas de menos de 660 px de alto (iPhone SE), manda que la navegación no se salga y las cuerdas pueden bajar de 40 px; el aviso para girar lo resuelve. Falta para F3.4: recorrer el mástil con teclado, auditar el contraste, que toda la fila de un interruptor responda al toque y el gesto de bajar para cerrar Ajustes.</t>
         </is>
       </c>
       <c r="P9" s="6" t="n"/>
@@ -1778,7 +1778,7 @@
       <c r="P18" s="6" t="n"/>
       <c r="Q18" s="5" t="inlineStr"/>
     </row>
-    <row r="19" ht="108" customHeight="1">
+    <row r="19" ht="120" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>PL-04</t>
@@ -1836,7 +1836,7 @@
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>docs/compatibilidad.md · Banco (node --test)</t>
+          <t>docs/compatibilidad.md v1.2 · Banco (node --test): sin matchMedia ni history</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
@@ -1851,11 +1851,15 @@
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>Decisión del 15/10. Inventario de capacidades, comportamiento por sistema y alternativas en docs/compatibilidad.md, que se revisa en cada etapa que añade una capacidad. Hoy ya se cumple para la vibración (se omite donde no existe) y para el audio interrumpido de iOS (0.1.4).</t>
+          <t>Decisión del 15/10. Inventario de capacidades, comportamiento por sistema y alternativas en docs/compatibilidad.md, que se revisa en cada etapa que añade una capacidad. Hoy ya se cumple para la vibración (se omite donde no existe) y para el audio interrumpido de iOS (0.1.4). En F3.2 (0.3.0) se añaden el tipo de puntero, el historial, grid y display: contents, y position: sticky, cada uno con su alternativa (compatibilidad.md v1.2), y el banco arranca la app sin ellos.</t>
         </is>
       </c>
       <c r="P19" s="6" t="n"/>
-      <c r="Q19" s="5" t="inlineStr"/>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="33" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
@@ -6481,27 +6485,27 @@
       </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>En horizontal, con un alto útil de 268 px o más, cada cuerda mide al menos 40 px (iPhone en Safari e instalada; simulador de Android). En vertical, en pantallas táctiles de menos de 600 px y en Libre, Adivinar y Escalas, aparece el aviso para girar; nunca en el Afinador; cerrado, no vuelve y «Restablecer» lo recupera.</t>
+          <t>En horizontal, con un alto útil de 268 px o más, cada cuerda mide al menos 40 px (iPhone en Safari e instalada; simulador de Android). En vertical, en pantallas táctiles de menos de 600 px de ancho y en Libre, Adivinar y Escalas, aparece el aviso para girar; nunca en el Afinador; cerrado, no vuelve y «Restablecer» lo recupera.</t>
         </is>
       </c>
       <c r="J79" s="5" t="inlineStr">
         <is>
-          <t>Cumple parcialmente</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K79" s="5" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="L79" s="5" t="inlineStr">
         <is>
-          <t>interfaz.md §7: bocetos medidos (52 px en el iPhone, 42 px en Android)</t>
+          <t>V-06: comprobar-disposicion.js en 14 pantallas: 52,8 / 60,8 / 42,5 px · Banco (node --test): aviso para girar</t>
         </is>
       </c>
       <c r="M79" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N79" s="5" t="inlineStr">
@@ -6511,7 +6515,7 @@
       </c>
       <c r="O79" s="5" t="inlineStr">
         <is>
-          <t>Criterio concreto el 20/10 (interfaz.md v1.0, aprobada el 20/10): el aviso sale solo en pantallas táctiles (pointer: coarse) en vertical de menos de 600 px de ancho, en Libre, Adivinar y Escalas, y nunca en el Afinador; si lo cierras, no vuelve (se guarda con los ajustes) y «Restablecer» lo recupera. En horizontal, raíl, mástil a todo el alto y panel: los bocetos dan 52 px por cuerda en el iPhone y 42 en un Android de 280 px de alto; los 40 px se exigen con un alto útil de 268 px o más. El bloqueo de orientación tiene mal soporte en iOS, así que no se fuerza.</t>
+          <t>Hecho en la 0.3.0 según interfaz.md §7. En horizontal, raíl, mástil a todo el alto y panel: medido en Chromium, 52,8 px por cuerda en el iPhone con Safari (antes 28,8), 60,8 con la app instalada y 42,5 en un Android de 280 px de alto (V-06). El aviso para girar sale solo con el dedo, en vertical y en pantallas de menos de 600 px de ancho, en Libre y Adivinar (y Escalas desde F5), nunca en el Afinador; cerrado no vuelve y «Restablecer» lo recupera. Falta validarlo en tu iPhone (Sesión 1). El bloqueo de orientación tiene mal soporte en iOS, así que no se fuerza.</t>
         </is>
       </c>
       <c r="P79" s="6" t="n"/>
@@ -6718,12 +6722,12 @@
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>El zoom cambia los trastes visibles entre 3 y el máximo que cabe, y la etiqueta dice la cifra real. Con pointer: coarse, un traste mide al menos 40 px y el zoom guardado se ajusta a ese límite.</t>
+          <t>El zoom cambia los trastes visibles entre 3 y el máximo que cabe, y la etiqueta dice la cifra real. Con pointer: coarse, un traste mide al menos 40 px; si el zoom guardado pide más trastes, se muestran los que caben y lo guardado se conserva (V-08).</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
-          <t>Cumple parcialmente</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K82" s="5" t="inlineStr">
@@ -6733,7 +6737,7 @@
       </c>
       <c r="L82" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7 y #8</t>
+          <t>F1.1 #7 y #8 · V-06: comprobar-disposicion.js en 14 pantallas · Banco (node --test): 40 px con el dedo</t>
         </is>
       </c>
       <c r="M82" s="5" t="inlineStr">
@@ -6748,7 +6752,7 @@
       </c>
       <c r="O82" s="5" t="inlineStr">
         <is>
-          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Añadido el 20/10 (interfaz.md v1.0, aprobada el 20/10): con pointer: coarse, un traste mide al menos 40 px y el zoom guardado se ajusta a ese límite; en el iPhone en vertical quedan como mucho 8 trastes a la vista. Se hace en F3.2.</t>
+          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Desde la 0.3.0, con el dedo un traste nunca mide menos de 40 px (34 con ratón), y la cejuela, 40: en el iPhone en vertical caben como mucho 7 trastes y en horizontal de 10 a 12 según el ancho (V-06). Si el zoom guardado pide más, se muestran los que caben y la etiqueta lo dice, pero lo guardado se conserva para que al girar vuelva (V-08).</t>
         </is>
       </c>
       <c r="P82" s="6" t="n"/>
@@ -7141,7 +7145,7 @@
       <c r="P87" s="6" t="n"/>
       <c r="Q87" s="5" t="inlineStr"/>
     </row>
-    <row r="88" ht="48" customHeight="1">
+    <row r="88" ht="78" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
         <is>
           <t>C-01</t>
@@ -7214,7 +7218,7 @@
       </c>
       <c r="O88" s="5" t="inlineStr">
         <is>
-          <t>Hoja que sube desde abajo en vertical; panel lateral en horizontal y en pantallas amplias (interfaz.md v1.0, aprobada el 20/10).</t>
+          <t>Hoja que sube desde abajo en vertical; panel lateral en horizontal y en pantallas amplias, con un segundo botón en el raíl (0.3.0). Es un diálogo: mientras está abierto, el resto de la página no responde (AT-04).</t>
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
@@ -7301,11 +7305,7 @@
         </is>
       </c>
       <c r="P89" s="6" t="n"/>
-      <c r="Q89" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q89" s="5" t="inlineStr"/>
     </row>
     <row r="90" ht="78" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
@@ -7380,7 +7380,7 @@
       </c>
       <c r="O90" s="5" t="inlineStr">
         <is>
-          <t>Nomenclatura y pentagrama en chips bajo la cabecera, o en el panel en horizontal; las dos pistas del juego, en la tarjeta del reto desde F3.2 (interfaz.md v1.0, aprobada el 20/10).</t>
+          <t>Nomenclatura y pentagrama en chips bajo la cabecera, o en el panel en horizontal, donde el pentagrama se rotula con la clave de sol; las dos pistas del juego, en la tarjeta del reto (0.3.0).</t>
         </is>
       </c>
       <c r="P90" s="6" t="n"/>
@@ -7390,7 +7390,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="63" customHeight="1">
+    <row r="91" ht="78" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
         <is>
           <t>C-04</t>
@@ -7463,7 +7463,7 @@
       </c>
       <c r="O91" s="5" t="inlineStr">
         <is>
-          <t>Barra inferior con cuatro destinos en vertical, raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (interfaz.md v1.0, aprobada el 20/10).</t>
+          <t>Barra inferior con cuatro destinos en vertical, raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05).</t>
         </is>
       </c>
       <c r="P91" s="6" t="n"/>
@@ -7629,13 +7629,9 @@
         </is>
       </c>
       <c r="P93" s="6" t="n"/>
-      <c r="Q93" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="78" customHeight="1">
+      <c r="Q93" s="5" t="inlineStr"/>
+    </row>
+    <row r="94" ht="120" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
         <is>
           <t>C-07</t>
@@ -7683,22 +7679,22 @@
       </c>
       <c r="J94" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="L94" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): historial simulado con popstate (3 pruebas)</t>
         </is>
       </c>
       <c r="M94" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N94" s="5" t="inlineStr">
@@ -7708,13 +7704,13 @@
       </c>
       <c r="O94" s="5" t="inlineStr">
         <is>
-          <t>Aprobado el 20/10 con interfaz.md v1.0. Usa el historial del navegador (history), estándar en todos los sistemas. En el iPhone instalado no hay botón atrás.</t>
+          <t>Hecho en la 0.3.0 con el historial del navegador (history): cada área tiene su dirección (#libre, #adivinar…). Un paso que deja la misma área, como tras recargar, se salta. El banco lo prueba con un historial simulado que avisa como el de verdad. Falta la prueba a mano en Windows y en el simulador de Android (Sesión 1). En el iPhone instalado no hay botón atrás.</t>
         </is>
       </c>
       <c r="P94" s="6" t="n"/>
       <c r="Q94" s="5" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Modificado</t>
         </is>
       </c>
     </row>
@@ -8684,7 +8680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8724,7 +8720,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -8734,24 +8730,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -8761,7 +8757,7 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
@@ -8771,14 +8767,14 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -8788,7 +8784,7 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
@@ -8798,24 +8794,24 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
@@ -8825,14 +8821,14 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -8842,24 +8838,24 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -8869,24 +8865,24 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -8896,51 +8892,51 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -8950,7 +8946,7 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
@@ -8960,32 +8956,59 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F3.4: resolver AR-06 y AT-05 y cerrar la etapa (G-05, L-03, J-12)
Ninguna casilla anuncia su nota en Adivinar; anillo para las posiciones
iguales con «ver todas»; asa con captura del puntero y sin rebote;
umbrales de la paleta escritos. Requisitos v1.13, matriz 1.11, roadmap
3.11 e interfaz 1.3. Fuera los .pyc, con .gitignore.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.10. Base: requisitos.md v1.12 · app 0.3.0 · roadmap 3.10 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.11. Base: requisitos.md v1.13 · app 0.3.1 · roadmap 3.11 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.12</t>
+          <t>Cambio en v1.13</t>
         </is>
       </c>
     </row>
@@ -1027,12 +1027,12 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Todo control es alcanzable con teclado y muestra el foco; contrastes ≥ 4,5:1 medidos; el movimiento se reduce con prefers-reduced-motion; en pantallas táctiles, todo control y toda casilla del mástil mide al menos 40 × 40 px, salvo las cuerdas en vertical con menos de 660 px de alto, donde manda que la navegación no se salga.</t>
+          <t>Todo control es alcanzable con teclado y muestra el foco; contrastes ≥ 4,5:1 medidos; el movimiento se reduce con prefers-reduced-motion; en pantallas táctiles, todo control y toda casilla del mástil mide al menos 40 × 40 px, salvo las cuerdas en vertical con menos de 660 px de alto. Paleta por nota: las 7 naturales a ≥ 7,5 (OKLab × 100) entre sí con visión normal y con protanopía, deuteranopía y tritanopía simuladas, y las 12 a ≥ 8 con visión normal; el nombre de la nota siempre escrito.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Cumple parcialmente</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -1042,12 +1042,12 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>V-06: comprobar-disposicion.js en 14 pantallas (40 × 40 px, también con Ajustes abierto) · Banco (node --test): Ajustes inerte</t>
+          <t>V-07: comprobar-accesibilidad.js (teclado, contraste, movimiento) · paleta.py · V-06: 40 × 40 px · Banco (node --test): teclado, etiquetas, paleta, grises, fila y asa</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>Hecho: foco visible, movimiento reducido, interruptores con role="switch" (0.1.1), aria-pressed en los selectores y aviso del reto para lectores de pantalla (0.1.2). Desde la 0.3.0, con el dedo todo botón, desplegable e interruptor mide al menos 40 × 40 px, también en Ajustes, y las casillas del mástil también; Ajustes es un diálogo que deja inerte el resto, y el orden del tabulador sigue al visual (V-06). Excepción (AR-05): en vertical, en pantallas de menos de 660 px de alto (iPhone SE), manda que la navegación no se salga y las cuerdas pueden bajar de 40 px; el aviso para girar lo resuelve. Falta para F3.4: recorrer el mástil con teclado, auditar el contraste, que toda la fila de un interruptor responda al toque y el gesto de bajar para cerrar Ajustes.</t>
+          <t>Hecho en la 0.3.1 (F3.4, V-07). Con el teclado se llega a todo y el foco se ve; el mástil es una cuadrícula (role="grid") que se recorre con las flechas y se toca con Intro; en Adivinar ninguna casilla anuncia su nota (J-12). Todos los textos a 4,5:1 o más, medidos en Chromium sobre su fondo real (con la 0.3.0 había 205 por debajo). Con «reducir movimiento» nada se anima. Con el dedo, controles y casillas de 40 × 40 px, también en Ajustes; la fila entera cambia su interruptor, y el asa cierra Ajustes deslizando. Paleta por nota con tu criterio del 20/10: 7 naturales bien separadas, también con daltonismo, y sostenidos derivados (herramientas/paleta.py). Excepción (AR-05): en vertical, por debajo de 660 px de alto, la navegación manda sobre los 40 px por cuerda. Falta probar con el dedo la fila y el asa en tu iPhone (Sesión 1).</t>
         </is>
       </c>
       <c r="P9" s="6" t="n"/>
@@ -1855,11 +1855,7 @@
         </is>
       </c>
       <c r="P19" s="6" t="n"/>
-      <c r="Q19" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q19" s="5" t="inlineStr"/>
     </row>
     <row r="20" ht="33" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
@@ -3875,7 +3871,7 @@
       <c r="P45" s="6" t="n"/>
       <c r="Q45" s="5" t="inlineStr"/>
     </row>
-    <row r="46" ht="63" customHeight="1">
+    <row r="46" ht="78" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>L-03</t>
@@ -3948,11 +3944,15 @@
       </c>
       <c r="O46" s="5" t="inlineStr">
         <is>
-          <t>Señal deliberadamente más tenue que la nota pulsada.</t>
+          <t>Desde la 0.3.1 se señalan con contorno, sin relleno, y con «Ver todas las notas» llevan además un anillo claro por fuera (AR-06). Señal deliberadamente más tenue que la nota pulsada.</t>
         </is>
       </c>
       <c r="P46" s="6" t="n"/>
-      <c r="Q46" s="5" t="inlineStr"/>
+      <c r="Q46" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="63" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
@@ -6519,11 +6519,7 @@
         </is>
       </c>
       <c r="P79" s="6" t="n"/>
-      <c r="Q79" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q79" s="5" t="inlineStr"/>
     </row>
     <row r="80" ht="33" customHeight="1">
       <c r="A80" s="4" t="inlineStr">
@@ -6756,11 +6752,7 @@
         </is>
       </c>
       <c r="P82" s="6" t="n"/>
-      <c r="Q82" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q82" s="5" t="inlineStr"/>
     </row>
     <row r="83" ht="33" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
@@ -7222,11 +7214,7 @@
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
-      <c r="Q88" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q88" s="5" t="inlineStr"/>
     </row>
     <row r="89" ht="78" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
@@ -7384,11 +7372,7 @@
         </is>
       </c>
       <c r="P90" s="6" t="n"/>
-      <c r="Q90" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q90" s="5" t="inlineStr"/>
     </row>
     <row r="91" ht="78" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
@@ -7467,11 +7451,7 @@
         </is>
       </c>
       <c r="P91" s="6" t="n"/>
-      <c r="Q91" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q91" s="5" t="inlineStr"/>
     </row>
     <row r="92" ht="33" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
@@ -7708,11 +7688,7 @@
         </is>
       </c>
       <c r="P94" s="6" t="n"/>
-      <c r="Q94" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q94" s="5" t="inlineStr"/>
     </row>
     <row r="95" ht="78" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
@@ -8680,7 +8656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8720,7 +8696,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -8730,24 +8706,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -8757,24 +8733,24 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -8784,7 +8760,7 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
@@ -8794,14 +8770,14 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -8811,7 +8787,7 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
@@ -8821,24 +8797,24 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
@@ -8848,14 +8824,14 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -8865,24 +8841,24 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -8892,24 +8868,24 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -8919,51 +8895,51 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -8973,7 +8949,7 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
@@ -8983,32 +8959,59 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F3: «+» enseña más trastes y se pueden pedir trastes de hasta 28 px con el dedo (V-04, G-05)
Comentario del cliente del 20/10. App 0.3.2. Requisitos v1.14, matriz
1.12, roadmap 3.12 e interfaz 1.4. Se audita en CP-3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.11. Base: requisitos.md v1.13 · app 0.3.1 · roadmap 3.11 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.12. Base: requisitos.md v1.14 · app 0.3.2 · roadmap 3.12 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.13</t>
+          <t>Cambio en v1.14</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Todo control es alcanzable con teclado y muestra el foco; contrastes ≥ 4,5:1 medidos; el movimiento se reduce con prefers-reduced-motion; en pantallas táctiles, todo control y toda casilla del mástil mide al menos 40 × 40 px, salvo las cuerdas en vertical con menos de 660 px de alto. Paleta por nota: las 7 naturales a ≥ 7,5 (OKLab × 100) entre sí con visión normal y con protanopía, deuteranopía y tritanopía simuladas, y las 12 a ≥ 8 con visión normal; el nombre de la nota siempre escrito.</t>
+          <t>Todo control es alcanzable con teclado y muestra el foco; contrastes ≥ 4,5:1 medidos; el movimiento se reduce con prefers-reduced-motion; en pantallas táctiles, todo control y toda casilla del mástil mide al menos 40 × 40 px en la vista por defecto, salvo las cuerdas en vertical con menos de 660 px de alto y los trastes que el usuario estreche con «+» (hasta 28 px). Paleta por nota: las 7 naturales a ≥ 7,5 (OKLab × 100) entre sí con visión normal y con protanopía, deuteranopía y tritanopía simuladas, y las 12 a ≥ 8 con visión normal; el nombre de la nota siempre escrito.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>Hecho en la 0.3.1 (F3.4, V-07). Con el teclado se llega a todo y el foco se ve; el mástil es una cuadrícula (role="grid") que se recorre con las flechas y se toca con Intro; en Adivinar ninguna casilla anuncia su nota (J-12). Todos los textos a 4,5:1 o más, medidos en Chromium sobre su fondo real (con la 0.3.0 había 205 por debajo). Con «reducir movimiento» nada se anima. Con el dedo, controles y casillas de 40 × 40 px, también en Ajustes; la fila entera cambia su interruptor, y el asa cierra Ajustes deslizando. Paleta por nota con tu criterio del 20/10: 7 naturales bien separadas, también con daltonismo, y sostenidos derivados (herramientas/paleta.py). Excepción (AR-05): en vertical, por debajo de 660 px de alto, la navegación manda sobre los 40 px por cuerda. Falta probar con el dedo la fila y el asa en tu iPhone (Sesión 1).</t>
+          <t>Hecho en la 0.3.1 (F3.4, V-07). Con el teclado se llega a todo y el foco se ve; el mástil es una cuadrícula (role="grid") que se recorre con las flechas y se toca con Intro; en Adivinar ninguna casilla anuncia su nota (J-12). Todos los textos a 4,5:1 o más, medidos en Chromium sobre su fondo real (con la 0.3.0 había 205 por debajo). Con «reducir movimiento» nada se anima. Con el dedo, controles y casillas de 40 × 40 px, también en Ajustes (salvo si pides más trastes con «+», que pueden estrecharse hasta 28 px); la fila entera cambia su interruptor, y el asa cierra Ajustes deslizando. Paleta por nota con tu criterio del 20/10: 7 naturales bien separadas, también con daltonismo, y sostenidos derivados (herramientas/paleta.py). Excepción (AR-05): en vertical, por debajo de 660 px de alto, la navegación manda sobre los 40 px por cuerda. Falta probar con el dedo la fila y el asa en tu iPhone (Sesión 1).</t>
         </is>
       </c>
       <c r="P9" s="6" t="n"/>
@@ -3948,11 +3948,7 @@
         </is>
       </c>
       <c r="P46" s="6" t="n"/>
-      <c r="Q46" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q46" s="5" t="inlineStr"/>
     </row>
     <row r="47" ht="63" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
@@ -6718,7 +6714,7 @@
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>El zoom cambia los trastes visibles entre 3 y el máximo que cabe, y la etiqueta dice la cifra real. Con pointer: coarse, un traste mide al menos 40 px; si el zoom guardado pide más trastes, se muestran los que caben y lo guardado se conserva (V-08).</t>
+          <t>El zoom cambia los trastes visibles entre 3 y el máximo que cabe, y la etiqueta dice la cifra real; «+» enseña más trastes y «−» menos. Con pointer: coarse, la vista por defecto usa trastes de al menos 40 px y el usuario puede pedir más trastes, de hasta 28 px; si el zoom guardado pide más de los que caben, se muestran los que caben y lo guardado se conserva (V-08).</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
@@ -6733,7 +6729,7 @@
       </c>
       <c r="L82" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7 y #8 · V-06: comprobar-disposicion.js en 14 pantallas · Banco (node --test): 40 px con el dedo</t>
+          <t>F1.1 #7 y #8 · V-06 · Banco (node --test): 40 px por defecto, 28 con «+», orden de los botones</t>
         </is>
       </c>
       <c r="M82" s="5" t="inlineStr">
@@ -6748,11 +6744,15 @@
       </c>
       <c r="O82" s="5" t="inlineStr">
         <is>
-          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Desde la 0.3.0, con el dedo un traste nunca mide menos de 40 px (34 con ratón), y la cejuela, 40: en el iPhone en vertical caben como mucho 7 trastes y en horizontal de 10 a 12 según el ancho (V-06). Si el zoom guardado pide más, se muestran los que caben y la etiqueta lo dice, pero lo guardado se conserva para que al girar vuelva (V-08).</t>
+          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Desde la 0.3.0, con el dedo la vista por defecto usa trastes de 40 px o más (34 con ratón), y la cejuela mide 40. Desde la 0.3.2 (tu comentario del 20/10), «+» enseña más trastes y «−» menos, y con el dedo puedes pedir trastes de hasta 28 px: en el iPhone con Safari, hasta 11 a la vista en vertical y 15 en horizontal. Si el zoom guardado pide más, se muestran los que caben y la etiqueta lo dice, pero lo guardado se conserva para que al girar vuelva (V-08).</t>
         </is>
       </c>
       <c r="P82" s="6" t="n"/>
-      <c r="Q82" s="5" t="inlineStr"/>
+      <c r="Q82" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="33" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
@@ -8656,7 +8656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8696,7 +8696,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -8706,24 +8706,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.3.1</t>
+          <t>0.3.2</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
+          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -8733,24 +8733,24 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -8760,24 +8760,24 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
@@ -8797,14 +8797,14 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
@@ -8824,24 +8824,24 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
@@ -8851,14 +8851,14 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -8868,24 +8868,24 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -8895,24 +8895,24 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -8922,51 +8922,51 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -8986,32 +8986,59 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
CP-3: correcciones de AR-07 y AT-06
- Sonido: el audio se rehace dentro de un toque (iOS solo deja arrancarlo
  ahí), el estado de Ajustes se actualiza solo y se evitan rehacer
  repetidos y textos atascados (AT-06 #1 a #6).
- Requisitos v1.15 corregida: 35 validados en la Sesión 1 (38 en total);
  J-01, J-08, J-10, S-02 y G-10 pendientes; evidencias por prueba.
- Informe V-08, roadmap, interfaz v1.5 y protocolo al día (AR-07).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -726,7 +726,7 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: A01</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>Naming cerrado: se descarta Trasting. Validado en la Sesión 1 (20/10, V-08): A01.</t>
+          <t>Naming cerrado: se descarta Trasting. Validado en la Sesión 1 (20/10, informe V-08): A01.</t>
         </is>
       </c>
       <c r="P5" s="6" t="n"/>
@@ -805,7 +805,7 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #1 y #14</t>
+          <t>F1.1 #1 y #14 · Sesión 1: A12</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>Escalas visible pero deshabilitada hasta F5. Validado en la Sesión 1 (20/10, V-08): A12.</t>
+          <t>Escalas visible pero deshabilitada hasta F5. Validado en la Sesión 1 (20/10, informe V-08): A12.</t>
         </is>
       </c>
       <c r="P6" s="6" t="n"/>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>V-07: comprobar-accesibilidad.js (teclado, contraste, movimiento) · paleta.py · V-06: 40 × 40 px · Banco (node --test): teclado, etiquetas, paleta, grises, fila y asa</t>
+          <t>V-07: comprobar-accesibilidad.js (teclado, contraste, movimiento) · paleta.py · V-06: 40 × 40 px · Banco (node --test): teclado, etiquetas, paleta, grises, fila y asa · Sesión 1: A18, C05 y C06</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>Hecho en la 0.3.1 (F3.4, V-07). Con el teclado se llega a todo y el foco se ve; el mástil es una cuadrícula (role="grid") que se recorre con las flechas y se toca con Intro; en Adivinar ninguna casilla anuncia su nota (J-12). Todos los textos a 4,5:1 o más, medidos en Chromium sobre su fondo real (con la 0.3.0 había 205 por debajo). Con «reducir movimiento» nada se anima. Con el dedo, controles y casillas de 40 × 40 px, también en Ajustes (salvo si pides más trastes con «+», que pueden estrecharse hasta 28 px); la fila entera cambia su interruptor, y el asa cierra Ajustes deslizando. Paleta por nota con tu criterio del 20/10: 7 naturales bien separadas, también con daltonismo, y sostenidos derivados (herramientas/paleta.py). Excepción (AR-05): en vertical, por debajo de 660 px de alto, la navegación manda sobre los 40 px por cuerda. Validado en la Sesión 1 (20/10, V-08): A18, C05 y C06.</t>
+          <t>Hecho en la 0.3.1 (F3.4, V-07). Con el teclado se llega a todo y el foco se ve; el mástil es una cuadrícula (role="grid") que se recorre con las flechas y se toca con Intro; en Adivinar ninguna casilla anuncia su nota (J-12). Todos los textos a 4,5:1 o más, medidos en Chromium sobre su fondo real (con la 0.3.0 había 205 por debajo). Con «reducir movimiento» nada se anima. Con el dedo, controles y casillas de 40 × 40 px, también en Ajustes (salvo si pides más trastes con «+», que pueden estrecharse hasta 28 px); la fila entera cambia su interruptor, y el asa cierra Ajustes deslizando. Paleta por nota con tu criterio del 20/10: 7 naturales bien separadas, también con daltonismo, y sostenidos derivados (herramientas/paleta.py). Excepción (AR-05): en vertical, por debajo de 660 px de alto, la navegación manda sobre los 40 px por cuerda. Validado en la Sesión 1 (20/10, informe V-08): A18, C05 y C06.</t>
         </is>
       </c>
       <c r="P9" s="6" t="n"/>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>V-03 y V-04: desde disco y sin conexión en Chromium, abre en 0,3 s y suena a menos de 1 cent · Banco (node --test): autónomo al día, con su audio, huellas y límites</t>
+          <t>V-03 y V-04: desde disco y sin conexión en Chromium, abre en 0,3 s y suena a menos de 1 cent · Banco (node --test): autónomo al día, con su audio, huellas y límites · Sesión 1: B02, B03, B04 y C09</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>dist/trasteando.html: la app con sus 17 grabaciones dentro (1,46 MB). Límites revisados en CP-2: el audio no pasa de 1,45 MB, y bajar su calidad exige tu escucha; el archivo entero no pasa de 2 MB, para dejar sitio al código de F3 a F6. Lo que cuenta para ti es que abra en ≤ 3 s en Windows: en Chromium tarda 0,3 s, y en tu PC se mide en la Sesión 1 (F2.5). Redacción limitada a Windows y Android tras AR-03. Validado en la Sesión 1 (20/10, V-08): B02, B03, B04 y C09.</t>
+          <t>dist/trasteando.html: la app con sus 17 grabaciones dentro (1,46 MB). Límites revisados en CP-2: el audio no pasa de 1,45 MB, y bajar su calidad exige tu escucha; el archivo entero no pasa de 2 MB, para dejar sitio al código de F3 a F6. Lo que cuenta para ti es que abra en ≤ 3 s en Windows: en Chromium tarda 0,3 s, y en tu PC se mide en la Sesión 1 (F2.5). Redacción limitada a Windows y Android tras AR-03. Validado en la Sesión 1 (20/10, informe V-08): B02, B03, B04 y C09.</t>
         </is>
       </c>
       <c r="P11" s="6" t="n"/>
@@ -1379,7 +1379,7 @@
       <c r="P13" s="6" t="n"/>
       <c r="Q13" s="5" t="inlineStr"/>
     </row>
-    <row r="14" ht="63" customHeight="1">
+    <row r="14" ht="108" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>G-10</t>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>Vincula cada versión con su fase del roadmap. Cada fase cerrada se marca además con una etiqueta de Git (F1.4). Validado en la Sesión 1 (20/10, V-08): A02.</t>
+          <t>Vincula cada versión con su fase del roadmap. Cada fase cerrada se marca además con una etiqueta de Git (F1.4). Sesión 1 (20/10, informe V-08): A02, la versión se ve en Ajustes. Se valida cuando existan las etiquetas v0.2.3 y v0.3.3 de los cierres de F2 y F3 (AR-07 #13).</t>
         </is>
       </c>
       <c r="P14" s="6" t="n"/>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>docs/compatibilidad.md v1.2 · Banco (node --test): sin matchMedia ni history</t>
+          <t>docs/compatibilidad.md v1.4 · Banco (node --test): sin matchMedia ni history</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>Decisión del 15/10. Inventario de capacidades, comportamiento por sistema y alternativas en docs/compatibilidad.md, que se revisa en cada etapa que añade una capacidad. Hoy ya se cumple para la vibración (se omite donde no existe) y para el audio interrumpido de iOS (0.1.4). En F3.2 (0.3.0) se añaden el tipo de puntero, el historial, grid y display: contents, y position: sticky, cada uno con su alternativa (compatibilidad.md v1.2), y el banco arranca la app sin ellos.</t>
+          <t>Decisión del 15/10. Inventario de capacidades, comportamiento por sistema y alternativas en docs/compatibilidad.md, que se revisa en cada etapa que añade una capacidad. Hoy ya se cumple para la vibración (se omite donde no existe) y para el audio interrumpido de iOS (0.1.4). En F3.2 (0.3.0) se añaden el tipo de puntero, el historial, grid y display: contents, y position: sticky, cada uno con su alternativa (compatibilidad.md v1.2), y el banco arranca la app sin ellos. Desde la 0.3.3: visibilitychange y suspend()/close() del audio, con su alternativa en compatibilidad.md v1.4.</t>
         </is>
       </c>
       <c r="P19" s="6" t="n"/>
@@ -1906,12 +1906,12 @@
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): A06.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A06.</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #6</t>
+          <t>F1.1 #6 · Sesión 1: A06</t>
         </is>
       </c>
       <c r="M20" s="5" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: A06</t>
         </is>
       </c>
       <c r="M22" s="5" t="inlineStr">
@@ -2076,13 +2076,13 @@
       </c>
       <c r="O22" s="5" t="inlineStr">
         <is>
-          <t>Chip en la barra de acceso rápido. Validado en la Sesión 1 (20/10, V-08): A06.</t>
+          <t>Chip en la barra de acceso rápido. Validado en la Sesión 1 (20/10, informe V-08): A06.</t>
         </is>
       </c>
       <c r="P22" s="6" t="n"/>
       <c r="Q22" s="5" t="inlineStr"/>
     </row>
-    <row r="23" ht="33" customHeight="1">
+    <row r="23" ht="48" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>N-04</t>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #6</t>
+          <t>F1.1 #6 · Sesión 1: A06</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="O23" s="5" t="inlineStr">
         <is>
-          <t>Verificar de nuevo al añadir Escalas (F5). Validado en la Sesión 1 (20/10, V-08): A06.</t>
+          <t>Verificar de nuevo al añadir Escalas (F5). Validado en la Sesión 1 (20/10, informe V-08): A06.</t>
         </is>
       </c>
       <c r="P23" s="6" t="n"/>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test) · F1.1 #11</t>
+          <t>Banco (node --test) · F1.1 #11 · Sesión 1: A11</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
-          <t>Sustituye al interruptor de la 0.1.1; quien lo tuviera apagado pasa automáticamente a «ninguno». Validado en la Sesión 1 (20/10, V-08): A11.</t>
+          <t>Sustituye al interruptor de la 0.1.1; quien lo tuviera apagado pasa automáticamente a «ninguno». Validado en la Sesión 1 (20/10, informe V-08): A11.</t>
         </is>
       </c>
       <c r="P28" s="6" t="n"/>
@@ -2605,12 +2605,12 @@
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): E03.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A03 y E03.</t>
         </is>
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #2</t>
+          <t>F1.1 #2 · Sesión 1: A03 y E03</t>
         </is>
       </c>
       <c r="M29" s="5" t="inlineStr">
@@ -2680,12 +2680,12 @@
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): E03.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): E03.</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: E03</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14 y #15 · V-05: escucha del cliente en su iPhone (0.2.0, 19/10)</t>
+          <t>F1.1 #14 y #15 · V-05: escucha del cliente en su iPhone (0.2.0, 19/10) · Sesión 1 (informe V-08): suena en el PC y el iPhone, pero en el iPhone se quedó mudo en C08 y D03; 0.3.3 con recuperación; pendiente de la Sesión 2</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>Reproductor propio con las grabaciones de samples/ desde la 0.2.0. Desde la 0.2.2 la guitarra clásica tiene también la grabación de La♯5: en afinación estándar ninguna nota se transporta más de 6 semitonos, y el traste 24 suena menos artificial. La acústica no tiene grabaciones por encima del Re5 y llega a 14: limitación conocida, aceptada por ti el 20/10; se comprueba de oído en la Sesión 1 (trastes 15 a 24 de la 1ª cuerda). Escuchada por ti en el iPhone con la 0.2.0 el 19/10 (V-05). La 0.1.3 corrigió el registro agudo de nylon, que sonaba medio tono alto. Sesión 1 (20/10, V-08): suena bien en el PC y en el iPhone, pero en el iPhone el sonido se quedó mudo dos veces (C08 y D03) y solo volvió cerrando la app; además seguía sonando con la pantalla bloqueada (C07). Es un fallo conocido de Safari en las apps de pantalla de inicio (WebKit 291892). Desde la 0.3.3, al ocultar la app se corta el sonido y se pausa el audio; al volver se reanuda, y si iOS no lo suelta se crea un audio nuevo; Ajustes enseña el estado del sonido y tiene «Reactivar sonido». Se valida cuando la Sesión 2 confirme que no vuelve a quedarse mudo.</t>
+          <t>Reproductor propio con las grabaciones de samples/ desde la 0.2.0. Desde la 0.2.2 la guitarra clásica tiene también la grabación de La♯5: en afinación estándar ninguna nota se transporta más de 6 semitonos, y el traste 24 suena menos artificial. La acústica no tiene grabaciones por encima del Re5 y llega a 14: limitación conocida, aceptada por ti el 20/10; se comprueba de oído en la Sesión 1 (trastes 15 a 24 de la 1ª cuerda). Escuchada por ti en el iPhone con la 0.2.0 el 19/10 (V-05). La 0.1.3 corrigió el registro agudo de nylon, que sonaba medio tono alto. Sesión 1 (20/10, informe V-08): suena bien en el PC y en el iPhone, pero en el iPhone el sonido se quedó mudo dos veces (C08 y D03) y solo volvió cerrando la app; además seguía sonando con la pantalla bloqueada (C07). Es un fallo conocido de Safari en las apps de pantalla de inicio (WebKit 291892). Desde la 0.3.3, al ocultar la app se corta el sonido y se pausa el audio; al volver se reanuda, y si iOS no lo suelta se crea un audio nuevo; Ajustes enseña el estado del sonido y tiene «Reactivar sonido». Se valida cuando la Sesión 2 confirme que no vuelve a quedarse mudo.</t>
         </is>
       </c>
       <c r="P32" s="6" t="n"/>
@@ -2860,7 +2860,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="108" customHeight="1">
+    <row r="33" ht="120" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
           <t>S-02</t>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="N33" s="5" t="inlineStr">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="O33" s="5" t="inlineStr">
         <is>
-          <t>Cambiar de timbre descarga otro set de muestras, con aviso. Desde 0.1.2, dos cambios seguidos ya no muestran el mensaje de la carga descartada. Desde la 0.3.3 (Sesión 1, A14), elegir guitarra ya no hace sonar una nota de muestra. Validado en la Sesión 1 (20/10, V-08): A14.</t>
+          <t>Cambiar de timbre descarga otro set de muestras, con aviso. Desde 0.1.2, dos cambios seguidos ya no muestran el mensaje de la carga descartada. Desde la 0.3.3 (Sesión 1, A14), elegir guitarra ya no hace sonar una nota de muestra. Sesión 1 (20/10, informe V-08): lo esencial cumplió en A14; el cambio de la 0.3.3 lo pediste tú y se confirma en la Sesión 2.</t>
         </is>
       </c>
       <c r="P33" s="6" t="n"/>
@@ -2996,12 +2996,12 @@
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): A03.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A14.</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: A14</t>
         </is>
       </c>
       <c r="M34" s="5" t="inlineStr">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>Análisis 15/09: ninguna nota fuera en todo el rango · F1.1 #3 y #4</t>
+          <t>Análisis 15/09: ninguna nota fuera en todo el rango · F1.1 #3 y #4 · Sesión 1: A05</t>
         </is>
       </c>
       <c r="M41" s="5" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="O41" s="5" t="inlineStr">
         <is>
-          <t>Clave de sol octavada. Desde 0.1.1 las notas muy agudas o graves se dibujan transportadas con 8va, 15ma u 8vb, y la clave es un trazado propio que no depende de las fuentes del sistema. Validado en la Sesión 1 (20/10, V-08): A05.</t>
+          <t>Clave de sol octavada. Desde 0.1.1 las notas muy agudas o graves se dibujan transportadas con 8va, 15ma u 8vb, y la clave es un trazado propio que no depende de las fuentes del sistema. Validado en la Sesión 1 (20/10, informe V-08): A05.</t>
         </is>
       </c>
       <c r="P41" s="6" t="n"/>
@@ -3782,12 +3782,12 @@
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): A13.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A13.</t>
         </is>
       </c>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: A13</t>
         </is>
       </c>
       <c r="M44" s="5" t="inlineStr">
@@ -3857,12 +3857,12 @@
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): A01.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A01.</t>
         </is>
       </c>
       <c r="L45" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: A01</t>
         </is>
       </c>
       <c r="M45" s="5" t="inlineStr">
@@ -3937,7 +3937,7 @@
       </c>
       <c r="L46" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test) · F1.1 #10</t>
+          <t>Banco (node --test) · F1.1 #10 · Sesión 1: A10</t>
         </is>
       </c>
       <c r="M46" s="5" t="inlineStr">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="O46" s="5" t="inlineStr">
         <is>
-          <t>Por defecto solo la pulsada, para no convertir el mástil en una chuleta permanente. En Adivinar no se aplica (J-12). Validado en la Sesión 1 (20/10, V-08): A10.</t>
+          <t>Por defecto solo la pulsada, para no convertir el mástil en una chuleta permanente. En Adivinar no se aplica (J-12). Validado en la Sesión 1 (20/10, informe V-08): A10.</t>
         </is>
       </c>
       <c r="P46" s="6" t="n"/>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="L47" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: E03</t>
         </is>
       </c>
       <c r="M47" s="5" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="O47" s="5" t="inlineStr">
         <is>
-          <t>Desde la 0.3.1 se señalan con contorno, sin relleno, y con «Ver todas las notas» llevan además un anillo claro por fuera (AR-06). Señal deliberadamente más tenue que la nota pulsada. Validado en la Sesión 1 (20/10, V-08): E03.</t>
+          <t>Desde la 0.3.1 se señalan con contorno, sin relleno, y con «Ver todas las notas» llevan además un anillo claro por fuera (AR-06). Señal deliberadamente más tenue que la nota pulsada. Validado en la Sesión 1 (20/10, informe V-08): E03.</t>
         </is>
       </c>
       <c r="P47" s="6" t="n"/>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="M48" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="N48" s="5" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="O48" s="5" t="inlineStr">
         <is>
-          <t>Con botón para repetir el sonido. Desde 0.1.1 los retos se limitan a los 12 primeros trastes por defecto, y desplazar el mástil ya no cuenta como pulsación. Desde la 0.3.3 (Sesión 1, E06), al entrar en Adivinar no suena nada hasta pulsar ▶, que aparece resaltado; antes de ▶ se puede tocar el mástil sin que puntúe. Después cada reto suena solo, y ▶ lo repite. La lectura grande y el pentagrama muestran la nota buscada («?» hasta acertar o fallar), no la pulsada. Validado en la Sesión 1 (20/10, V-08): C07 y E04.</t>
+          <t>Con botón para repetir el sonido. Desde 0.1.1 los retos se limitan a los 12 primeros trastes por defecto, y desplazar el mástil ya no cuenta como pulsación. Desde la 0.3.3 (Sesión 1, E06), al entrar en Adivinar no suena nada hasta pulsar ▶, que aparece resaltado; antes de ▶ se puede tocar el mástil sin que puntúe. Después cada reto suena solo, y ▶ lo repite. La lectura grande y el pentagrama muestran la nota buscada («?» hasta acertar o fallar), no la pulsada. Sesión 1 (20/10, informe V-08): lo esencial cumplió en C07 y E04; el cambio de la 0.3.3 lo pediste tú y se confirma en la Sesión 2.</t>
         </is>
       </c>
       <c r="P48" s="6" t="n"/>
@@ -4173,12 +4173,12 @@
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): E04.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): E04.</t>
         </is>
       </c>
       <c r="L49" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): acierto</t>
+          <t>Banco (node --test): acierto · Sesión 1: E04</t>
         </is>
       </c>
       <c r="M49" s="5" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="L50" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: E04</t>
         </is>
       </c>
       <c r="M50" s="5" t="inlineStr">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="O50" s="5" t="inlineStr">
         <is>
-          <t>Reutiliza la lógica de L-03. Validado en la Sesión 1 (20/10, V-08): E04.</t>
+          <t>Reutiliza la lógica de L-03. Validado en la Sesión 1 (20/10, informe V-08): E04.</t>
         </is>
       </c>
       <c r="P50" s="6" t="n"/>
@@ -4327,12 +4327,12 @@
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): E04.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): E04.</t>
         </is>
       </c>
       <c r="L51" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: E04</t>
         </is>
       </c>
       <c r="M51" s="5" t="inlineStr">
@@ -4402,12 +4402,12 @@
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): E04.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): E04.</t>
         </is>
       </c>
       <c r="L52" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: E04</t>
         </is>
       </c>
       <c r="M52" s="5" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="L53" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: E04</t>
         </is>
       </c>
       <c r="M53" s="5" t="inlineStr">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="O53" s="5" t="inlineStr">
         <is>
-          <t>Con las dos pistas activas equivale a «busca esta nota en esta cuerda»; sin ninguna, a «adivina de oído». Validado en la Sesión 1 (20/10, V-08): E04.</t>
+          <t>Con las dos pistas activas equivale a «busca esta nota en esta cuerda»; sin ninguna, a «adivina de oído». Validado en la Sesión 1 (20/10, informe V-08): E04.</t>
         </is>
       </c>
       <c r="P53" s="6" t="n"/>
@@ -4556,12 +4556,12 @@
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): E04.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): E04.</t>
         </is>
       </c>
       <c r="L54" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): acierto y fallo</t>
+          <t>Banco (node --test): acierto y fallo · Sesión 1: E04</t>
         </is>
       </c>
       <c r="M54" s="5" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>El récord persiste tras recargar y tras «Restablecer todos los ajustes»; solo «Borrar el récord» lo pone a cero.</t>
+          <t>El récord persiste tras recargar y tras «Restablecer todos los ajustes»; solo «Borrar el récord de racha» lo pone a cero.</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
@@ -4641,7 +4641,7 @@
       </c>
       <c r="M55" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N55" s="5" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="O55" s="5" t="inlineStr">
         <is>
-          <t>localStorage. No funciona en las previsualizaciones de artefactos; probar en local o en la web. Desde la 0.3.3 (Sesión 1, A14), «Restablecer todos los ajustes» conserva el récord, que se borra con su propio botón en Ajustes. No hacen falta usuarios: el récord es tuyo y vive en este navegador. Validado en la Sesión 1 (20/10, V-08): A15.</t>
+          <t>localStorage. No funciona en las previsualizaciones de artefactos; probar en local o en la web. Desde la 0.3.3 (Sesión 1, A14), «Restablecer todos los ajustes» conserva el récord, que se borra con su propio botón en Ajustes. No hacen falta usuarios: el récord es tuyo y vive en este navegador. Sesión 1 (20/10, informe V-08): lo esencial cumplió en A15; el cambio de la 0.3.3 lo pediste tú y se confirma en la Sesión 2.</t>
         </is>
       </c>
       <c r="P55" s="6" t="n"/>
@@ -4719,7 +4719,7 @@
       </c>
       <c r="L56" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #9</t>
+          <t>F1.1 #9 · Sesión 1: A09 y E04</t>
         </is>
       </c>
       <c r="M56" s="5" t="inlineStr">
@@ -4734,7 +4734,7 @@
       </c>
       <c r="O56" s="5" t="inlineStr">
         <is>
-          <t>Color en la posición pulsada y destello en la barra del reto. Validado en la Sesión 1 (20/10, V-08): A09 y E04.</t>
+          <t>Color en la posición pulsada y destello en la barra del reto. Validado en la Sesión 1 (20/10, informe V-08): A09 y E04.</t>
         </is>
       </c>
       <c r="P56" s="6" t="n"/>
@@ -4803,7 +4803,7 @@
       </c>
       <c r="M57" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N57" s="5" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="O57" s="5" t="inlineStr">
         <is>
-          <t>El fallo rompe la racha siempre. Se iluminan todas las posiciones correctas y se vuelve a oír la nota buscada justo después de la pulsada, para aprender por contraste; luego llega el reto siguiente. Desde la 0.3.3 (Sesión 1, A09), la corrección llega a los 1,2 s (antes 0,65) y el reto siguiente 3 s después, para poder comparar las dos notas; el fallo se rellena en rojo con ✗ y las posiciones correctas en verde con ✓, de modo que no dependa solo del color. Validado en la Sesión 1 (20/10, V-08): A09.</t>
+          <t>El fallo rompe la racha siempre. Se iluminan todas las posiciones correctas y se vuelve a oír la nota buscada justo después de la pulsada, para aprender por contraste; luego llega el reto siguiente. Desde la 0.3.3 (Sesión 1, A09), la corrección llega a los 1,2 s (antes 0,65) y el reto siguiente 3 s después, para poder comparar las dos notas; el fallo se rellena en rojo con ✗ y las posiciones correctas en verde con ✓, de modo que no dependa solo del color. Sesión 1 (20/10, informe V-08): lo esencial cumplió en A09; el cambio de la 0.3.3 lo pediste tú y se confirma en la Sesión 2.</t>
         </is>
       </c>
       <c r="P57" s="6" t="n"/>
@@ -4960,7 +4960,7 @@
       </c>
       <c r="L59" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test) · F1.1 #10</t>
+          <t>Banco (node --test) · F1.1 #10 · Sesión 1: A10</t>
         </is>
       </c>
       <c r="M59" s="5" t="inlineStr">
@@ -4975,7 +4975,7 @@
       </c>
       <c r="O59" s="5" t="inlineStr">
         <is>
-          <t>Encontrado al revisar el código: con «ver todas las notas» activo, el juego mostraba la solución. Validado en la Sesión 1 (20/10, V-08): A10.</t>
+          <t>Encontrado al revisar el código: con «ver todas las notas» activo, el juego mostraba la solución. Validado en la Sesión 1 (20/10, informe V-08): A10.</t>
         </is>
       </c>
       <c r="P59" s="6" t="n"/>
@@ -6225,7 +6225,7 @@
       <c r="P75" s="6" t="n"/>
       <c r="Q75" s="5" t="inlineStr"/>
     </row>
-    <row r="76" ht="48" customHeight="1">
+    <row r="76" ht="63" customHeight="1">
       <c r="A76" s="4" t="inlineStr">
         <is>
           <t>A-08</t>
@@ -6283,7 +6283,7 @@
       </c>
       <c r="L76" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #4</t>
+          <t>F1.1 #4 · Sesión 1: A13</t>
         </is>
       </c>
       <c r="M76" s="5" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="O76" s="5" t="inlineStr">
         <is>
-          <t>Cualquier ajuste convierte la afinación en personalizada sin alterar los presets. Validado en la Sesión 1 (20/10, V-08): A13.</t>
+          <t>Cualquier ajuste convierte la afinación en personalizada sin alterar los presets. Validado en la Sesión 1 (20/10, informe V-08): A13.</t>
         </is>
       </c>
       <c r="P76" s="6" t="n"/>
@@ -6595,7 +6595,7 @@
       </c>
       <c r="L80" s="5" t="inlineStr">
         <is>
-          <t>V-06: comprobar-disposicion.js en 14 pantallas: 52,8 / 60,8 / 42,5 px · Banco (node --test): aviso para girar</t>
+          <t>V-06: comprobar-disposicion.js en 14 pantallas: 52,8 / 60,8 / 42,5 px · Banco (node --test): aviso para girar · Sesión 1: C02, C03 y D03</t>
         </is>
       </c>
       <c r="M80" s="5" t="inlineStr">
@@ -6610,7 +6610,7 @@
       </c>
       <c r="O80" s="5" t="inlineStr">
         <is>
-          <t>Hecho en la 0.3.0 según interfaz.md §7. En horizontal, raíl, mástil a todo el alto y panel: medido en Chromium, 52,8 px por cuerda en el iPhone con Safari (antes 28,8), 60,8 con la app instalada y 42,5 en un Android de 280 px de alto (V-06). El aviso para girar sale solo con el dedo, en vertical y en pantallas de menos de 600 px de ancho, en Libre y Adivinar (y Escalas desde F5), nunca en el Afinador; cerrado no vuelve y «Restablecer» lo recupera. El bloqueo de orientación tiene mal soporte en iOS, así que no se fuerza. Validado en la Sesión 1 (20/10, V-08): C02, C03 y D03.</t>
+          <t>Hecho en la 0.3.0 según interfaz.md §7. En horizontal, raíl, mástil a todo el alto y panel: medido en Chromium, 52,8 px por cuerda en el iPhone con Safari (antes 28,8), 60,8 con la app instalada y 42,5 en un Android de 280 px de alto (V-06). El aviso para girar sale solo con el dedo, en vertical y en pantallas de menos de 600 px de ancho, en Libre y Adivinar (y Escalas desde F5), nunca en el Afinador; cerrado no vuelve y «Restablecer» lo recupera. El bloqueo de orientación tiene mal soporte en iOS, así que no se fuerza. Validado en la Sesión 1 (20/10, informe V-08): C02, C03 y D03.</t>
         </is>
       </c>
       <c r="P80" s="6" t="n"/>
@@ -6828,7 +6828,7 @@
       </c>
       <c r="L83" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7 y #8 · V-06 · Banco (node --test): 40 px por defecto, 28 con «+», orden de los botones</t>
+          <t>F1.1 #7 y #8 · V-06 · Banco (node --test): 40 px por defecto, 28 con «+», orden de los botones · Sesión 1: A07, A08 y C04</t>
         </is>
       </c>
       <c r="M83" s="5" t="inlineStr">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="O83" s="5" t="inlineStr">
         <is>
-          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Desde la 0.3.0, con el dedo la vista por defecto usa trastes de 40 px o más (34 con ratón), y la cejuela mide 40. Desde la 0.3.2 (tu comentario del 20/10), «+» enseña más trastes y «−» menos, y con el dedo puedes pedir trastes de hasta 28 px: en el iPhone con Safari, hasta 11 a la vista en vertical y 15 en horizontal. Si el zoom guardado pide más, se muestran los que caben y la etiqueta lo dice, pero lo guardado se conserva para que al girar vuelva (V-08). Validado en la Sesión 1 (20/10, V-08): A07, A08 y C04.</t>
+          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Desde la 0.3.0, con el dedo la vista por defecto usa trastes de 40 px o más (34 con ratón), y la cejuela mide 40. Desde la 0.3.2 (tu comentario del 20/10), «+» enseña más trastes y «−» menos, y con el dedo puedes pedir trastes de hasta 28 px: en el iPhone con Safari, hasta 11 a la vista en vertical y 15 en horizontal. Si el zoom guardado pide más, se muestran los que caben y la etiqueta lo dice, pero lo guardado se conserva para que al girar vuelva (V-08). Validado en la Sesión 1 (20/10, informe V-08): A07, A08 y C04.</t>
         </is>
       </c>
       <c r="P83" s="6" t="n"/>
@@ -6902,12 +6902,12 @@
       </c>
       <c r="K84" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): A08.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A08.</t>
         </is>
       </c>
       <c r="L84" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: A08</t>
         </is>
       </c>
       <c r="M84" s="5" t="inlineStr">
@@ -6977,12 +6977,12 @@
       </c>
       <c r="K85" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): A07.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A07.</t>
         </is>
       </c>
       <c r="L85" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7</t>
+          <t>F1.1 #7 · Sesión 1: A07</t>
         </is>
       </c>
       <c r="M85" s="5" t="inlineStr">
@@ -7052,12 +7052,12 @@
       </c>
       <c r="K86" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, `V-08`): A08.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A08.</t>
         </is>
       </c>
       <c r="L86" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7</t>
+          <t>F1.1 #7 · Sesión 1: A08</t>
         </is>
       </c>
       <c r="M86" s="5" t="inlineStr">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="L88" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test) · F1.1 #11</t>
+          <t>Banco (node --test) · F1.1 #11 · Sesión 1: A11</t>
         </is>
       </c>
       <c r="M88" s="5" t="inlineStr">
@@ -7226,13 +7226,13 @@
       </c>
       <c r="O88" s="5" t="inlineStr">
         <is>
-          <t>Sin números, los trastes 5 y 17 llevan la misma marca y se confunden. Se descartó el minimapa por desproporcionado. Validado en la Sesión 1 (20/10, V-08): A11.</t>
+          <t>Sin números, los trastes 5 y 17 llevan la misma marca y se confunden. Se descartó el minimapa por desproporcionado. Validado en la Sesión 1 (20/10, informe V-08): A11.</t>
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
       <c r="Q88" s="5" t="inlineStr"/>
     </row>
-    <row r="89" ht="93" customHeight="1">
+    <row r="89" ht="108" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
         <is>
           <t>C-01</t>
@@ -7290,7 +7290,7 @@
       </c>
       <c r="L89" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: A19 y C05</t>
         </is>
       </c>
       <c r="M89" s="5" t="inlineStr">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="O89" s="5" t="inlineStr">
         <is>
-          <t>Hoja que sube desde abajo en vertical; panel lateral en horizontal y en pantallas amplias, con un segundo botón en el raíl (0.3.0). Es un diálogo: mientras está abierto, el resto de la página no responde (AT-04). Validado en la Sesión 1 (20/10, V-08): A19 y C05.</t>
+          <t>Hoja que sube desde abajo en vertical; panel lateral en horizontal y en pantallas amplias, con un segundo botón en el raíl (0.3.0). Es un diálogo: mientras está abierto, el resto de la página no responde (AT-04). Validado en la Sesión 1 (20/10, informe V-08): A19 y C05.</t>
         </is>
       </c>
       <c r="P89" s="6" t="n"/>
@@ -7527,7 +7527,7 @@
       </c>
       <c r="L92" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #14 · Sesión 1: A19</t>
         </is>
       </c>
       <c r="M92" s="5" t="inlineStr">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="O92" s="5" t="inlineStr">
         <is>
-          <t>Barra inferior con cuatro destinos en vertical, raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05). Validado en la Sesión 1 (20/10, V-08): A19.</t>
+          <t>Barra inferior con cuatro destinos en vertical, raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05). Validado en la Sesión 1 (20/10, informe V-08): A19.</t>
         </is>
       </c>
       <c r="P92" s="6" t="n"/>
@@ -7606,7 +7606,7 @@
       </c>
       <c r="L93" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): migración · F1.1 #13</t>
+          <t>Banco (node --test): migración · F1.1 #13 · Sesión 1: A14 y A15</t>
         </is>
       </c>
       <c r="M93" s="5" t="inlineStr">
@@ -7621,7 +7621,7 @@
       </c>
       <c r="O93" s="5" t="inlineStr">
         <is>
-          <t>Un único objeto de estado, validado campo a campo al leerlo (0.1.1). Validado en la Sesión 1 (20/10, V-08): A14 y A15.</t>
+          <t>Un único objeto de estado, validado campo a campo al leerlo (0.1.1). Validado en la Sesión 1 (20/10, informe V-08): A14 y A15.</t>
         </is>
       </c>
       <c r="P93" s="6" t="n"/>
@@ -7764,7 +7764,7 @@
       </c>
       <c r="L95" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): historial simulado con popstate (3 pruebas)</t>
+          <t>Banco (node --test): historial simulado con popstate (3 pruebas) · Sesión 1: A17</t>
         </is>
       </c>
       <c r="M95" s="5" t="inlineStr">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="O95" s="5" t="inlineStr">
         <is>
-          <t>Hecho en la 0.3.0 con el historial del navegador (history): cada área tiene su dirección (#libre, #adivinar…). Un paso que deja la misma área, como tras recargar, se salta. El banco lo prueba con un historial simulado que avisa como el de verdad. Falta la prueba a mano en Windows y en el simulador de Android (Sesión 1). En el iPhone instalado no hay botón atrás. Validado en la Sesión 1 (20/10, V-08): A17.</t>
+          <t>Hecho en la 0.3.0 con el historial del navegador (history): cada área tiene su dirección (#libre, #adivinar…). Un paso que deja la misma área, como tras recargar, se salta. El banco lo prueba con un historial simulado que avisa como el de verdad. Falta la prueba a mano en Windows y en el simulador de Android (Sesión 1). En el iPhone instalado no hay botón atrás. Validado en la Sesión 1 (20/10, informe V-08): A17.</t>
         </is>
       </c>
       <c r="P95" s="6" t="n"/>
@@ -8894,7 +8894,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Sesión 1: 40 requisitos verificados en el iPhone y el PC del cliente (V-08). Criterios nuevos de J-01, J-08, J-10 y S-02; C-08 y S-09 nuevos, fuera de alcance.</t>
+          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F4: documentos de la 0.4.0 (requisitos v1.16, V-09, IT-02)
- requisitos.md v1.16: A-02 a A-05 y A-02-CA implementados; A-02-CA,
  A-04 y G-10 validados; G-08 y PL-04 con notas. Matriz v1.14.
- roadmap v3.14, compatibilidad v1.5, CHANGELOG 0.4.0.
- Informe V-09 con la comprobación de 10 minutos con la guitarra, e
  informe didáctico IT-02.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.13. Base: requisitos.md v1.15 · app 0.3.3 · roadmap 3.13 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.14. Base: requisitos.md v1.16 · app 0.4.0 · roadmap 3.14 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.15</t>
+          <t>Cambio en v1.16</t>
         </is>
       </c>
     </row>
@@ -1294,11 +1294,15 @@
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>Desde la 0.2.1 hay dos formas reales: index.html para servir (Live Server y web) y dist/trasteando.html, generado a partir de él con herramientas/generar-autonomo.py. El banco comprueba que el autónomo está al día con index.html. Se vuelve más exigente al pasar a módulos (F4.1); F6.1 generará el archivo autónomo a partir de ellos.</t>
+          <t>Desde la 0.2.1 hay dos formas reales: index.html para servir (Live Server y web) y dist/trasteando.html, generado a partir de él con herramientas/generar-autonomo.py. El banco comprueba que el autónomo está al día con index.html. Se vuelve más exigente al pasar a módulos (F4.1); F6.1 generará el archivo autónomo a partir de ellos. Desde la 0.4.0 (F4.1), la app vive en varios archivos (css/ y js/, uno por tema); herramientas/ensamblar.js los une para el archivo autónomo, y el banco comprueba que este es exactamente la app más su audio.</t>
         </is>
       </c>
       <c r="P12" s="6" t="n"/>
-      <c r="Q12" s="5" t="inlineStr"/>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="63" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -1379,7 +1383,7 @@
       <c r="P13" s="6" t="n"/>
       <c r="Q13" s="5" t="inlineStr"/>
     </row>
-    <row r="14" ht="108" customHeight="1">
+    <row r="14" ht="120" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>G-10</t>
@@ -1442,7 +1446,7 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Verificado parcialmente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -1452,11 +1456,15 @@
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>Vincula cada versión con su fase del roadmap. Cada fase cerrada se marca además con una etiqueta de Git (F1.4). Sesión 1 (20/10, informe V-08): A02, la versión se ve en Ajustes. Se valida cuando existan las etiquetas v0.2.3 y v0.3.3 de los cierres de F2 y F3 (AR-07 #13).</t>
+          <t>Vincula cada versión con su fase del roadmap. Cada fase cerrada se marca además con una etiqueta de Git (F1.4). Validado el 21/10: la Sesión 1 (A02) vio la versión en Ajustes, CHANGELOG tiene cada versión y existen las etiquetas v0.1.5, v0.2.3 y v0.3.3 de los cierres de F1, F2 y F3 (las creaste tú en GitHub).</t>
         </is>
       </c>
       <c r="P14" s="6" t="n"/>
-      <c r="Q14" s="5" t="inlineStr"/>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="63" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1847,11 +1855,15 @@
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>Decisión del 15/10. Inventario de capacidades, comportamiento por sistema y alternativas en docs/compatibilidad.md, que se revisa en cada etapa que añade una capacidad. Hoy ya se cumple para la vibración (se omite donde no existe) y para el audio interrumpido de iOS (0.1.4). En F3.2 (0.3.0) se añaden el tipo de puntero, el historial, grid y display: contents, y position: sticky, cada uno con su alternativa (compatibilidad.md v1.2), y el banco arranca la app sin ellos. Desde la 0.3.3: visibilitychange y suspend()/close() del audio, con su alternativa en compatibilidad.md v1.4.</t>
+          <t>Decisión del 15/10. Inventario de capacidades, comportamiento por sistema y alternativas en docs/compatibilidad.md, que se revisa en cada etapa que añade una capacidad. Hoy ya se cumple para la vibración (se omite donde no existe) y para el audio interrumpido de iOS (0.1.4). En F3.2 (0.3.0) se añaden el tipo de puntero, el historial, grid y display: contents, y position: sticky, cada uno con su alternativa (compatibilidad.md v1.2), y el banco arranca la app sin ellos. Desde la 0.3.3: visibilitychange y suspend()/close() del audio, con su alternativa en compatibilidad.md v1.4. Desde la 0.4.0: hilo aparte (Worker), con el detector en el principal si falta, y micrófono (getUserMedia), con el motivo y De oído si falta (compatibilidad.md v1.5).</t>
         </is>
       </c>
       <c r="P19" s="6" t="n"/>
-      <c r="Q19" s="5" t="inlineStr"/>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="33" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
@@ -2854,11 +2866,7 @@
         </is>
       </c>
       <c r="P32" s="6" t="n"/>
-      <c r="Q32" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q32" s="5" t="inlineStr"/>
     </row>
     <row r="33" ht="120" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -2937,11 +2945,7 @@
         </is>
       </c>
       <c r="P33" s="6" t="n"/>
-      <c r="Q33" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q33" s="5" t="inlineStr"/>
     </row>
     <row r="34" ht="33" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
@@ -3486,11 +3490,7 @@
         </is>
       </c>
       <c r="P40" s="6" t="n"/>
-      <c r="Q40" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="Q40" s="5" t="inlineStr"/>
     </row>
     <row r="41" ht="93" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
@@ -4114,11 +4114,7 @@
         </is>
       </c>
       <c r="P48" s="6" t="n"/>
-      <c r="Q48" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q48" s="5" t="inlineStr"/>
     </row>
     <row r="49" ht="33" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
@@ -4655,11 +4651,7 @@
         </is>
       </c>
       <c r="P55" s="6" t="n"/>
-      <c r="Q55" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q55" s="5" t="inlineStr"/>
     </row>
     <row r="56" ht="48" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
@@ -4817,11 +4809,7 @@
         </is>
       </c>
       <c r="P57" s="6" t="n"/>
-      <c r="Q57" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q57" s="5" t="inlineStr"/>
     </row>
     <row r="58" ht="48" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
@@ -5684,7 +5672,7 @@
       <c r="P68" s="6" t="n"/>
       <c r="Q68" s="5" t="inlineStr"/>
     </row>
-    <row r="69" ht="93" customHeight="1">
+    <row r="69" ht="120" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
           <t>A-02</t>
@@ -5732,17 +5720,17 @@
       </c>
       <c r="J69" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="L69" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>comprobar-afinador.js (Chromium, grabación real 12 cents baja → «La2 · −11 cents · Sube un poco»; hilo aparte; se apaga al salir) · Banco (node --test): flujo del permiso</t>
         </is>
       </c>
       <c r="M69" s="5" t="inlineStr">
@@ -5757,13 +5745,17 @@
       </c>
       <c r="O69" s="5" t="inlineStr">
         <is>
-          <t>Exige contexto seguro: funciona en https y en localhost. No funciona con file:// ni desde el móvil por WiFi contra el Live Server del ordenador (http://192.168… no es contexto seguro). En el móvil llega con la publicación (F7.2).</t>
+          <t>Exige contexto seguro: funciona en https y en localhost, no abriendo el archivo (file://). Hecho en la 0.4.0 (F4.3): Afinador › Micrófono › «Activar el micrófono»; se apaga al salir del Afinador o al ocultar la app, y el sonido se analiza solo en el dispositivo. En Chromium, con una grabación real de la 5ª cuerda 12 cents baja como micrófono, dice «La2 · −11 cents · ▲ Sube un poco» (herramientas/comprobar-afinador.js). En el iPhone se prueba en la web de pruebas, que es https. Falta tu comprobación con la guitarra (10 minutos).</t>
         </is>
       </c>
       <c r="P69" s="6" t="n"/>
-      <c r="Q69" s="5" t="inlineStr"/>
-    </row>
-    <row r="70" ht="63" customHeight="1">
+      <c r="Q69" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="120" customHeight="1">
       <c r="A70" s="4" t="inlineStr">
         <is>
           <t>A-02-CA</t>
@@ -5811,269 +5803,289 @@
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K70" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="L70" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>tests/tono.test.js: 12 grabaciones reales de −45 a +40 cents; peor error 1,86 cents frente a su medida y 1,01 trozo a trozo; aguja en su nota en ≤ 168 ms + 3 ms de cálculo</t>
         </is>
       </c>
       <c r="M70" s="5" t="inlineStr">
         <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="N70" s="5" t="inlineStr">
+        <is>
+          <t>Banco automático + auditor técnico</t>
+        </is>
+      </c>
+      <c r="O70" s="5" t="inlineStr">
+        <is>
+          <t>La precisión de detección debe ser mejor que el umbral de «afinado» de A-03. Hecho y validado en la 0.4.0 (F4.2, banco tests/tono.test.js): método YIN en un hilo aparte. Con las 12 grabaciones de cuerdas al aire de la app, desafinadas de −45 a +40 cents: peor error 1,86 cents frente a su frecuencia medida y 1,01 cents trozo a trozo; la aguja sale en su nota en 168 ms como mucho (más hasta 3 ms de cálculo). Nota: al pulsarla, una cuerda real suena unos cents alta y se asienta en unos 0,3 s; la aguja lo refleja, y eso es la cuerda, no el detector.</t>
+        </is>
+      </c>
+      <c r="P70" s="6" t="n"/>
+      <c r="Q70" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="78" customHeight="1">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>A-03</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Afinador</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Indicador de desviación en cents, con umbral de afinado en ±5 cents.</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Cliente · listado 14/09</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>F4.3</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr">
+        <is>
+          <t>La aguja indica la desviación en cents y marca «afinado» dentro de ±5 cents.</t>
+        </is>
+      </c>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="K71" s="5" t="inlineStr">
+        <is>
+          <t>0.4.0</t>
+        </is>
+      </c>
+      <c r="L71" s="5" t="inlineStr">
+        <is>
+          <t>Banco (node --test): «Sube un poco» a −12, «Afinada» a +3 · comprobar-afinador.js</t>
+        </is>
+      </c>
+      <c r="M71" s="5" t="inlineStr">
+        <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="N70" s="5" t="inlineStr">
+      <c r="N71" s="5" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="O71" s="5" t="inlineStr">
+        <is>
+          <t>Hecho en la 0.4.0: aguja de −50 a +50 cents con la franja verde de ±5, los cents en número y la orden «▲ Sube (un poco)», «▼ Baja (un poco)» o «✓ Afinada». Falta tu comprobación con la guitarra.</t>
+        </is>
+      </c>
+      <c r="P71" s="6" t="n"/>
+      <c r="Q71" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="93" customHeight="1">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>A-04</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Afinador</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Detección automática de cuerda por proximidad a la nota detectada.</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Cliente · listado 14/09</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>F4.3</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Con la cuerda a menos de un semitono de su nota, el afinador identifica la cuerda correcta.</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>0.4.0</t>
+        </is>
+      </c>
+      <c r="L72" s="5" t="inlineStr">
+        <is>
+          <t>Banco (node --test): Si3 −80 cents → 2ª; Fa4 → 1ª</t>
+        </is>
+      </c>
+      <c r="M72" s="5" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="N72" s="5" t="inlineStr">
         <is>
           <t>Banco automático + auditor técnico</t>
         </is>
       </c>
-      <c r="O70" s="5" t="inlineStr">
-        <is>
-          <t>La precisión de detección debe ser mejor que el umbral de «afinado» de A-03.</t>
-        </is>
-      </c>
-      <c r="P70" s="6" t="n"/>
-      <c r="Q70" s="5" t="inlineStr"/>
-    </row>
-    <row r="71" ht="33" customHeight="1">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>A-03</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
+      <c r="O72" s="5" t="inlineStr">
+        <is>
+          <t>Limitación asumida: con una cuerda muy desafinada puede elegir la equivocada. Hecho y validado en la 0.4.0 (banco): con «Auto», la cuerda de nota más cercana en la afinación activa; una Si3 80 cents baja sigue siendo la 2ª y un Fa4, la 1ª.</t>
+        </is>
+      </c>
+      <c r="P72" s="6" t="n"/>
+      <c r="Q72" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="93" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>A-05</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>Afinador</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>Indicador de desviación en cents, con umbral de afinado en ±5 cents.</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Selección manual de cuerda, que prevalece sobre A-04.</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr">
+      <c r="E73" s="5" t="inlineStr">
         <is>
           <t>Cliente · listado 14/09</t>
         </is>
       </c>
-      <c r="F71" s="5" t="inlineStr">
+      <c r="F73" s="5" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="G71" s="5" t="inlineStr">
+      <c r="G73" s="5" t="inlineStr">
         <is>
           <t>F4.3</t>
         </is>
       </c>
-      <c r="H71" s="5" t="inlineStr">
+      <c r="H73" s="5" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="I71" s="5" t="inlineStr">
-        <is>
-          <t>La aguja indica la desviación en cents y marca «afinado» dentro de ±5 cents.</t>
-        </is>
-      </c>
-      <c r="J71" s="5" t="inlineStr">
-        <is>
-          <t>No cumple</t>
-        </is>
-      </c>
-      <c r="K71" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L71" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M71" s="5" t="inlineStr">
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>Con una cuerda fijada a mano, el afinador la usa como referencia aunque esté muy desafinada.</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="K73" s="5" t="inlineStr">
+        <is>
+          <t>0.4.0</t>
+        </is>
+      </c>
+      <c r="L73" s="5" t="inlineStr">
+        <is>
+          <t>Banco (node --test): 6ª elegida con un La2 sonando → +500 cents, y sin confundir la octava</t>
+        </is>
+      </c>
+      <c r="M73" s="5" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="N71" s="5" t="inlineStr">
+      <c r="N73" s="5" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O71" s="5" t="inlineStr"/>
-      <c r="P71" s="6" t="n"/>
-      <c r="Q71" s="5" t="inlineStr"/>
-    </row>
-    <row r="72" ht="33" customHeight="1">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>A-04</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>Afinador</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>Detección automática de cuerda por proximidad a la nota detectada.</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>Cliente · listado 14/09</t>
-        </is>
-      </c>
-      <c r="F72" s="5" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="inlineStr">
-        <is>
-          <t>F4.3</t>
-        </is>
-      </c>
-      <c r="H72" s="5" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="I72" s="5" t="inlineStr">
-        <is>
-          <t>Con la cuerda a menos de un semitono de su nota, el afinador identifica la cuerda correcta.</t>
-        </is>
-      </c>
-      <c r="J72" s="5" t="inlineStr">
-        <is>
-          <t>No cumple</t>
-        </is>
-      </c>
-      <c r="K72" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L72" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M72" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="N72" s="5" t="inlineStr">
-        <is>
-          <t>Banco automático + auditor técnico</t>
-        </is>
-      </c>
-      <c r="O72" s="5" t="inlineStr">
-        <is>
-          <t>Limitación asumida: con una cuerda muy desafinada puede elegir la equivocada.</t>
-        </is>
-      </c>
-      <c r="P72" s="6" t="n"/>
-      <c r="Q72" s="5" t="inlineStr"/>
-    </row>
-    <row r="73" ht="33" customHeight="1">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>A-05</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>Afinador</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>Selección manual de cuerda, que prevalece sobre A-04.</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>Cliente · listado 14/09</t>
-        </is>
-      </c>
-      <c r="F73" s="5" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="G73" s="5" t="inlineStr">
-        <is>
-          <t>F4.3</t>
-        </is>
-      </c>
-      <c r="H73" s="5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="I73" s="5" t="inlineStr">
-        <is>
-          <t>Con una cuerda fijada a mano, el afinador la usa como referencia aunque esté muy desafinada.</t>
-        </is>
-      </c>
-      <c r="J73" s="5" t="inlineStr">
-        <is>
-          <t>No cumple</t>
-        </is>
-      </c>
-      <c r="K73" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L73" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M73" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="N73" s="5" t="inlineStr">
-        <is>
-          <t>Cliente</t>
-        </is>
-      </c>
       <c r="O73" s="5" t="inlineStr">
         <is>
-          <t>Resuelve la limitación anterior.</t>
+          <t>Resuelve la limitación anterior. Hecho en la 0.4.0: botones Auto · 6 … 1. Con una cuerda elegida, el afinador la usa aunque suene otra nota, y un salto de octava del detector no se confunde con «baja 12 semitonos». Falta tu comprobación con la guitarra.</t>
         </is>
       </c>
       <c r="P73" s="6" t="n"/>
-      <c r="Q73" s="5" t="inlineStr"/>
+      <c r="Q73" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="33" customHeight="1">
       <c r="A74" s="4" t="inlineStr">
@@ -7862,11 +7874,7 @@
         </is>
       </c>
       <c r="P96" s="6" t="n"/>
-      <c r="Q96" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="Q96" s="5" t="inlineStr"/>
     </row>
     <row r="97" ht="78" customHeight="1">
       <c r="A97" s="4" t="inlineStr">
@@ -8834,7 +8842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8874,34 +8882,34 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.3.3</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
+          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -8911,24 +8919,24 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.3.2</t>
+          <t>0.3.3</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
+          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -8938,24 +8946,24 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.3.1</t>
+          <t>0.3.2</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
+          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -8965,24 +8973,24 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -8992,24 +9000,24 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -9019,7 +9027,7 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
@@ -9029,14 +9037,14 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -9046,7 +9054,7 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
@@ -9056,24 +9064,24 @@
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
@@ -9083,14 +9091,14 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -9100,24 +9108,24 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -9127,24 +9135,24 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -9154,51 +9162,51 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -9208,7 +9216,7 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
@@ -9218,32 +9226,59 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
CP-4: correcciones de AR-08 y AT-07
- Detector: trozo según la tarjeta de sonido (96 kHz), guardas y límite
  si el hilo no contesta. Afinador: octava de la 6ª en Auto, «Afinada»
  sin parpadeo, lector de pantalla y foco, aviso si el sistema corta el
  micrófono. ?v= en css/ y js/ contra la caché. 51 de 51.
- Documentos: interfaz v1.6, automatización v1.2, V-09 con requisitos
  por paso, roadmap unificado, CREDITOS con los recortes del banco,
  capturas de V-06 restauradas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -1279,7 +1279,7 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): el autónomo es exactamente la app ensamblada (ensamblar.js) más su audio; la app en js/ se carga archivo a archivo</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>Desde la 0.2.1 hay dos formas reales: index.html para servir (Live Server y web) y dist/trasteando.html, generado a partir de él con herramientas/generar-autonomo.py. El banco comprueba que el autónomo está al día con index.html. Se vuelve más exigente al pasar a módulos (F4.1); F6.1 generará el archivo autónomo a partir de ellos. Desde la 0.4.0 (F4.1), la app vive en varios archivos (css/ y js/, uno por tema); herramientas/ensamblar.js los une para el archivo autónomo, y el banco comprueba que este es exactamente la app más su audio.</t>
+          <t>Desde la 0.2.1 hay dos formas reales: index.html para servir (Live Server y web) y dist/trasteando.html, generado a partir de él con herramientas/generar-autonomo.py. El banco comprueba que el autónomo está al día con index.html. Se vuelve más exigente al pasar a módulos (F4.1); F6.1 generará el archivo autónomo a partir de ellos. Desde la 0.4.0 (F4.1), la app vive en varios archivos (css/ y js/, uno por tema); herramientas/generar-autonomo.py sigue generando el archivo autónomo, y ahora usa herramientas/ensamblar.js para unirlos; el banco comprueba que el resultado es exactamente la app más su audio.</t>
         </is>
       </c>
       <c r="P12" s="6" t="n"/>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test) · CHANGELOG.md · F1.1 #12</t>
+          <t>Banco (node --test) · CHANGELOG.md · F1.1 #12 · etiquetas v0.1.5, v0.2.3 y v0.3.3 (21/10)</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>docs/compatibilidad.md v1.4 · Banco (node --test): sin matchMedia ni history</t>
+          <t>docs/compatibilidad.md v1.5 · Banco (node --test): sin matchMedia ni history</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
@@ -5921,7 +5921,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="93" customHeight="1">
+    <row r="72" ht="108" customHeight="1">
       <c r="A72" s="4" t="inlineStr">
         <is>
           <t>A-04</t>
@@ -5979,7 +5979,7 @@
       </c>
       <c r="L72" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): Si3 −80 cents → 2ª; Fa4 → 1ª</t>
+          <t>Banco (node --test): las 6 cuerdas a −90 y +90 cents, y la 6ª en Drop D</t>
         </is>
       </c>
       <c r="M72" s="5" t="inlineStr">
@@ -5994,7 +5994,7 @@
       </c>
       <c r="O72" s="5" t="inlineStr">
         <is>
-          <t>Limitación asumida: con una cuerda muy desafinada puede elegir la equivocada. Hecho y validado en la 0.4.0 (banco): con «Auto», la cuerda de nota más cercana en la afinación activa; una Si3 80 cents baja sigue siendo la 2ª y un Fa4, la 1ª.</t>
+          <t>Limitación asumida: con una cuerda muy desafinada puede elegir la equivocada. Hecho y validado en la 0.4.0 (banco): con «Auto», la cuerda de nota más cercana en la afinación activa. Cada una de las 6 cuerdas, 90 cents baja o alta, se identifica bien, y con Drop D también la 6ª (Re2).</t>
         </is>
       </c>
       <c r="P72" s="6" t="n"/>

</xml_diff>

<commit_message>
AR-09: documentos coherentes con la 0.4.1 y la 0.4.2
- J-01 e interfaz: la lectura y el pentagrama muestran la nota tocada.
- Matriz: criterios de J-01, J-08 y C-02; «Español / English» sin romper
  la tabla. J-11 sale de las decisiones abiertas (cerrada el 21/10).
- Roadmap: F4.4 lleva las pistas, F4.5 solo el idioma; F4 5/5 con
  pendientes; pendiente también ver la app en inglés. IT-02 al día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -1580,7 +1580,7 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>En Ajustes, Español | English cambia todos los textos de la app; la elección se guarda; la primera vez sigue al navegador.</t>
+          <t>En Ajustes, Español / English cambia todos los textos de la app; la elección se guarda; la primera vez sigue al navegador.</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10. Hecho en la 0.4.2: Ajustes › «Idioma · Language» (Español | English), cada idioma nombrado en su lengua. Todos los textos tienen clave y versión en las dos lenguas (el banco lo comprueba); los nombres de las notas siguen su propio ajuste (Do Re Mi o C D E), aunque quien estrena la app en inglés empieza con C D E. Restablecer no cambia el idioma. Falta que veas la app en inglés y digas si algo suena raro.</t>
+          <t>Tu petición del 21/10. Hecho en la 0.4.2: Ajustes › «Idioma · Language» (Español / English), cada idioma nombrado en su lengua. Todos los textos tienen clave y versión en las dos lenguas (el banco lo comprueba); los nombres de las notas siguen su propio ajuste (Do Re Mi o C D E), aunque quien estrena la app en inglés empieza con C D E. Restablecer no cambia el idioma. Falta que veas la app en inglés y digas si algo suena raro.</t>
         </is>
       </c>
       <c r="P16" s="6" t="n"/>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>En Adivinar nada suena hasta pulsar ▶ (resaltado); antes de ▶ el mástil suena pero no puntúa; después cada reto suena solo y ▶ lo repite. La lectura grande muestra la nota buscada, no la pulsada.</t>
+          <t>En Adivinar nada suena hasta pulsar ▶ (resaltado); antes de ▶ el mástil suena pero no puntúa; después cada reto suena solo y ▶ lo repite. La lectura grande y el pentagrama muestran la nota que tocas (0.4.1); la buscada, solo con la pista de nombre o al responder.</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="L49" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14 · Banco (node --test): ▶ y lectura de la nota buscada · Sesión 1: C07 y E04</t>
+          <t>F1.1 #14 · Banco (node --test): ▶, y lectura de la nota tocada con las pistas aparte · Sesión 1: C07 y E04</t>
         </is>
       </c>
       <c r="M49" s="5" t="inlineStr">
@@ -4181,7 +4181,7 @@
       </c>
       <c r="O49" s="5" t="inlineStr">
         <is>
-          <t>Con botón para repetir el sonido. Desde 0.1.1 los retos se limitan a los 12 primeros trastes por defecto, y desplazar el mástil ya no cuenta como pulsación. Desde la 0.3.3 (Sesión 1, E06), al entrar en Adivinar no suena nada hasta pulsar ▶, que aparece resaltado; antes de ▶ se puede tocar el mástil sin que puntúe. Después cada reto suena solo, y ▶ lo repite. Desde la 0.4.1 (tu comentario del 21/10), la lectura grande vuelve a ser la nota que tocas, y la respuesta de las pistas sale aparte, grande, en sus botones (J-06). Sesión 1 (20/10, informe V-08): lo esencial cumplió en C07 y E04; el cambio de la 0.3.3 lo pediste tú y se confirma en la Sesión 2.</t>
+          <t>Con botón para repetir el sonido. Desde 0.1.1 los retos se limitan a los 12 primeros trastes por defecto, y desplazar el mástil ya no cuenta como pulsación. Desde la 0.3.3 (Sesión 1, E06), al entrar en Adivinar no suena nada hasta pulsar ▶, que aparece resaltado; antes de ▶ se puede tocar el mástil sin que puntúe. Después cada reto suena solo, y ▶ lo repite. Desde la 0.4.1 (tu comentario del 21/10), la lectura grande y el pentagrama vuelven a mostrar la nota que tocas; la buscada solo se ve con la pista de nombre, que sale aparte y grande en su botón (J-06), o al responder. Sesión 1 (20/10, informe V-08): lo esencial cumplió en C07 y E04; el cambio de la 0.3.3 lo pediste tú y se confirma en la Sesión 2.</t>
         </is>
       </c>
       <c r="P49" s="6" t="n"/>
@@ -4696,7 +4696,7 @@
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>El récord persiste tras recargar y tras «Restablecer todos los ajustes»; solo «Borrar el récord de racha» lo pone a cero.</t>
+          <t>El récord de cada afinación persiste tras recargar y tras «Restablecer todos los ajustes»; solo «Borrar los récords de racha» los pone a cero.</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
@@ -4711,7 +4711,7 @@
       </c>
       <c r="L56" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): récord guardado y restablecer · F1.1 #13 · Sesión 1: A15</t>
+          <t>Banco (node --test): récords por afinación guardados y restablecer · F1.1 #13 · Sesión 1: A15</t>
         </is>
       </c>
       <c r="M56" s="5" t="inlineStr">
@@ -7433,7 +7433,7 @@
       </c>
       <c r="I91" s="5" t="inlineStr">
         <is>
-          <t>El panel contiene todos los ajustes listados y la versión de la app.</t>
+          <t>El panel contiene todos los ajustes listados, el idioma (0.4.2) y la versión de la app.</t>
         </is>
       </c>
       <c r="J91" s="5" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="L91" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #12</t>
+          <t>F1.1 #12 · Banco (node --test): grupo Idioma</t>
         </is>
       </c>
       <c r="M91" s="5" t="inlineStr">
@@ -8973,7 +8973,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; J-06 con las pistas grandes.</t>
+          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F5 docs y Adivinar: al fallar, ver la respuesta o seguir intentando (J-13)
- requisitos.md v1.18 (E-01 a E-06, P-03), roadmap v3.16, interfaz v1.8,
  CHANGELOG 0.5.0 e informe IT-03.
- Ajustes › Adivinar › «Al fallar»: Ver respuesta | Reintentar (tu
  petición del 21/10). Reintentando, el reto sigue, la racha se rompe y
  «Ver la respuesta» se rinde. 65 de 65. Versión 0.5.1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.15. Base: requisitos.md v1.17 · app 0.4.2 · roadmap 3.15 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.16. Base: requisitos.md v1.18 · app 0.5.0 · roadmap 3.16 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.17</t>
+          <t>Cambio en v1.18</t>
         </is>
       </c>
     </row>
@@ -1614,11 +1614,7 @@
         </is>
       </c>
       <c r="P16" s="6" t="n"/>
-      <c r="Q16" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="Q16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -2165,7 +2161,7 @@
       <c r="P23" s="6" t="n"/>
       <c r="Q23" s="5" t="inlineStr"/>
     </row>
-    <row r="24" ht="48" customHeight="1">
+    <row r="24" ht="78" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>N-04</t>
@@ -2238,11 +2234,15 @@
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
-          <t>Verificar de nuevo al añadir Escalas (F5). Validado en la Sesión 1 (20/10, informe V-08): A06.</t>
+          <t>Verificar de nuevo al añadir Escalas (F5). Validado en la Sesión 1 (20/10, informe V-08): A06. Desde la 0.5.0, también Escalas: tónicas, nombres escritos e intervalos siguen la nomenclatura.</t>
         </is>
       </c>
       <c r="P24" s="6" t="n"/>
-      <c r="Q24" s="5" t="inlineStr"/>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="33" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -3721,7 +3721,7 @@
       <c r="P43" s="6" t="n"/>
       <c r="Q43" s="5" t="inlineStr"/>
     </row>
-    <row r="44" ht="33" customHeight="1">
+    <row r="44" ht="63" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
           <t>P-03</t>
@@ -3769,17 +3769,17 @@
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>Cumple parcialmente</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): la escala escrita en el pentagrama (8 notas en Mostrar; las encontradas en Práctica)</t>
         </is>
       </c>
       <c r="M44" s="5" t="inlineStr">
@@ -3794,11 +3794,15 @@
       </c>
       <c r="O44" s="5" t="inlineStr">
         <is>
-          <t>Libre y Adivinar sí. Escalas, en F5.</t>
+          <t>Libre y Adivinar sí. Escalas, en F5. Desde la 0.5.0, en Escalas el pentagrama escribe la escala entera, con sus alteraciones (♯ y ♭ según la tonalidad).</t>
         </is>
       </c>
       <c r="P44" s="6" t="n"/>
-      <c r="Q44" s="5" t="inlineStr"/>
+      <c r="Q44" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="33" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
@@ -4185,11 +4189,7 @@
         </is>
       </c>
       <c r="P49" s="6" t="n"/>
-      <c r="Q49" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q49" s="5" t="inlineStr"/>
     </row>
     <row r="50" ht="33" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
@@ -4572,11 +4572,7 @@
         </is>
       </c>
       <c r="P54" s="6" t="n"/>
-      <c r="Q54" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q54" s="5" t="inlineStr"/>
     </row>
     <row r="55" ht="33" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
@@ -4730,11 +4726,7 @@
         </is>
       </c>
       <c r="P56" s="6" t="n"/>
-      <c r="Q56" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q56" s="5" t="inlineStr"/>
     </row>
     <row r="57" ht="48" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
@@ -4971,11 +4963,7 @@
         </is>
       </c>
       <c r="P59" s="6" t="n"/>
-      <c r="Q59" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q59" s="5" t="inlineStr"/>
     </row>
     <row r="60" ht="63" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
@@ -5056,7 +5044,7 @@
       <c r="P60" s="6" t="n"/>
       <c r="Q60" s="5" t="inlineStr"/>
     </row>
-    <row r="61" ht="33" customHeight="1">
+    <row r="61" ht="93" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
           <t>E-01</t>
@@ -5099,22 +5087,22 @@
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>Se puede elegir tónica y tipo de escala entre el catálogo aprobado.</t>
+          <t>Se puede elegir tónica y tipo de escala entre el catálogo aprobado (mayor, menor natural, pentatónicas mayor y menor; 21/10).</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="L61" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): selectores de tónica y tipo</t>
         </is>
       </c>
       <c r="M61" s="5" t="inlineStr">
@@ -5129,13 +5117,17 @@
       </c>
       <c r="O61" s="5" t="inlineStr">
         <is>
-          <t>Catálogo inicial por decidir.</t>
+          <t>Catálogo decidido el 21/10 (tu elección): mayor, menor natural, pentatónica mayor y pentatónica menor, en las 12 tónicas. Hecho en la 0.5.0: Escalas › tónica y tipo; la tónica se escribe según el tipo (Re♭ mayor, Do♯ menor). Falta que lo veas.</t>
         </is>
       </c>
       <c r="P61" s="6" t="n"/>
-      <c r="Q61" s="5" t="inlineStr"/>
-    </row>
-    <row r="62" ht="48" customHeight="1">
+      <c r="Q61" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="120" customHeight="1">
       <c r="A62" s="4" t="inlineStr">
         <is>
           <t>E-02</t>
@@ -5183,22 +5175,22 @@
       </c>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>tests/escalas.test.js: las 48 escalas frente al círculo de quintas; casillas por clase de altura</t>
         </is>
       </c>
       <c r="M62" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N62" s="5" t="inlineStr">
@@ -5208,11 +5200,15 @@
       </c>
       <c r="O62" s="5" t="inlineStr">
         <is>
-          <t>Alcance acotado. Las demás afinaciones pasan a E-02b.</t>
+          <t>Alcance acotado. Las demás afinaciones pasan a E-02b. Hecho y validado en la 0.5.0 (banco tests/escalas.test.js): las 48 escalas se escriben como en el círculo de quintas, con siete letras distintas en las mayores y menores y sin mezclar ♯ y ♭. Las casillas salen de la clase de altura de cada nota, así que también funcionan en las demás afinaciones; lo que sigue fuera (E-02b) son las digitaciones.</t>
         </is>
       </c>
       <c r="P62" s="6" t="n"/>
-      <c r="Q62" s="5" t="inlineStr"/>
+      <c r="Q62" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="48" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -5293,7 +5289,7 @@
       <c r="P63" s="6" t="n"/>
       <c r="Q63" s="5" t="inlineStr"/>
     </row>
-    <row r="64" ht="33" customHeight="1">
+    <row r="64" ht="63" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
         <is>
           <t>E-03</t>
@@ -5336,22 +5332,22 @@
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Mostrar ilumina únicamente las notas de la escala.</t>
+          <t>Mostrar ilumina únicamente las notas de la escala, con su nombre escrito y la tónica con anillo.</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="L64" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): casillas de Do mayor y de Fa mayor (Si♭)</t>
         </is>
       </c>
       <c r="M64" s="5" t="inlineStr">
@@ -5364,11 +5360,19 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O64" s="5" t="inlineStr"/>
+      <c r="O64" s="5" t="inlineStr">
+        <is>
+          <t>Hecho en la 0.5.0: el mástil enseña solo las notas de la escala, con su nombre escrito (Si♭ en Fa mayor, no La#) y la tónica con anillo. Falta que lo veas.</t>
+        </is>
+      </c>
       <c r="P64" s="6" t="n"/>
-      <c r="Q64" s="5" t="inlineStr"/>
-    </row>
-    <row r="65" ht="48" customHeight="1">
+      <c r="Q64" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="93" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
           <t>E-04</t>
@@ -5411,22 +5415,22 @@
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>Cada nota iluminada muestra su nombre y el intervalo T o ST respecto al grado anterior.</t>
+          <t>Las notas de la escala muestran su nombre y la línea de notas indica el intervalo T, ST o T½ respecto al grado anterior.</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="L65" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): «Do T Re T Mi ST Fa…» y la pentatónica menor</t>
         </is>
       </c>
       <c r="M65" s="5" t="inlineStr">
@@ -5441,13 +5445,17 @@
       </c>
       <c r="O65" s="5" t="inlineStr">
         <is>
-          <t>Etiquetas tipo T — T — ST — T — T — T — ST.</t>
+          <t>Etiquetas tipo T — T — ST — T — T — T — ST. Hecho en la 0.5.0: encima del paso a paso, «Do T Re T Mi ST Fa…»; en las pentatónicas aparece también T½ (tono y medio). Los intervalos van en esa línea y no en cada casilla, donde no caben. Falta que lo veas.</t>
         </is>
       </c>
       <c r="P65" s="6" t="n"/>
-      <c r="Q65" s="5" t="inlineStr"/>
-    </row>
-    <row r="66" ht="48" customHeight="1">
+      <c r="Q65" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="108" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
         <is>
           <t>E-05</t>
@@ -5495,22 +5503,22 @@
       </c>
       <c r="J66" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K66" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="L66" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): conteo de notas distintas, fallo, revelado y reinicio</t>
         </is>
       </c>
       <c r="M66" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N66" s="5" t="inlineStr">
@@ -5520,11 +5528,15 @@
       </c>
       <c r="O66" s="5" t="inlineStr">
         <is>
-          <t>Alcance acotado: no valida orden ni digitación.</t>
+          <t>Alcance acotado: no valida orden ni digitación. Hecho y validado en la 0.5.0 (banco): cada nota distinta cuenta una vez («3 de 7»); una ajena se marca en rojo y se enseñan un momento las buenas; el pentagrama solo escribe las que ya has encontrado. Falta probarlo con la guitarra (Sesión 2).</t>
         </is>
       </c>
       <c r="P66" s="6" t="n"/>
-      <c r="Q66" s="5" t="inlineStr"/>
+      <c r="Q66" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="33" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
@@ -5605,7 +5617,7 @@
       <c r="P67" s="6" t="n"/>
       <c r="Q67" s="5" t="inlineStr"/>
     </row>
-    <row r="68" ht="33" customHeight="1">
+    <row r="68" ht="78" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
           <t>E-06</t>
@@ -5653,17 +5665,17 @@
       </c>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K68" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="L68" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): pasos que suenan y se resaltan, de la tónica grave a su octava</t>
         </is>
       </c>
       <c r="M68" s="5" t="inlineStr">
@@ -5676,9 +5688,17 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O68" s="5" t="inlineStr"/>
+      <c r="O68" s="5" t="inlineStr">
+        <is>
+          <t>Hecho en la 0.5.0: ◀ ▶ recorre la escala desde la tónica más grave del mástil hasta su octava; cada paso suena, se resalta en el mástil y en el pentagrama, y se explica («Mi, un tono sobre Re»). Falta que lo veas.</t>
+        </is>
+      </c>
       <c r="P68" s="6" t="n"/>
-      <c r="Q68" s="5" t="inlineStr"/>
+      <c r="Q68" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="33" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
@@ -7467,11 +7487,7 @@
         </is>
       </c>
       <c r="P91" s="6" t="n"/>
-      <c r="Q91" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q91" s="5" t="inlineStr"/>
     </row>
     <row r="92" ht="78" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
@@ -8913,7 +8929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8953,7 +8969,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -8963,24 +8979,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.4.2</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
+          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -8990,51 +9006,51 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.4.0</t>
+          <t>0.4.2</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
+          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.3.3</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
+          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -9044,24 +9060,24 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.3.2</t>
+          <t>0.3.3</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
+          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -9071,24 +9087,24 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.3.1</t>
+          <t>0.3.2</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
+          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -9098,24 +9114,24 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -9125,24 +9141,24 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -9152,7 +9168,7 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
@@ -9162,14 +9178,14 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -9179,7 +9195,7 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
@@ -9189,24 +9205,24 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
@@ -9216,14 +9232,14 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -9233,24 +9249,24 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -9260,24 +9276,24 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -9287,51 +9303,51 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -9341,7 +9357,7 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
@@ -9351,32 +9367,59 @@
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
Documentar el metrónomo como área propia y cerrar AR-10 y AT-09 (requisitos v1.20, MT-05, J-13)
- requisitos v1.20: J-13 con reintentar por defecto; MT-05, el metrónomo con
  su pestaña; G-02, C-04, C-02, J-06, E-05, N-06, MT-01, AC-01, AC-02 y AC-05
  al día; objetivo O-05; decisión abierta: las seis pestañas.
- matriz v1.18, roadmap v3.18, interfaz v1.10 (§7b, propuesta pendiente) e
  IT-03 al día.
- Informes AR-10 y AT-09.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.17. Base: requisitos.md v1.19 · app 0.5.2 · roadmap 3.17 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.18. Base: requisitos.md v1.20 · app 0.5.3 · roadmap 3.18 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>El nombre «Trasteando» aparece en la pantalla de entrada, en la pestaña del navegador y en el manifiesto.</t>
+          <t>El nombre «Trasteando» aparece en la pantalla de entrada, en la pestaña del navegador y en el manifiesto; en horizontal, arriba del panel.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14 · Sesión 1: A01</t>
+          <t>F1.1 #14 · 0.5.2: comprobar-disposicion, título visible en horizontal · Sesión 1: A01</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
@@ -745,90 +745,90 @@
         </is>
       </c>
       <c r="P5" s="6" t="n"/>
-      <c r="Q5" s="5" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="63" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>G-02</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Requisitos generales y de producto</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>La app se organiza en áreas accesibles desde una navegación principal: Libre, Adivinar, Afinador y Escalas. Cada área nueva (Metrónomo y Acordes, en F5) se suma a esa navegación.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Cliente · listado 14/09</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>F1.1</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>La barra inferior muestra Libre, Adivinar, Afinador y Escalas; cada destino activo abre su vista y cada área nueva (Metrónomo, Acordes) suma su destino.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>F1.1 #1 y #14 · Sesión 1 A12 · Sesión 1: A12</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>Escalas, habilitada desde la 0.5.0. Metrónomo (F5.6) y Acordes (F5.7) serán áreas propias (tu decisión del 21/10). Validado en la Sesión 1 (20/10, informe V-08): A12.</t>
+        </is>
+      </c>
+      <c r="P6" s="6" t="n"/>
+      <c r="Q6" s="5" t="inlineStr">
         <is>
           <t>Modificado</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>G-02</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Requisitos generales y de producto</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>La app se organiza en áreas accesibles desde una navegación principal: Libre, Adivinar, Afinador y Escalas.</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Cliente · listado 14/09</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>F1.1</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>La barra inferior muestra Libre, Adivinar, Afinador y Escalas; cada destino activo abre su vista y Escalas aparece deshabilitada.</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>Cumple</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>F1.1 #1 y #14 · Sesión 1: A12</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>Verificado</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>Cliente</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Escalas visible pero deshabilitada hasta F5. Validado en la Sesión 1 (20/10, informe V-08): A12.</t>
-        </is>
-      </c>
-      <c r="P6" s="6" t="n"/>
-      <c r="Q6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="108" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -2323,7 +2323,7 @@
       <c r="P25" s="6" t="n"/>
       <c r="Q25" s="5" t="inlineStr"/>
     </row>
-    <row r="26" ht="78" customHeight="1">
+    <row r="26" ht="120" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>N-06</t>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Elegido ♭ para una tecla negra, todas sus notas se escriben así en mástil, lectura y pentagrama; las demás no cambian; en una escala manda la escala.</t>
+          <t>Elegido ♭ para una tecla negra, todas sus notas se escriben así en mástil, lectura, pentagrama y Afinador; las demás no cambian; en una escala manda la escala, también en el lector grande y el de pantalla.</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): Sol♭ en todo el mástil, Fa♯ en Sol mayor, botones según la nomenclatura</t>
+          <t>Banco (node --test): Sol♭ en todo el mástil, Fa♯ en Sol mayor, botones según la nomenclatura; Si♭ en Fa mayor (AT-09)</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
@@ -2396,13 +2396,13 @@
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>Tu comentario del 21/10. Hecho en la 0.5.2: Ajustes › Notación › Notas alteradas (Do♯ o Re♭, Re♯ o Mi♭, Fa♯ o Sol♭, Sol♯ o La♭, La♯ o Si♭); se usan los signos ♯ y ♭, también en el pentagrama. Validado por el banco.</t>
+          <t>Tu comentario del 21/10. Hecho en la 0.5.2: Ajustes › Notación › Notas alteradas (Do♯ o Re♭, Re♯ o Mi♭, Fa♯ o Sol♭, Sol♯ o La♭, La♯ o Si♭); se usan los signos ♯ y ♭, también en el pentagrama. Validado por el banco. Desde la 0.5.3, también el pentagrama del Afinador; y en Escalas, el lector grande y el lector de pantalla escriben como la escala (AT-09).</t>
         </is>
       </c>
       <c r="P26" s="6" t="n"/>
       <c r="Q26" s="5" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Modificado</t>
         </is>
       </c>
     </row>
@@ -3704,7 +3704,7 @@
       </c>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>Análisis 15/09: ninguna nota fuera en todo el rango · F1.1 #3 y #4 · Sesión 1: A05</t>
+          <t>Análisis 15/09: ninguna nota fuera en todo el rango · F1.1 #3 y #4 · 0.5.2: pentagrama de una nota de 152 px de alto en el iPhone en horizontal (comprobar-disposicion) · Sesión 1: A05</t>
         </is>
       </c>
       <c r="M43" s="5" t="inlineStr">
@@ -3723,11 +3723,7 @@
         </is>
       </c>
       <c r="P43" s="6" t="n"/>
-      <c r="Q43" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q43" s="5" t="inlineStr"/>
     </row>
     <row r="44" ht="33" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
@@ -4651,11 +4647,15 @@
       </c>
       <c r="O55" s="5" t="inlineStr">
         <is>
-          <t>Con las dos pistas activas equivale a «busca esta nota en esta cuerda»; sin ninguna, a «adivina de oído». Validado en la Sesión 1 (20/10, informe V-08): E04. Desde la 0.4.1 (tu comentario del 21/10): encendida, cada pista enseña su respuesta dentro de su botón, en grande y con borde discontinuo de «pista» («NOTA Sol#3», «CUERDAS 3ª 4ª»), para no confundirla con la nota que tocas. Se ve también antes de pulsar ▶ (antes no salía). Lo esencial ya estaba validado; el aspecto nuevo lo verás en la próxima prueba.</t>
+          <t>Con las dos pistas activas equivale a «busca esta nota en esta cuerda»; sin ninguna, a «adivina de oído». Validado en la Sesión 1 (20/10, informe V-08): E04. Desde la 0.4.1 (tu comentario del 21/10): encendida, cada pista enseña su respuesta dentro de su botón, en grande y con borde discontinuo de «pista» («NOTA Sol♯3», «CUERDAS 3ª 4ª»), para no confundirla con la nota que tocas. Se ve también antes de pulsar ▶ (antes no salía). Lo esencial ya estaba validado; el aspecto nuevo lo verás en la próxima prueba.</t>
         </is>
       </c>
       <c r="P55" s="6" t="n"/>
-      <c r="Q55" s="5" t="inlineStr"/>
+      <c r="Q55" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="33" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
@@ -5127,7 +5127,7 @@
       <c r="P61" s="6" t="n"/>
       <c r="Q61" s="5" t="inlineStr"/>
     </row>
-    <row r="62" ht="78" customHeight="1">
+    <row r="62" ht="93" customHeight="1">
       <c r="A62" s="4" t="inlineStr">
         <is>
           <t>J-13</t>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Al fallar en Adivinar, eliges en Ajustes entre ver la respuesta (como siempre) o seguir intentándolo; si sigues, puedes rendirte con «Ver la respuesta», y acertar tras fallar pasa al reto siguiente sin sumar a la racha.</t>
+          <t>Al fallar en Adivinar, por defecto sigues intentándolo hasta que aciertes o pidas «Ver la respuesta»; en Ajustes puedes elegir que la respuesta se enseñe nada más fallar. Acertar tras fallar pasa al reto siguiente sin sumar a la racha.</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -5150,7 +5150,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>Con «Reintentar», un fallo rompe la racha pero el reto sigue; «Ver la respuesta» la enseña y suena; acertar tras fallar no suma. Con «Ver respuesta», como J-10.</t>
+          <t>Por defecto, «Reintentar»: un fallo rompe la racha pero el reto sigue; «Ver la respuesta» la enseña y suena; acertar tras fallar no suma. Con «Ver respuesta», como J-10.</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): modo reintentar y ajuste guardado</t>
+          <t>Banco (node --test): modo reintentar, ajuste guardado y valor por defecto; dos fallos seguidos no dejan casillas rojas (AT-09)</t>
         </is>
       </c>
       <c r="M62" s="5" t="inlineStr">
@@ -5200,13 +5200,13 @@
       </c>
       <c r="O62" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10. Hecho en la 0.5.1: Ajustes › Adivinar › «Al fallar»: Ver respuesta | Reintentar. El fallo rompe la racha en los dos casos (J-10). Validado por el banco.</t>
+          <t>Tu petición del 21/10. Hecho en la 0.5.1: Ajustes › Adivinar › «Al fallar»: Ver respuesta | Reintentar. El fallo rompe la racha en los dos casos (J-10). Validado por el banco. Desde la 0.5.3, seguir intentando es lo de fábrica (tu decisión del 21/10).</t>
         </is>
       </c>
       <c r="P62" s="6" t="n"/>
       <c r="Q62" s="5" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Modificado</t>
         </is>
       </c>
     </row>
@@ -5605,7 +5605,7 @@
       <c r="P67" s="6" t="n"/>
       <c r="Q67" s="5" t="inlineStr"/>
     </row>
-    <row r="68" ht="108" customHeight="1">
+    <row r="68" ht="120" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
           <t>E-05</t>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="L68" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): conteo de notas distintas, fallo, revelado y reinicio</t>
+          <t>Banco (node --test): conteo de notas distintas, fallo, revelado y reinicio; reinicio al cambiar de afinación (AT-09)</t>
         </is>
       </c>
       <c r="M68" s="5" t="inlineStr">
@@ -5678,11 +5678,15 @@
       </c>
       <c r="O68" s="5" t="inlineStr">
         <is>
-          <t>Alcance acotado: no valida orden ni digitación. Hecho y validado en la 0.5.0 (banco): cada nota distinta cuenta una vez («3 de 7»); una ajena se marca en rojo y se enseñan un momento las buenas; el pentagrama solo escribe las que ya has encontrado. Falta probarlo con la guitarra (Sesión 2).</t>
+          <t>Alcance acotado: no valida orden ni digitación. Hecho y validado en la 0.5.0 (banco): cada nota distinta cuenta una vez («3 de 7»); una ajena se marca en rojo y se enseñan un momento las buenas; el pentagrama solo escribe las que ya has encontrado. Falta probarlo con la guitarra (Sesión 2). Desde la 0.5.3, el progreso empieza de nuevo al cambiar de afinación: cada casilla suena ya a otra nota (AT-09).</t>
         </is>
       </c>
       <c r="P68" s="6" t="n"/>
-      <c r="Q68" s="5" t="inlineStr"/>
+      <c r="Q68" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="33" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
@@ -6801,7 +6805,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
@@ -6821,7 +6825,7 @@
       </c>
       <c r="I83" s="5" t="inlineStr">
         <is>
-          <t>Tempo de 30 a 250 con botones y marcando el tempo; arranca y para con un toque.</t>
+          <t>Tempo de 30 a 250 con botones y marcando el tempo; arranca y para con un toque; se usa en vertical y en horizontal sin aviso de girar.</t>
         </is>
       </c>
       <c r="J83" s="5" t="inlineStr">
@@ -6851,13 +6855,13 @@
       </c>
       <c r="O83" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10.</t>
+          <t>Tu petición del 21/10. Se usa igual en vertical y en horizontal: como el Afinador, no pide girar el móvil.</t>
         </is>
       </c>
       <c r="P83" s="6" t="n"/>
       <c r="Q83" s="5" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Modificado</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6888,7 @@
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F84" s="5" t="inlineStr">
@@ -6938,11 +6942,7 @@
         </is>
       </c>
       <c r="P84" s="6" t="n"/>
-      <c r="Q84" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="Q84" s="5" t="inlineStr"/>
     </row>
     <row r="85" ht="48" customHeight="1">
       <c r="A85" s="4" t="inlineStr">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F85" s="5" t="inlineStr">
@@ -7021,11 +7021,7 @@
         </is>
       </c>
       <c r="P85" s="6" t="n"/>
-      <c r="Q85" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="Q85" s="5" t="inlineStr"/>
     </row>
     <row r="86" ht="63" customHeight="1">
       <c r="A86" s="4" t="inlineStr">
@@ -7050,7 +7046,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr">
@@ -7104,13 +7100,9 @@
         </is>
       </c>
       <c r="P86" s="6" t="n"/>
-      <c r="Q86" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="63" customHeight="1">
+      <c r="Q86" s="5" t="inlineStr"/>
+    </row>
+    <row r="87" ht="93" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
         <is>
           <t>MT-05</t>
@@ -7123,7 +7115,7 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>El metrónomo se usa a la vez que Libre, Adivinar o Escalas, y recuerda el último tempo, compás, acentos y subdivisión.</t>
+          <t>El metrónomo es un área propia, con su pestaña en la navegación principal. Sigue sonando al pasar a Libre, Adivinar, Escalas o Acordes hasta que lo pares, y su pestaña late con el pulso mientras suena. Recuerda el último tempo, compás, acentos y subdivisión.</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
@@ -7133,7 +7125,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
@@ -7153,7 +7145,7 @@
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>Con el metrónomo en marcha se puede tocar en Libre, Adivinar y Escalas; tempo, compás, acentos y subdivisión se recuerdan.</t>
+          <t>El metrónomo tiene su pestaña; en marcha, sigue sonando en Libre, Adivinar, Escalas y Acordes y su pestaña late con el pulso; al escuchar con el micrófono se para y lo dice; tempo, compás, acentos y subdivisión se recuerdan.</t>
         </is>
       </c>
       <c r="J87" s="5" t="inlineStr">
@@ -7183,17 +7175,17 @@
       </c>
       <c r="O87" s="5" t="inlineStr">
         <is>
-          <t>Propuesta de interfaz: un chip en el acceso rápido («♩ 80») que abre un panel; mientras suena, el chip late con el pulso. Así no hace falta una pestaña más.</t>
+          <t>Tu decisión del 21/10: función propia, no un chip del acceso rápido. Al escuchar con el micrófono en el Afinador, el metrónomo se para y lo dice: su clic confundiría al detector. Distribución de la pestaña: interfaz.md §7b, propuesta pendiente de tu visto bueno.</t>
         </is>
       </c>
       <c r="P87" s="6" t="n"/>
       <c r="Q87" s="5" t="inlineStr">
         <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="48" customHeight="1">
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="63" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
         <is>
           <t>AC-01</t>
@@ -7216,7 +7208,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
@@ -7266,17 +7258,17 @@
       </c>
       <c r="O88" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10; el catálogo lo propone el agente: unos 30 acordes, los que salen en la mayoría de canciones.</t>
+          <t>Tu petición del 21/10; el catálogo lo propone el agente: unos 30 acordes, los que salen en la mayoría de canciones. Es un área propia, con su pestaña (interfaz.md §7b).</t>
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
       <c r="Q88" s="5" t="inlineStr">
         <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="93" customHeight="1">
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="120" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
         <is>
           <t>AC-02</t>
@@ -7299,7 +7291,7 @@
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
@@ -7319,7 +7311,7 @@
       </c>
       <c r="I89" s="5" t="inlineStr">
         <is>
-          <t>Cada dedo tiene su número y su color, iguales en todos los acordes; cuerdas al aire y apagadas marcadas; cejilla marcada.</t>
+          <t>Cada dedo tiene su número y su color, iguales en todos los acordes y distintos de la paleta de notas; círculo ≥ 3:1 contra el mástil y número ≥ 4,5:1 contra el círculo; cuerdas al aire y apagadas marcadas; cejilla marcada.</t>
         </is>
       </c>
       <c r="J89" s="5" t="inlineStr">
@@ -7349,13 +7341,13 @@
       </c>
       <c r="O89" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10: número y color a la vez, con el color constante entre acordes.</t>
+          <t>Tu petición del 21/10: número y color a la vez, con el color constante entre acordes. Los cuatro colores de dedo son distintos de la paleta de notas (que va por nota) y distintos entre sí también para daltónicos; cada círculo contrasta al menos 3:1 con el mástil y su número al menos 4,5:1 con el círculo (G-05).</t>
         </is>
       </c>
       <c r="P89" s="6" t="n"/>
       <c r="Q89" s="5" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Modificado</t>
         </is>
       </c>
     </row>
@@ -7382,7 +7374,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
@@ -7432,11 +7424,7 @@
       </c>
       <c r="O90" s="5" t="inlineStr"/>
       <c r="P90" s="6" t="n"/>
-      <c r="Q90" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="Q90" s="5" t="inlineStr"/>
     </row>
     <row r="91" ht="33" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
@@ -7461,7 +7449,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
@@ -7511,13 +7499,9 @@
       </c>
       <c r="O91" s="5" t="inlineStr"/>
       <c r="P91" s="6" t="n"/>
-      <c r="Q91" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="33" customHeight="1">
+      <c r="Q91" s="5" t="inlineStr"/>
+    </row>
+    <row r="92" ht="93" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
         <is>
           <t>AC-05</t>
@@ -7540,7 +7524,7 @@
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
@@ -7560,7 +7544,7 @@
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Las digitaciones indican que son para la afinación estándar.</t>
+          <t>Las digitaciones indican que son para la afinación estándar; con otra afinación, Acordes lo avisa y ofrece pasar a la estándar; el selector no ofrece combinaciones sin digitación.</t>
         </is>
       </c>
       <c r="J92" s="5" t="inlineStr">
@@ -7590,13 +7574,13 @@
       </c>
       <c r="O92" s="5" t="inlineStr">
         <is>
-          <t>Las digitaciones dependen de la afinación; las demás, para después.</t>
+          <t>Las digitaciones dependen de la afinación; las demás, para después. Con otra afinación activa, Acordes lo avisa y ofrece pasar a la estándar. El selector de tipo solo ofrece los tipos que el catálogo tiene para esa tónica: no hay combinaciones vacías.</t>
         </is>
       </c>
       <c r="P92" s="6" t="n"/>
       <c r="Q92" s="5" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Modificado</t>
         </is>
       </c>
     </row>
@@ -8374,7 +8358,7 @@
       <c r="P102" s="6" t="n"/>
       <c r="Q102" s="5" t="inlineStr"/>
     </row>
-    <row r="103" ht="108" customHeight="1">
+    <row r="103" ht="120" customHeight="1">
       <c r="A103" s="4" t="inlineStr">
         <is>
           <t>C-02</t>
@@ -8447,11 +8431,15 @@
       </c>
       <c r="O103" s="5" t="inlineStr">
         <is>
-          <t>Ampliado en 0.1.2 con la numeración en tres modos y la versión (G-10). En F6.4 se añade el grupo «Acerca de», con los créditos (G-06) y la privacidad (G-11) (interfaz.md v1.0, aprobada el 20/10). Desde la 0.4.2, Ajustes empieza con el grupo «Idioma · Language» (G-12).</t>
+          <t>Ampliado en 0.1.2 con la numeración en tres modos y la versión (G-10). En F6.4 se añade el grupo «Acerca de», con los créditos (G-06) y la privacidad (G-11) (interfaz.md v1.0, aprobada el 20/10). Desde la 0.4.2, Ajustes empieza con el grupo «Idioma · Language» (G-12). Tiene también «Al fallar» en Adivinar (J-13, 0.5.1) y «Notas alteradas», ♯ o ♭ por tecla negra (N-06, 0.5.2).</t>
         </is>
       </c>
       <c r="P103" s="6" t="n"/>
-      <c r="Q103" s="5" t="inlineStr"/>
+      <c r="Q103" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="78" customHeight="1">
       <c r="A104" s="4" t="inlineStr">
@@ -8532,7 +8520,7 @@
       <c r="P104" s="6" t="n"/>
       <c r="Q104" s="5" t="inlineStr"/>
     </row>
-    <row r="105" ht="93" customHeight="1">
+    <row r="105" ht="120" customHeight="1">
       <c r="A105" s="4" t="inlineStr">
         <is>
           <t>C-04</t>
@@ -8605,11 +8593,15 @@
       </c>
       <c r="O105" s="5" t="inlineStr">
         <is>
-          <t>Barra inferior con cuatro destinos en vertical, raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05). Validado en la Sesión 1 (20/10, informe V-08): A19.</t>
+          <t>Barra inferior con un destino por área en vertical (cuatro hoy; seis con Metrónomo y Acordes, con pestañas de al menos 44 px), raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05). Validado en la Sesión 1 (20/10, informe V-08): A19.</t>
         </is>
       </c>
       <c r="P105" s="6" t="n"/>
-      <c r="Q105" s="5" t="inlineStr"/>
+      <c r="Q105" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="48" customHeight="1">
       <c r="A106" s="4" t="inlineStr">
@@ -9893,7 +9885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9933,7 +9925,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -9943,24 +9935,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.5.2</t>
+          <t>0.5.3</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
+          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -9970,24 +9962,24 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.5.0</t>
+          <t>0.5.2</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
+          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -9997,24 +9989,24 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.4.2</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
+          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -10024,51 +10016,51 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.4.0</t>
+          <t>0.4.2</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
+          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.3.3</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
+          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -10078,24 +10070,24 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.3.2</t>
+          <t>0.3.3</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
+          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -10105,24 +10097,24 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.3.1</t>
+          <t>0.3.2</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
+          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -10132,24 +10124,24 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -10159,24 +10151,24 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -10186,7 +10178,7 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
@@ -10196,14 +10188,14 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -10213,7 +10205,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -10223,24 +10215,24 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -10250,14 +10242,14 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -10267,24 +10259,24 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -10294,24 +10286,24 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -10321,51 +10313,51 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -10375,7 +10367,7 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
@@ -10385,32 +10377,59 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="46" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F5.6: metrónomo como área propia, al estilo de tu app de referencia (MT-01 a MT-05)
- Barra vertical del tempo (30 a 250) con su nombre italiano, − y +,
  un punto por pulso, compás, «Marcar» y Empezar.
- Ventana de compás: doce compases, cuatro figuras y acento en el primer
  tiempo; en 6/8, 9/8 y 12/8 el pulso es la negra con puntillo.
- Golpes programados en el reloj de audio (menos de 1 ms de desviación);
  sigue sonando en otras áreas, se para al ocultar la app y con el micrófono.
- Banco 73 de 73; disposición del metrónomo en cinco pantallas.
- Documentos: requisitos v1.21, matriz v1.19, roadmap v3.19 (F5.8
  saneamiento), interfaz v1.11 (§7b aprobada), compatibilidad v1.7, IT-03.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.18. Base: requisitos.md v1.20 · app 0.5.3 · roadmap 3.18 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.19. Base: requisitos.md v1.21 · app 0.5.4 · roadmap 3.19 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>Escalas, habilitada desde la 0.5.0. Metrónomo (F5.6) y Acordes (F5.7) serán áreas propias (tu decisión del 21/10). Validado en la Sesión 1 (20/10, informe V-08): A12.</t>
+          <t>Escalas, habilitada desde la 0.5.0. Metrónomo, área propia desde la 0.5.4; Acordes lo será en F5.7 (tu decisión del 21/10). Validado en la Sesión 1 (20/10, informe V-08): A12.</t>
         </is>
       </c>
       <c r="P6" s="6" t="n"/>
@@ -2400,11 +2400,7 @@
         </is>
       </c>
       <c r="P26" s="6" t="n"/>
-      <c r="Q26" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q26" s="5" t="inlineStr"/>
     </row>
     <row r="27" ht="33" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -4651,11 +4647,7 @@
         </is>
       </c>
       <c r="P55" s="6" t="n"/>
-      <c r="Q55" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q55" s="5" t="inlineStr"/>
     </row>
     <row r="56" ht="33" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
@@ -5204,11 +5196,7 @@
         </is>
       </c>
       <c r="P62" s="6" t="n"/>
-      <c r="Q62" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q62" s="5" t="inlineStr"/>
     </row>
     <row r="63" ht="93" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -5682,11 +5670,7 @@
         </is>
       </c>
       <c r="P68" s="6" t="n"/>
-      <c r="Q68" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q68" s="5" t="inlineStr"/>
     </row>
     <row r="69" ht="33" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
@@ -6782,7 +6766,7 @@
       <c r="P82" s="6" t="n"/>
       <c r="Q82" s="5" t="inlineStr"/>
     </row>
-    <row r="83" ht="48" customHeight="1">
+    <row r="83" ht="108" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
         <is>
           <t>MT-01</t>
@@ -6795,7 +6779,7 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Metrónomo: tempo de 30 a 250 pulsos por minuto, con botones y «marcar el tempo» tocando a ritmo; arranca y para con un toque.</t>
+          <t>Metrónomo: tempo de 30 a 250 pulsos por minuto con una barra vertical, − y + y «Marcar» (tocando a ritmo), con su nombre italiano (Lento, Andante, Allegro…); arranca y para con un toque.</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
@@ -6825,27 +6809,27 @@
       </c>
       <c r="I83" s="5" t="inlineStr">
         <is>
-          <t>Tempo de 30 a 250 con botones y marcando el tempo; arranca y para con un toque; se usa en vertical y en horizontal sin aviso de girar.</t>
+          <t>Tempo de 30 a 250 con la barra vertical (también con el teclado), con − y + y marcando a ritmo, con su nombre italiano; arranca y para con un toque; en vertical y en horizontal sin aviso de girar.</t>
         </is>
       </c>
       <c r="J83" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K83" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="L83" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): barra con teclado, − y +, «Marcar» (media y reinicio tras 2 s), límites y nombre del tempo · comprobar-disposicion: cinco pantallas</t>
         </is>
       </c>
       <c r="M83" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N83" s="5" t="inlineStr">
@@ -6855,7 +6839,7 @@
       </c>
       <c r="O83" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10. Se usa igual en vertical y en horizontal: como el Afinador, no pide girar el móvil.</t>
+          <t>Tu petición del 21/10 y tu guía con la app que nos enseñaste: lo más directo. Se usa igual en vertical y en horizontal: como el Afinador, no pide girar el móvil. La barra se mueve también con las flechas del teclado. Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2).</t>
         </is>
       </c>
       <c r="P83" s="6" t="n"/>
@@ -6865,7 +6849,7 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="63" customHeight="1">
+    <row r="84" ht="108" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
         <is>
           <t>MT-02</t>
@@ -6878,7 +6862,7 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Compás elegible (2/4, 3/4, 4/4, 5/4, 6/8, 7/8 y 12/8) con acentos editables en cada tiempo: fuerte, normal o en silencio. Por defecto, el primero fuerte.</t>
+          <t>Compás elegible entre 1/4, 2/4, 3/4, 4/4, 5/4, 6/4, 3/8, 5/8, 6/8, 7/8, 9/8 y 12/8, en una ventana que se abre al tocar el compás; un punto por pulso (en 6/8, 9/8 y 12/8 el pulso es la negra con puntillo: dos, tres o cuatro puntos), y acento en el primer tiempo, que se puede quitar.</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
@@ -6908,27 +6892,27 @@
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>Cada compás del catálogo da su número de tiempos, con el primero fuerte por defecto; los acentos editados suenan como se marcan.</t>
+          <t>Los doce compases dan su número de pulsos (6/8, 9/8 y 12/8: 2, 3 y 4) y un punto por pulso; con acento, el primer pulso suena más agudo y fuerte, y sin él todos iguales.</t>
         </is>
       </c>
       <c r="J84" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K84" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="L84" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): puntos por compás, golpes con y sin acento, ventana que se abre y se cierra, datos guardados y validados</t>
         </is>
       </c>
       <c r="M84" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N84" s="5" t="inlineStr">
@@ -6938,13 +6922,17 @@
       </c>
       <c r="O84" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10.</t>
+          <t>Tu decisión del 21/10: como la app de referencia, un solo acento (el del primer tiempo) en vez de acentos en cada tiempo. Por defecto, con acento. Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2).</t>
         </is>
       </c>
       <c r="P84" s="6" t="n"/>
-      <c r="Q84" s="5" t="inlineStr"/>
-    </row>
-    <row r="85" ht="48" customHeight="1">
+      <c r="Q84" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="78" customHeight="1">
       <c r="A85" s="4" t="inlineStr">
         <is>
           <t>MT-03</t>
@@ -6957,7 +6945,7 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Subdivisión elegible: solo el pulso, corcheas, tresillos o semicorcheas; la subdivisión suena más suave que el pulso.</t>
+          <t>Subdivisión elegible con figuras en la misma ventana: solo el pulso, dos, tres o cuatro golpes por pulso; la subdivisión suena más suave que el pulso.</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
@@ -6987,27 +6975,27 @@
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>Cada subdivisión reparte el pulso en partes iguales, más suaves que el pulso.</t>
+          <t>Cada figura reparte el pulso en 1, 2, 3 o 4 golpes iguales, más suaves que el pulso; cambiarla sonando empieza en el próximo pulso, sin mover el pulso.</t>
         </is>
       </c>
       <c r="J85" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K85" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="L85" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): separación de las corcheas, volumen menor, cambio sonando</t>
         </is>
       </c>
       <c r="M85" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N85" s="5" t="inlineStr">
@@ -7017,13 +7005,17 @@
       </c>
       <c r="O85" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10 («ritmos»).</t>
+          <t>Tu petición del 21/10 («ritmos»). En los compases compuestos, tres golpes por pulso son las corcheas. Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2).</t>
         </is>
       </c>
       <c r="P85" s="6" t="n"/>
-      <c r="Q85" s="5" t="inlineStr"/>
-    </row>
-    <row r="86" ht="63" customHeight="1">
+      <c r="Q85" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="93" customHeight="1">
       <c r="A86" s="4" t="inlineStr">
         <is>
           <t>MT-04</t>
@@ -7066,27 +7058,27 @@
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>Los golpes programados a 30, 120 y 250 ppm se separan exactamente 60/tempo s (±1 ms) y el indicador marca el tiempo en curso; al ocultar la app se para.</t>
+          <t>Los golpes programados a 30, 120 y 250 ppm se separan exactamente 60/tempo s (±1 ms), nunca se programan más de 100 ms por adelantado y el punto del pulso se ilumina; al ocultar la app se para.</t>
         </is>
       </c>
       <c r="J86" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K86" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="L86" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): separación a 30, 120 y 250 ppm, cambio de tempo sonando sin adelantar ni repetir, parada al ocultar</t>
         </is>
       </c>
       <c r="M86" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N86" s="5" t="inlineStr">
@@ -7096,13 +7088,17 @@
       </c>
       <c r="O86" s="5" t="inlineStr">
         <is>
-          <t>Con un temporizador normal el pulso «se arrastra»: el reloj de audio es exacto. Lo de pararse sigue la regla del sonido en segundo plano (Sesión 1, C07).</t>
+          <t>Con un temporizador normal el pulso «se arrastra»: el reloj de audio es exacto. Lo de pararse sigue la regla del sonido en segundo plano (Sesión 1, C07). Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2).</t>
         </is>
       </c>
       <c r="P86" s="6" t="n"/>
-      <c r="Q86" s="5" t="inlineStr"/>
-    </row>
-    <row r="87" ht="93" customHeight="1">
+      <c r="Q86" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="120" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
         <is>
           <t>MT-05</t>
@@ -7145,27 +7141,27 @@
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>El metrónomo tiene su pestaña; en marcha, sigue sonando en Libre, Adivinar, Escalas y Acordes y su pestaña late con el pulso; al escuchar con el micrófono se para y lo dice; tempo, compás, acentos y subdivisión se recuerdan.</t>
+          <t>El metrónomo tiene su pestaña; en marcha, sigue sonando en las demás áreas y su pestaña late con el pulso; al escuchar con el micrófono se para y lo dice; tempo, compás, figura y acento se recuerdan.</t>
         </is>
       </c>
       <c r="J87" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K87" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="L87" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): sigue en Libre, pestaña que late, parada con el micrófono y aviso, datos guardados</t>
         </is>
       </c>
       <c r="M87" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N87" s="5" t="inlineStr">
@@ -7175,7 +7171,7 @@
       </c>
       <c r="O87" s="5" t="inlineStr">
         <is>
-          <t>Tu decisión del 21/10: función propia, no un chip del acceso rápido. Al escuchar con el micrófono en el Afinador, el metrónomo se para y lo dice: su clic confundiría al detector. Distribución de la pestaña: interfaz.md §7b, propuesta pendiente de tu visto bueno.</t>
+          <t>Tu decisión del 21/10: función propia, no un chip del acceso rápido. Al escuchar con el micrófono en el Afinador, el metrónomo se para y lo dice: su clic confundiría al detector. Distribución: interfaz.md §7b, aprobada el 21/10. Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2).</t>
         </is>
       </c>
       <c r="P87" s="6" t="n"/>
@@ -7262,11 +7258,7 @@
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
-      <c r="Q88" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q88" s="5" t="inlineStr"/>
     </row>
     <row r="89" ht="120" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
@@ -7345,11 +7337,7 @@
         </is>
       </c>
       <c r="P89" s="6" t="n"/>
-      <c r="Q89" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q89" s="5" t="inlineStr"/>
     </row>
     <row r="90" ht="48" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
@@ -7578,11 +7566,7 @@
         </is>
       </c>
       <c r="P92" s="6" t="n"/>
-      <c r="Q92" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q92" s="5" t="inlineStr"/>
     </row>
     <row r="93" ht="120" customHeight="1">
       <c r="A93" s="4" t="inlineStr">
@@ -8435,11 +8419,7 @@
         </is>
       </c>
       <c r="P103" s="6" t="n"/>
-      <c r="Q103" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q103" s="5" t="inlineStr"/>
     </row>
     <row r="104" ht="78" customHeight="1">
       <c r="A104" s="4" t="inlineStr">
@@ -8593,7 +8573,7 @@
       </c>
       <c r="O105" s="5" t="inlineStr">
         <is>
-          <t>Barra inferior con un destino por área en vertical (cuatro hoy; seis con Metrónomo y Acordes, con pestañas de al menos 44 px), raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05). Validado en la Sesión 1 (20/10, informe V-08): A19.</t>
+          <t>Barra inferior con un destino por área en vertical (cinco desde la 0.5.4, con Metrónomo; seis con Acordes; en el raíl, pestañas de 44 px), raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05). Validado en la Sesión 1 (20/10, informe V-08): A19.</t>
         </is>
       </c>
       <c r="P105" s="6" t="n"/>
@@ -9885,7 +9865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9925,7 +9905,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -9935,24 +9915,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.5.3</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
+          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -9962,24 +9942,24 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.5.2</t>
+          <t>0.5.3</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
+          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -9989,24 +9969,24 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.5.0</t>
+          <t>0.5.2</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
+          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -10016,24 +9996,24 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.4.2</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
+          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -10043,51 +10023,51 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.4.0</t>
+          <t>0.4.2</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
+          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.3.3</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
+          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -10097,24 +10077,24 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.3.2</t>
+          <t>0.3.3</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
+          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -10124,24 +10104,24 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>0.3.1</t>
+          <t>0.3.2</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
+          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -10151,24 +10131,24 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -10178,24 +10158,24 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -10205,7 +10185,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -10215,14 +10195,14 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -10232,7 +10212,7 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -10242,24 +10222,24 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
@@ -10269,14 +10249,14 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -10286,24 +10266,24 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -10313,24 +10293,24 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -10340,51 +10320,51 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -10394,7 +10374,7 @@
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
@@ -10404,32 +10384,59 @@
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="46" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F5.7: librería de acordes con listado, buscador y el acorde en el mástil (AC-01 a AC-06)
- Listado a un lado: populares (C, G, D, A, E, Am, Em, Dm, F) y los 30
  acordes más habituales; buscador por el principio del nombre, en las dos
  nomenclaturas («G» deja G, Gm, G7, G/B).
- El acorde en el mástil: dedos con número y color constante (Okabe-Ito),
  ○ y ✕ junto a cada cuerda, cejilla como barra; pentagrama con las notas
  escritas como manda el acorde; rasgueo de grave a agudo.
- Con otra afinación, aviso y «Pasar a estándar».
- Seis pestañas: raíl de 44 px y cabecera alineada a la derecha entre 600 y 959 px.
- Banco 78 de 78 (las 30 digitaciones, una a una); disposición en seis pantallas.
- Documentos: requisitos v1.22 (AC-06 nuevo), matriz v1.20, roadmap v3.20,
  interfaz v1.12, IT-03 y CHANGELOG.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control de cambios" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz'!$A$4:$Q$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz'!$A$4:$Q$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q112"/>
+  <dimension ref="A1:Q113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.19. Base: requisitos.md v1.21 · app 0.5.4 · roadmap 3.19 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.20. Base: requisitos.md v1.22 · app 0.5.5 · roadmap 3.20 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>Escalas, habilitada desde la 0.5.0. Metrónomo, área propia desde la 0.5.4; Acordes lo será en F5.7 (tu decisión del 21/10). Validado en la Sesión 1 (20/10, informe V-08): A12.</t>
+          <t>Escalas, habilitada desde la 0.5.0. Metrónomo, área propia desde la 0.5.4, y Acordes desde la 0.5.5 (tu decisión del 21/10). Validado en la Sesión 1 (20/10, informe V-08): A12.</t>
         </is>
       </c>
       <c r="P6" s="6" t="n"/>
@@ -6843,11 +6843,7 @@
         </is>
       </c>
       <c r="P83" s="6" t="n"/>
-      <c r="Q83" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q83" s="5" t="inlineStr"/>
     </row>
     <row r="84" ht="108" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
@@ -6926,11 +6922,7 @@
         </is>
       </c>
       <c r="P84" s="6" t="n"/>
-      <c r="Q84" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q84" s="5" t="inlineStr"/>
     </row>
     <row r="85" ht="78" customHeight="1">
       <c r="A85" s="4" t="inlineStr">
@@ -7009,11 +7001,7 @@
         </is>
       </c>
       <c r="P85" s="6" t="n"/>
-      <c r="Q85" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q85" s="5" t="inlineStr"/>
     </row>
     <row r="86" ht="93" customHeight="1">
       <c r="A86" s="4" t="inlineStr">
@@ -7092,11 +7080,7 @@
         </is>
       </c>
       <c r="P86" s="6" t="n"/>
-      <c r="Q86" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q86" s="5" t="inlineStr"/>
     </row>
     <row r="87" ht="120" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
@@ -7175,90 +7159,90 @@
         </is>
       </c>
       <c r="P87" s="6" t="n"/>
-      <c r="Q87" s="5" t="inlineStr">
+      <c r="Q87" s="5" t="inlineStr"/>
+    </row>
+    <row r="88" ht="120" customHeight="1">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>AC-01</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Acordes</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Librería de acordes, un área propia: a un lado, el listado de nombres, con una sección de populares arriba y debajo los 30 acordes más habituales; al otro, el acorde dibujado en el mástil.</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Cliente · 21/10</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>F5.7</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>El listado tiene populares arriba y los 30 acordes debajo; cada digitación suena solo a notas del acorde, con la raíz, la tercera y la séptima (la quinta se puede omitir) y la raíz o el bajo indicado como nota más grave.</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="K88" s="5" t="inlineStr">
+        <is>
+          <t>0.5.5</t>
+        </is>
+      </c>
+      <c r="L88" s="5" t="inlineStr">
+        <is>
+          <t>Banco (node --test): las 30 digitaciones, una a una; populares y listado</t>
+        </is>
+      </c>
+      <c r="M88" s="5" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="N88" s="5" t="inlineStr">
+        <is>
+          <t>Banco automático + auditor técnico</t>
+        </is>
+      </c>
+      <c r="O88" s="5" t="inlineStr">
+        <is>
+          <t>Tu petición del 21/10 («ya iremos ampliando»). Populares: C, G, D, A, E, Am, Em, Dm y F. Los 30: mayores, menores, 7, m7 y maj7 de uso común, Dsus4, C/G y G/B, en posición abierta o con las cejillas más habituales. En vertical el listado va arriba y el mástil abajo; en horizontal, el listado a la derecha. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
+        </is>
+      </c>
+      <c r="P88" s="6" t="n"/>
+      <c r="Q88" s="5" t="inlineStr">
         <is>
           <t>Modificado</t>
         </is>
       </c>
-    </row>
-    <row r="88" ht="63" customHeight="1">
-      <c r="A88" s="4" t="inlineStr">
-        <is>
-          <t>AC-01</t>
-        </is>
-      </c>
-      <c r="B88" s="5" t="inlineStr">
-        <is>
-          <t>Acordes</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>Librería de acordes con tónica y tipo: mayores, menores y de séptima (7, maj7 y m7) en posición abierta, más las cejillas más habituales.</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
-          <t>Cliente · 21/10</t>
-        </is>
-      </c>
-      <c r="F88" s="5" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="inlineStr">
-        <is>
-          <t>F5.7</t>
-        </is>
-      </c>
-      <c r="H88" s="5" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="I88" s="5" t="inlineStr">
-        <is>
-          <t>El catálogo tiene mayores, menores, 7, maj7 y m7 abiertos y cejillas habituales; cada digitación produce exactamente las notas del acorde.</t>
-        </is>
-      </c>
-      <c r="J88" s="5" t="inlineStr">
-        <is>
-          <t>No cumple</t>
-        </is>
-      </c>
-      <c r="K88" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L88" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M88" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="N88" s="5" t="inlineStr">
-        <is>
-          <t>Banco automático + auditor técnico</t>
-        </is>
-      </c>
-      <c r="O88" s="5" t="inlineStr">
-        <is>
-          <t>Tu petición del 21/10; el catálogo lo propone el agente: unos 30 acordes, los que salen en la mayoría de canciones. Es un área propia, con su pestaña (interfaz.md §7b).</t>
-        </is>
-      </c>
-      <c r="P88" s="6" t="n"/>
-      <c r="Q88" s="5" t="inlineStr"/>
     </row>
     <row r="89" ht="120" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
@@ -7273,7 +7257,7 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>En el mástil, cada nota del acorde lleva un círculo del color de su dedo (1 índice, 2 medio, 3 anular, 4 meñique; el mismo color en todos los acordes) con el número del dedo dentro. Junto a la cejuela, ○ para cuerda al aire y ✕ para cuerda que no suena; la cejilla, marcada.</t>
+          <t>En el mástil, cada nota del acorde lleva un círculo del color de su dedo (1 índice, 2 medio, 3 anular, 4 meñique; el mismo color en todos los acordes) con el número del dedo dentro. Junto al nombre de cada cuerda, ○ si suena al aire y ✕ si no suena; la cejilla, como una barra que une sus cuerdas.</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
@@ -7303,27 +7287,27 @@
       </c>
       <c r="I89" s="5" t="inlineStr">
         <is>
-          <t>Cada dedo tiene su número y su color, iguales en todos los acordes y distintos de la paleta de notas; círculo ≥ 3:1 contra el mástil y número ≥ 4,5:1 contra el círculo; cuerdas al aire y apagadas marcadas; cejilla marcada.</t>
+          <t>Cada dedo tiene su número y su color, iguales en todos los acordes (Okabe-Ito); círculo ≥ 3:1 contra el mástil y número ≥ 4,5:1 contra el círculo; ○ y ✕ junto al nombre de la cuerda; cejilla como barra; el lector de pantalla dice el dedo.</t>
         </is>
       </c>
       <c r="J89" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K89" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.5</t>
         </is>
       </c>
       <c r="L89" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): La menor y Fa dibujados, contraste de los cuatro colores · comprobar-accesibilidad: Acordes con Fa</t>
         </is>
       </c>
       <c r="M89" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N89" s="5" t="inlineStr">
@@ -7333,13 +7317,17 @@
       </c>
       <c r="O89" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10: número y color a la vez, con el color constante entre acordes. Los cuatro colores de dedo son distintos de la paleta de notas (que va por nota) y distintos entre sí también para daltónicos; cada círculo contrasta al menos 3:1 con el mástil y su número al menos 4,5:1 con el círculo (G-05).</t>
+          <t>Tu petición del 21/10: número y color a la vez, con el color constante entre acordes. Colores de la paleta Okabe-Ito, que se distinguen también con daltonismo; en Acordes no se ven los colores de nota, así que no se confunden con ellos. Cada círculo contrasta al menos 3:1 con el mástil y su número al menos 4,5:1 con el círculo (G-05). El lector de pantalla dice el dedo de cada casilla. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
         </is>
       </c>
       <c r="P89" s="6" t="n"/>
-      <c r="Q89" s="5" t="inlineStr"/>
-    </row>
-    <row r="90" ht="48" customHeight="1">
+      <c r="Q89" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="93" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
         <is>
           <t>AC-03</t>
@@ -7352,7 +7340,7 @@
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>El pentagrama escribe el acorde con sus notas apiladas; se oculta con el ajuste de pentagrama de siempre.</t>
+          <t>El pentagrama escribe el acorde con sus notas apiladas, escritas como manda el acorde (B7: Re♯); se oculta con el ajuste de pentagrama de siempre.</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
@@ -7382,27 +7370,27 @@
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>El pentagrama escribe las notas del acorde apiladas y se oculta con su ajuste.</t>
+          <t>El pentagrama escribe las notas del acorde apiladas, escritas como manda el acorde, y se oculta con su ajuste; en el móvil en vertical se aparta y vuelve al girarlo.</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K90" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.5</t>
         </is>
       </c>
       <c r="L90" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): cinco notas de La menor; B7 con Re♯ · comprobar-disposicion: seis pantallas</t>
         </is>
       </c>
       <c r="M90" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N90" s="5" t="inlineStr">
@@ -7410,11 +7398,19 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O90" s="5" t="inlineStr"/>
+      <c r="O90" s="5" t="inlineStr">
+        <is>
+          <t>En el móvil en vertical el pentagrama se aparta para que el listado y el mástil quepan; se ve al girar el móvil y en pantallas amplias. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
+        </is>
+      </c>
       <c r="P90" s="6" t="n"/>
-      <c r="Q90" s="5" t="inlineStr"/>
-    </row>
-    <row r="91" ht="33" customHeight="1">
+      <c r="Q90" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="48" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
         <is>
           <t>AC-04</t>
@@ -7427,7 +7423,7 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>El acorde suena rasgueado, de grave a agudo, al tocarlo; cada cuerda se puede tocar suelta.</t>
+          <t>El acorde suena rasgueado, de grave a agudo, al elegirlo y con «Tocar»; cada cuerda se puede tocar suelta.</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
@@ -7457,27 +7453,27 @@
       </c>
       <c r="I91" s="5" t="inlineStr">
         <is>
-          <t>El acorde suena rasgueado de grave a agudo; cada cuerda se puede tocar suelta.</t>
+          <t>El acorde suena rasgueado de grave a agudo al elegirlo y con «Tocar»; cada cuerda se puede tocar suelta.</t>
         </is>
       </c>
       <c r="J91" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K91" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.5</t>
         </is>
       </c>
       <c r="L91" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): orden del rasgueo</t>
         </is>
       </c>
       <c r="M91" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N91" s="5" t="inlineStr">
@@ -7485,11 +7481,19 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O91" s="5" t="inlineStr"/>
+      <c r="O91" s="5" t="inlineStr">
+        <is>
+          <t>35 ms entre cuerda y cuerda. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
+        </is>
+      </c>
       <c r="P91" s="6" t="n"/>
-      <c r="Q91" s="5" t="inlineStr"/>
-    </row>
-    <row r="92" ht="93" customHeight="1">
+      <c r="Q91" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="63" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
         <is>
           <t>AC-05</t>
@@ -7502,7 +7506,7 @@
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Las digitaciones son para la afinación estándar en la primera entrega.</t>
+          <t>Las digitaciones son para la afinación estándar en la primera entrega: con otra afinación activa, Acordes lo avisa, no las dibuja y ofrece pasar a la estándar.</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
@@ -7527,205 +7531,217 @@
       </c>
       <c r="H92" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>T</t>
         </is>
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Las digitaciones indican que son para la afinación estándar; con otra afinación, Acordes lo avisa y ofrece pasar a la estándar; el selector no ofrece combinaciones sin digitación.</t>
+          <t>Con otra afinación, Acordes avisa, no dibuja las digitaciones y «Pasar a estándar» las recupera.</t>
         </is>
       </c>
       <c r="J92" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K92" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.5.5</t>
         </is>
       </c>
       <c r="L92" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): Drop D y vuelta a la estándar</t>
         </is>
       </c>
       <c r="M92" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N92" s="5" t="inlineStr">
         <is>
-          <t>Auditor de requisitos</t>
+          <t>Banco automático + auditor técnico</t>
         </is>
       </c>
       <c r="O92" s="5" t="inlineStr">
         <is>
-          <t>Las digitaciones dependen de la afinación; las demás, para después. Con otra afinación activa, Acordes lo avisa y ofrece pasar a la estándar. El selector de tipo solo ofrece los tipos que el catálogo tiene para esa tónica: no hay combinaciones vacías.</t>
+          <t>Las digitaciones dependen de la afinación; las demás, para después. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
         </is>
       </c>
       <c r="P92" s="6" t="n"/>
-      <c r="Q92" s="5" t="inlineStr"/>
-    </row>
-    <row r="93" ht="120" customHeight="1">
+      <c r="Q92" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="93" customHeight="1">
       <c r="A93" s="4" t="inlineStr">
         <is>
+          <t>AC-06</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Acordes</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Un buscador filtra el listado por cómo empieza el nombre: «G» deja G, Gm, G7, G/B…; vale en las dos nomenclaturas («Sol» encuentra lo mismo) y sin distinguir mayúsculas.</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>Cliente · 21/10</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>F5.7</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>El buscador deja los acordes que empiezan por lo escrito, sin distinguir mayúsculas y en las dos nomenclaturas; una letra sola, solo en la inglesa.</t>
+        </is>
+      </c>
+      <c r="J93" s="5" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="K93" s="5" t="inlineStr">
+        <is>
+          <t>0.5.5</t>
+        </is>
+      </c>
+      <c r="L93" s="5" t="inlineStr">
+        <is>
+          <t>Banco (node --test): G, g, Sol, D, Am, f# y vacío</t>
+        </is>
+      </c>
+      <c r="M93" s="5" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="N93" s="5" t="inlineStr">
+        <is>
+          <t>Banco automático + auditor técnico</t>
+        </is>
+      </c>
+      <c r="O93" s="5" t="inlineStr">
+        <is>
+          <t>Tu petición del 21/10. Una sola letra solo se busca en la nomenclatura inglesa, para que «D» no traiga también los Do; # y b valen por ♯ y ♭. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
+        </is>
+      </c>
+      <c r="P93" s="6" t="n"/>
+      <c r="Q93" s="5" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="120" customHeight="1">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
           <t>V-01</t>
         </is>
       </c>
-      <c r="B93" s="5" t="inlineStr">
+      <c r="B94" s="5" t="inlineStr">
         <is>
           <t>Visualización</t>
         </is>
       </c>
-      <c r="C93" s="5" t="inlineStr">
+      <c r="C94" s="5" t="inlineStr">
         <is>
           <t>En móvil se sugiere la orientación horizontal con un aviso discreto; no se fuerza.</t>
         </is>
       </c>
-      <c r="D93" s="5" t="inlineStr">
+      <c r="D94" s="5" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="E93" s="5" t="inlineStr">
+      <c r="E94" s="5" t="inlineStr">
         <is>
           <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
-      <c r="F93" s="5" t="inlineStr">
+      <c r="F94" s="5" t="inlineStr">
         <is>
           <t>F3</t>
         </is>
       </c>
-      <c r="G93" s="5" t="inlineStr">
+      <c r="G94" s="5" t="inlineStr">
         <is>
           <t>F3.2</t>
         </is>
       </c>
-      <c r="H93" s="5" t="inlineStr">
+      <c r="H94" s="5" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="I93" s="5" t="inlineStr">
+      <c r="I94" s="5" t="inlineStr">
         <is>
           <t>En horizontal, con un alto útil de 268 px o más, cada cuerda mide al menos 40 px (iPhone en Safari e instalada; simulador de Android). En vertical, en pantallas táctiles de menos de 600 px de ancho y en Libre, Adivinar y Escalas, aparece el aviso para girar; nunca en el Afinador; cerrado, no vuelve y «Restablecer» lo recupera.</t>
         </is>
       </c>
-      <c r="J93" s="5" t="inlineStr">
+      <c r="J94" s="5" t="inlineStr">
         <is>
           <t>Cumple</t>
         </is>
       </c>
-      <c r="K93" s="5" t="inlineStr">
+      <c r="K94" s="5" t="inlineStr">
         <is>
           <t>0.3.0</t>
         </is>
       </c>
-      <c r="L93" s="5" t="inlineStr">
+      <c r="L94" s="5" t="inlineStr">
         <is>
           <t>V-06: comprobar-disposicion.js en 14 pantallas: 52,8 / 60,8 / 42,5 px · Banco (node --test): aviso para girar · Sesión 1: C02, C03 y D03</t>
         </is>
       </c>
-      <c r="M93" s="5" t="inlineStr">
+      <c r="M94" s="5" t="inlineStr">
         <is>
           <t>Verificado</t>
         </is>
       </c>
-      <c r="N93" s="5" t="inlineStr">
+      <c r="N94" s="5" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O93" s="5" t="inlineStr">
+      <c r="O94" s="5" t="inlineStr">
         <is>
           <t>Hecho en la 0.3.0 según interfaz.md §7. En horizontal, raíl, mástil a todo el alto y panel: medido en Chromium, 52,8 px por cuerda en el iPhone con Safari (antes 28,8), 60,8 con la app instalada y 42,5 en un Android de 280 px de alto (V-06). El aviso para girar sale solo con el dedo, en vertical y en pantallas de menos de 600 px de ancho, en Libre y Adivinar (y Escalas desde F5), nunca en el Afinador; cerrado no vuelve y «Restablecer» lo recupera. El bloqueo de orientación tiene mal soporte en iOS, así que no se fuerza. Validado en la Sesión 1 (20/10, informe V-08): C02, C03 y D03.</t>
         </is>
       </c>
-      <c r="P93" s="6" t="n"/>
-      <c r="Q93" s="5" t="inlineStr"/>
-    </row>
-    <row r="94" ht="33" customHeight="1">
-      <c r="A94" s="4" t="inlineStr">
-        <is>
-          <t>V-02</t>
-        </is>
-      </c>
-      <c r="B94" s="5" t="inlineStr">
-        <is>
-          <t>Visualización</t>
-        </is>
-      </c>
-      <c r="C94" s="5" t="inlineStr">
-        <is>
-          <t>El afinador funciona en vertical y en horizontal.</t>
-        </is>
-      </c>
-      <c r="D94" s="5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="E94" s="5" t="inlineStr">
-        <is>
-          <t>Cliente · listado 14/09</t>
-        </is>
-      </c>
-      <c r="F94" s="5" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="G94" s="5" t="inlineStr">
-        <is>
-          <t>F1.1</t>
-        </is>
-      </c>
-      <c r="H94" s="5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="I94" s="5" t="inlineStr">
-        <is>
-          <t>El afinador se usa con comodidad en vertical y en horizontal.</t>
-        </is>
-      </c>
-      <c r="J94" s="5" t="inlineStr">
-        <is>
-          <t>Cumple</t>
-        </is>
-      </c>
-      <c r="K94" s="5" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="L94" s="5" t="inlineStr">
-        <is>
-          <t>F1.1 #14</t>
-        </is>
-      </c>
-      <c r="M94" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="N94" s="5" t="inlineStr">
-        <is>
-          <t>Cliente</t>
-        </is>
-      </c>
-      <c r="O94" s="5" t="inlineStr"/>
       <c r="P94" s="6" t="n"/>
       <c r="Q94" s="5" t="inlineStr"/>
     </row>
     <row r="95" ht="33" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>V-03</t>
+          <t>V-02</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -7735,7 +7751,7 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>En escritorio el mástil aprovecha el ancho disponible.</t>
+          <t>El afinador funciona en vertical y en horizontal.</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
@@ -7765,7 +7781,7 @@
       </c>
       <c r="I95" s="5" t="inlineStr">
         <is>
-          <t>En una pantalla de 1280 px se ven los 24 trastes sin desplazarse.</t>
+          <t>El afinador se usa con comodidad en vertical y en horizontal.</t>
         </is>
       </c>
       <c r="J95" s="5" t="inlineStr">
@@ -7793,18 +7809,14 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O95" s="5" t="inlineStr">
-        <is>
-          <t>Arranca mostrando el mástil completo en pantallas anchas.</t>
-        </is>
-      </c>
+      <c r="O95" s="5" t="inlineStr"/>
       <c r="P95" s="6" t="n"/>
       <c r="Q95" s="5" t="inlineStr"/>
     </row>
-    <row r="96" ht="120" customHeight="1">
+    <row r="96" ht="33" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>V-04</t>
+          <t>V-03</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
@@ -7814,7 +7826,7 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Control de zoom que determina qué porción del mástil se ve.</t>
+          <t>En escritorio el mástil aprovecha el ancho disponible.</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
@@ -7824,17 +7836,17 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
+          <t>Cliente · listado 14/09</t>
         </is>
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>F1 · F3</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
-          <t>F1.1 · F3.2</t>
+          <t>F1.1</t>
         </is>
       </c>
       <c r="H96" s="5" t="inlineStr">
@@ -7844,7 +7856,7 @@
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>El zoom cambia los trastes visibles entre 3 y el máximo que cabe, y la etiqueta dice la cifra real; «+» enseña más trastes y «−» menos. Con pointer: coarse, la vista por defecto usa trastes de al menos 40 px y el usuario puede pedir más trastes, de hasta 28 px; si el zoom guardado pide más de los que caben, se muestran los que caben y lo guardado se conserva (V-08).</t>
+          <t>En una pantalla de 1280 px se ven los 24 trastes sin desplazarse.</t>
         </is>
       </c>
       <c r="J96" s="5" t="inlineStr">
@@ -7859,12 +7871,12 @@
       </c>
       <c r="L96" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7 y #8 · V-06 · Banco (node --test): 40 px por defecto, 28 con «+», orden de los botones · Sesión 1: A07, A08 y C04</t>
+          <t>F1.1 #14</t>
         </is>
       </c>
       <c r="M96" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="N96" s="5" t="inlineStr">
@@ -7874,16 +7886,16 @@
       </c>
       <c r="O96" s="5" t="inlineStr">
         <is>
-          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Desde la 0.3.0, con el dedo la vista por defecto usa trastes de 40 px o más (34 con ratón), y la cejuela mide 40. Desde la 0.3.2 (tu comentario del 20/10), «+» enseña más trastes y «−» menos, y con el dedo puedes pedir trastes de hasta 28 px: en el iPhone con Safari, hasta 11 a la vista en vertical y 15 en horizontal. Si el zoom guardado pide más, se muestran los que caben y la etiqueta lo dice, pero lo guardado se conserva para que al girar vuelva (V-08). Validado en la Sesión 1 (20/10, informe V-08): A07, A08 y C04.</t>
+          <t>Arranca mostrando el mástil completo en pantallas anchas.</t>
         </is>
       </c>
       <c r="P96" s="6" t="n"/>
       <c r="Q96" s="5" t="inlineStr"/>
     </row>
-    <row r="97" ht="33" customHeight="1">
+    <row r="97" ht="120" customHeight="1">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>V-05</t>
+          <t>V-04</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -7893,7 +7905,7 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Cuando el mástil no cabe, el usuario se desplaza lateralmente.</t>
+          <t>Control de zoom que determina qué porción del mástil se ve.</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
@@ -7903,17 +7915,17 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 · F3</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>F1.1</t>
+          <t>F1.1 · F3.2</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr">
@@ -7923,7 +7935,7 @@
       </c>
       <c r="I97" s="5" t="inlineStr">
         <is>
-          <t>Con el mástil más ancho que la pantalla se puede desplazar hasta el traste 24.</t>
+          <t>El zoom cambia los trastes visibles entre 3 y el máximo que cabe, y la etiqueta dice la cifra real; «+» enseña más trastes y «−» menos. Con pointer: coarse, la vista por defecto usa trastes de al menos 40 px y el usuario puede pedir más trastes, de hasta 28 px; si el zoom guardado pide más de los que caben, se muestran los que caben y lo guardado se conserva (V-08).</t>
         </is>
       </c>
       <c r="J97" s="5" t="inlineStr">
@@ -7933,12 +7945,12 @@
       </c>
       <c r="K97" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A08.</t>
+          <t>0.1.0</t>
         </is>
       </c>
       <c r="L97" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14 · Sesión 1: A08</t>
+          <t>F1.1 #7 y #8 · V-06 · Banco (node --test): 40 px por defecto, 28 con «+», orden de los botones · Sesión 1: A07, A08 y C04</t>
         </is>
       </c>
       <c r="M97" s="5" t="inlineStr">
@@ -7951,14 +7963,18 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O97" s="5" t="inlineStr"/>
+      <c r="O97" s="5" t="inlineStr">
+        <is>
+          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Desde la 0.3.0, con el dedo la vista por defecto usa trastes de 40 px o más (34 con ratón), y la cejuela mide 40. Desde la 0.3.2 (tu comentario del 20/10), «+» enseña más trastes y «−» menos, y con el dedo puedes pedir trastes de hasta 28 px: en el iPhone con Safari, hasta 11 a la vista en vertical y 15 en horizontal. Si el zoom guardado pide más, se muestran los que caben y la etiqueta lo dice, pero lo guardado se conserva para que al girar vuelva (V-08). Validado en la Sesión 1 (20/10, informe V-08): A07, A08 y C04.</t>
+        </is>
+      </c>
       <c r="P97" s="6" t="n"/>
       <c r="Q97" s="5" t="inlineStr"/>
     </row>
-    <row r="98" ht="48" customHeight="1">
+    <row r="98" ht="33" customHeight="1">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>V-06</t>
+          <t>V-05</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
@@ -7968,7 +7984,7 @@
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>El ancho de traste no cambia al desplazarse: el zoom fija el tamaño y el desplazamiento mueve la ventana.</t>
+          <t>Cuando el mástil no cabe, el usuario se desplaza lateralmente.</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
@@ -7998,7 +8014,7 @@
       </c>
       <c r="I98" s="5" t="inlineStr">
         <is>
-          <t>Desplazarse no cambia el ancho de los trastes.</t>
+          <t>Con el mástil más ancho que la pantalla se puede desplazar hasta el traste 24.</t>
         </is>
       </c>
       <c r="J98" s="5" t="inlineStr">
@@ -8008,12 +8024,12 @@
       </c>
       <c r="K98" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A07.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A08.</t>
         </is>
       </c>
       <c r="L98" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7 · Sesión 1: A07</t>
+          <t>F1.1 #14 · Sesión 1: A08</t>
         </is>
       </c>
       <c r="M98" s="5" t="inlineStr">
@@ -8030,10 +8046,10 @@
       <c r="P98" s="6" t="n"/>
       <c r="Q98" s="5" t="inlineStr"/>
     </row>
-    <row r="99" ht="33" customHeight="1">
+    <row r="99" ht="48" customHeight="1">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>V-07</t>
+          <t>V-06</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -8043,7 +8059,7 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>El mástil se readapta al redimensionar la ventana.</t>
+          <t>El ancho de traste no cambia al desplazarse: el zoom fija el tamaño y el desplazamiento mueve la ventana.</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
@@ -8073,7 +8089,7 @@
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>Al redimensionar la ventana el mástil se reajusta sin perder el tramo visible.</t>
+          <t>Desplazarse no cambia el ancho de los trastes.</t>
         </is>
       </c>
       <c r="J99" s="5" t="inlineStr">
@@ -8083,12 +8099,12 @@
       </c>
       <c r="K99" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A08.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A07.</t>
         </is>
       </c>
       <c r="L99" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7 · Sesión 1: A08</t>
+          <t>F1.1 #7 · Sesión 1: A07</t>
         </is>
       </c>
       <c r="M99" s="5" t="inlineStr">
@@ -8108,7 +8124,7 @@
     <row r="100" ht="33" customHeight="1">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>V-08</t>
+          <t>V-07</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
@@ -8118,12 +8134,12 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>El nivel de zoom persiste entre sesiones.</t>
+          <t>El mástil se readapta al redimensionar la ventana.</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -8148,7 +8164,7 @@
       </c>
       <c r="I100" s="5" t="inlineStr">
         <is>
-          <t>El zoom se mantiene tras recargar y tras girar el móvil.</t>
+          <t>Al redimensionar la ventana el mástil se reajusta sin perder el tramo visible.</t>
         </is>
       </c>
       <c r="J100" s="5" t="inlineStr">
@@ -8158,17 +8174,17 @@
       </c>
       <c r="K100" s="5" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A08.</t>
         </is>
       </c>
       <c r="L100" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #13</t>
+          <t>F1.1 #7 · Sesión 1: A08</t>
         </is>
       </c>
       <c r="M100" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N100" s="5" t="inlineStr">
@@ -8176,18 +8192,14 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O100" s="5" t="inlineStr">
-        <is>
-          <t>Desde 0.1.1 girar el móvil ya no pisa el zoom elegido.</t>
-        </is>
-      </c>
+      <c r="O100" s="5" t="inlineStr"/>
       <c r="P100" s="6" t="n"/>
       <c r="Q100" s="5" t="inlineStr"/>
     </row>
-    <row r="101" ht="63" customHeight="1">
+    <row r="101" ht="33" customHeight="1">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>V-09</t>
+          <t>V-08</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -8197,17 +8209,17 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Al ocultar la numeración se puede conservar una referencia de tramo: el modo «Guía» deja solo los números de los trastes con marca.</t>
+          <t>El nivel de zoom persiste entre sesiones.</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>AR-01</t>
+          <t>Cliente · listado 14/09</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
@@ -8217,17 +8229,17 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>F1.3</t>
+          <t>F1.1</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>D</t>
         </is>
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>El modo Guía mantiene visibles solo los números de los trastes con marca.</t>
+          <t>El zoom se mantiene tras recargar y tras girar el móvil.</t>
         </is>
       </c>
       <c r="J101" s="5" t="inlineStr">
@@ -8237,56 +8249,56 @@
       </c>
       <c r="K101" s="5" t="inlineStr">
         <is>
-          <t>0.1.2</t>
+          <t>0.1.0</t>
         </is>
       </c>
       <c r="L101" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test) · F1.1 #11 · Sesión 1: A11</t>
+          <t>F1.1 #13</t>
         </is>
       </c>
       <c r="M101" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="N101" s="5" t="inlineStr">
         <is>
-          <t>Banco automático + auditor técnico</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="O101" s="5" t="inlineStr">
         <is>
-          <t>Sin números, los trastes 5 y 17 llevan la misma marca y se confunden. Se descartó el minimapa por desproporcionado. Validado en la Sesión 1 (20/10, informe V-08): A11.</t>
+          <t>Desde 0.1.1 girar el móvil ya no pisa el zoom elegido.</t>
         </is>
       </c>
       <c r="P101" s="6" t="n"/>
       <c r="Q101" s="5" t="inlineStr"/>
     </row>
-    <row r="102" ht="108" customHeight="1">
+    <row r="102" ht="63" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>C-01</t>
+          <t>V-09</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>Configuración y navegación</t>
+          <t>Visualización</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>Menú de configuración accesible desde cualquier pantalla.</t>
+          <t>Al ocultar la numeración se puede conservar una referencia de tramo: el modo «Guía» deja solo los números de los trastes con marca.</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>AR-01</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
@@ -8296,17 +8308,17 @@
       </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
-          <t>F1.1</t>
+          <t>F1.3</t>
         </is>
       </c>
       <c r="H102" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T</t>
         </is>
       </c>
       <c r="I102" s="5" t="inlineStr">
         <is>
-          <t>El botón de Ajustes abre el panel desde cualquier pantalla y Escape lo cierra.</t>
+          <t>El modo Guía mantiene visibles solo los números de los trastes con marca.</t>
         </is>
       </c>
       <c r="J102" s="5" t="inlineStr">
@@ -8316,12 +8328,12 @@
       </c>
       <c r="K102" s="5" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>0.1.2</t>
         </is>
       </c>
       <c r="L102" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14 · Sesión 1: A19 y C05</t>
+          <t>Banco (node --test) · F1.1 #11 · Sesión 1: A11</t>
         </is>
       </c>
       <c r="M102" s="5" t="inlineStr">
@@ -8331,21 +8343,21 @@
       </c>
       <c r="N102" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Banco automático + auditor técnico</t>
         </is>
       </c>
       <c r="O102" s="5" t="inlineStr">
         <is>
-          <t>Hoja que sube desde abajo en vertical; panel lateral en horizontal y en pantallas amplias, con un segundo botón en el raíl (0.3.0). Es un diálogo: mientras está abierto, el resto de la página no responde (AT-04). Validado en la Sesión 1 (20/10, informe V-08): A19 y C05.</t>
+          <t>Sin números, los trastes 5 y 17 llevan la misma marca y se confunden. Se descartó el minimapa por desproporcionado. Validado en la Sesión 1 (20/10, informe V-08): A11.</t>
         </is>
       </c>
       <c r="P102" s="6" t="n"/>
       <c r="Q102" s="5" t="inlineStr"/>
     </row>
-    <row r="103" ht="120" customHeight="1">
+    <row r="103" ht="108" customHeight="1">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>C-02</t>
+          <t>C-01</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
@@ -8355,7 +8367,7 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>El menú contiene nomenclatura, pentagrama, timbre, numeración de trastes (tres modos), ver todas las notas, señalar iguales y afinación activa, y muestra la versión de la app.</t>
+          <t>Menú de configuración accesible desde cualquier pantalla.</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
@@ -8380,12 +8392,12 @@
       </c>
       <c r="H103" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>D</t>
         </is>
       </c>
       <c r="I103" s="5" t="inlineStr">
         <is>
-          <t>El panel contiene todos los ajustes listados, el idioma (0.4.2) y la versión de la app.</t>
+          <t>El botón de Ajustes abre el panel desde cualquier pantalla y Escape lo cierra.</t>
         </is>
       </c>
       <c r="J103" s="5" t="inlineStr">
@@ -8400,31 +8412,31 @@
       </c>
       <c r="L103" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #12 · Banco (node --test): grupo Idioma</t>
+          <t>F1.1 #14 · Sesión 1: A19 y C05</t>
         </is>
       </c>
       <c r="M103" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N103" s="5" t="inlineStr">
         <is>
-          <t>Auditor de requisitos</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="O103" s="5" t="inlineStr">
         <is>
-          <t>Ampliado en 0.1.2 con la numeración en tres modos y la versión (G-10). En F6.4 se añade el grupo «Acerca de», con los créditos (G-06) y la privacidad (G-11) (interfaz.md v1.0, aprobada el 20/10). Desde la 0.4.2, Ajustes empieza con el grupo «Idioma · Language» (G-12). Tiene también «Al fallar» en Adivinar (J-13, 0.5.1) y «Notas alteradas», ♯ o ♭ por tecla negra (N-06, 0.5.2).</t>
+          <t>Hoja que sube desde abajo en vertical; panel lateral en horizontal y en pantallas amplias, con un segundo botón en el raíl (0.3.0). Es un diálogo: mientras está abierto, el resto de la página no responde (AT-04). Validado en la Sesión 1 (20/10, informe V-08): A19 y C05.</t>
         </is>
       </c>
       <c r="P103" s="6" t="n"/>
       <c r="Q103" s="5" t="inlineStr"/>
     </row>
-    <row r="104" ht="78" customHeight="1">
+    <row r="104" ht="120" customHeight="1">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>C-03</t>
+          <t>C-02</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
@@ -8434,7 +8446,7 @@
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>Los ajustes frecuentes tienen acceso rápido sin abrir el menú.</t>
+          <t>El menú contiene nomenclatura, pentagrama, timbre, numeración de trastes (tres modos), ver todas las notas, señalar iguales y afinación activa, y muestra la versión de la app.</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
@@ -8459,12 +8471,12 @@
       </c>
       <c r="H104" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>I</t>
         </is>
       </c>
       <c r="I104" s="5" t="inlineStr">
         <is>
-          <t>Nomenclatura, pentagrama y pistas tienen chips de acceso rápido.</t>
+          <t>El panel contiene todos los ajustes listados, el idioma (0.4.2) y la versión de la app.</t>
         </is>
       </c>
       <c r="J104" s="5" t="inlineStr">
@@ -8479,7 +8491,7 @@
       </c>
       <c r="L104" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #12 · Banco (node --test): grupo Idioma</t>
         </is>
       </c>
       <c r="M104" s="5" t="inlineStr">
@@ -8489,262 +8501,262 @@
       </c>
       <c r="N104" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Auditor de requisitos</t>
         </is>
       </c>
       <c r="O104" s="5" t="inlineStr">
         <is>
-          <t>Nomenclatura y pentagrama en chips bajo la cabecera, o en el panel en horizontal, donde el pentagrama se rotula con la clave de sol; las dos pistas del juego, en la tarjeta del reto (0.3.0).</t>
+          <t>Ampliado en 0.1.2 con la numeración en tres modos y la versión (G-10). En F6.4 se añade el grupo «Acerca de», con los créditos (G-06) y la privacidad (G-11) (interfaz.md v1.0, aprobada el 20/10). Desde la 0.4.2, Ajustes empieza con el grupo «Idioma · Language» (G-12). Tiene también «Al fallar» en Adivinar (J-13, 0.5.1) y «Notas alteradas», ♯ o ♭ por tecla negra (N-06, 0.5.2).</t>
         </is>
       </c>
       <c r="P104" s="6" t="n"/>
       <c r="Q104" s="5" t="inlineStr"/>
     </row>
-    <row r="105" ht="120" customHeight="1">
+    <row r="105" ht="78" customHeight="1">
       <c r="A105" s="4" t="inlineStr">
         <is>
+          <t>C-03</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Configuración y navegación</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Los ajustes frecuentes tienen acceso rápido sin abrir el menú.</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>Cliente · listado 14/09</t>
+        </is>
+      </c>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>F1.1</t>
+        </is>
+      </c>
+      <c r="H105" s="5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I105" s="5" t="inlineStr">
+        <is>
+          <t>Nomenclatura, pentagrama y pistas tienen chips de acceso rápido.</t>
+        </is>
+      </c>
+      <c r="J105" s="5" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="K105" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="L105" s="5" t="inlineStr">
+        <is>
+          <t>F1.1 #14</t>
+        </is>
+      </c>
+      <c r="M105" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="N105" s="5" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="O105" s="5" t="inlineStr">
+        <is>
+          <t>Nomenclatura y pentagrama en chips bajo la cabecera, o en el panel en horizontal, donde el pentagrama se rotula con la clave de sol; las dos pistas del juego, en la tarjeta del reto (0.3.0).</t>
+        </is>
+      </c>
+      <c r="P105" s="6" t="n"/>
+      <c r="Q105" s="5" t="inlineStr"/>
+    </row>
+    <row r="106" ht="120" customHeight="1">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
           <t>C-04</t>
         </is>
       </c>
-      <c r="B105" s="5" t="inlineStr">
+      <c r="B106" s="5" t="inlineStr">
         <is>
           <t>Configuración y navegación</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
+      <c r="C106" s="5" t="inlineStr">
         <is>
           <t>Navegación principal clara entre las áreas de la app.</t>
         </is>
       </c>
-      <c r="D105" s="5" t="inlineStr">
+      <c r="D106" s="5" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="E105" s="5" t="inlineStr">
+      <c r="E106" s="5" t="inlineStr">
         <is>
           <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
-      <c r="F105" s="5" t="inlineStr">
+      <c r="F106" s="5" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="G105" s="5" t="inlineStr">
+      <c r="G106" s="5" t="inlineStr">
         <is>
           <t>F1.1</t>
         </is>
       </c>
-      <c r="H105" s="5" t="inlineStr">
+      <c r="H106" s="5" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="I105" s="5" t="inlineStr">
+      <c r="I106" s="5" t="inlineStr">
         <is>
           <t>La navegación (barra inferior, raíl o pestañas en la cabecera, según la disposición) lleva a cada área con un toque.</t>
         </is>
       </c>
-      <c r="J105" s="5" t="inlineStr">
+      <c r="J106" s="5" t="inlineStr">
         <is>
           <t>Cumple</t>
         </is>
       </c>
-      <c r="K105" s="5" t="inlineStr">
+      <c r="K106" s="5" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="L105" s="5" t="inlineStr">
+      <c r="L106" s="5" t="inlineStr">
         <is>
           <t>F1.1 #14 · Sesión 1: A19</t>
         </is>
       </c>
-      <c r="M105" s="5" t="inlineStr">
+      <c r="M106" s="5" t="inlineStr">
         <is>
           <t>Verificado</t>
         </is>
       </c>
-      <c r="N105" s="5" t="inlineStr">
+      <c r="N106" s="5" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O105" s="5" t="inlineStr">
-        <is>
-          <t>Barra inferior con un destino por área en vertical (cinco desde la 0.5.4, con Metrónomo; seis con Acordes; en el raíl, pestañas de 44 px), raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05). Validado en la Sesión 1 (20/10, informe V-08): A19.</t>
-        </is>
-      </c>
-      <c r="P105" s="6" t="n"/>
-      <c r="Q105" s="5" t="inlineStr">
+      <c r="O106" s="5" t="inlineStr">
+        <is>
+          <t>Barra inferior con un destino por área en vertical (seis desde la 0.5.5, con Metrónomo y Acordes; en el raíl, pestañas de 44 px; entre 600 y 959 px, las pestañas se alinean a la derecha), raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05). Validado en la Sesión 1 (20/10, informe V-08): A19.</t>
+        </is>
+      </c>
+      <c r="P106" s="6" t="n"/>
+      <c r="Q106" s="5" t="inlineStr">
         <is>
           <t>Modificado</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="48" customHeight="1">
-      <c r="A106" s="4" t="inlineStr">
+    <row r="107" ht="48" customHeight="1">
+      <c r="A107" s="4" t="inlineStr">
         <is>
           <t>C-05</t>
         </is>
       </c>
-      <c r="B106" s="5" t="inlineStr">
+      <c r="B107" s="5" t="inlineStr">
         <is>
           <t>Configuración y navegación</t>
         </is>
       </c>
-      <c r="C106" s="5" t="inlineStr">
+      <c r="C107" s="5" t="inlineStr">
         <is>
           <t>Todos los ajustes persisten entre sesiones.</t>
         </is>
       </c>
-      <c r="D106" s="5" t="inlineStr">
+      <c r="D107" s="5" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="E106" s="5" t="inlineStr">
+      <c r="E107" s="5" t="inlineStr">
         <is>
           <t>Cliente · listado 14/09</t>
         </is>
       </c>
-      <c r="F106" s="5" t="inlineStr">
+      <c r="F107" s="5" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="G106" s="5" t="inlineStr">
+      <c r="G107" s="5" t="inlineStr">
         <is>
           <t>F1.1</t>
         </is>
       </c>
-      <c r="H106" s="5" t="inlineStr">
+      <c r="H107" s="5" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="I106" s="5" t="inlineStr">
+      <c r="I107" s="5" t="inlineStr">
         <is>
           <t>Todos los ajustes persisten tras recargar, y unos ajustes corruptos o antiguos no rompen la app.</t>
         </is>
       </c>
-      <c r="J106" s="5" t="inlineStr">
+      <c r="J107" s="5" t="inlineStr">
         <is>
           <t>Cumple</t>
         </is>
       </c>
-      <c r="K106" s="5" t="inlineStr">
+      <c r="K107" s="5" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="L106" s="5" t="inlineStr">
+      <c r="L107" s="5" t="inlineStr">
         <is>
           <t>Banco (node --test): migración · F1.1 #13 · Sesión 1: A14 y A15</t>
         </is>
       </c>
-      <c r="M106" s="5" t="inlineStr">
+      <c r="M107" s="5" t="inlineStr">
         <is>
           <t>Verificado</t>
         </is>
       </c>
-      <c r="N106" s="5" t="inlineStr">
+      <c r="N107" s="5" t="inlineStr">
         <is>
           <t>Banco automático + auditor técnico</t>
         </is>
       </c>
-      <c r="O106" s="5" t="inlineStr">
+      <c r="O107" s="5" t="inlineStr">
         <is>
           <t>Un único objeto de estado, validado campo a campo al leerlo (0.1.1). Validado en la Sesión 1 (20/10, informe V-08): A14 y A15.</t>
-        </is>
-      </c>
-      <c r="P106" s="6" t="n"/>
-      <c r="Q106" s="5" t="inlineStr"/>
-    </row>
-    <row r="107" ht="93" customHeight="1">
-      <c r="A107" s="4" t="inlineStr">
-        <is>
-          <t>C-06</t>
-        </is>
-      </c>
-      <c r="B107" s="5" t="inlineStr">
-        <is>
-          <t>Configuración y navegación</t>
-        </is>
-      </c>
-      <c r="C107" s="5" t="inlineStr">
-        <is>
-          <t>Especificación detallada de la interfaz: estructura de menús, jerarquía de controles y flujos de navegación.</t>
-        </is>
-      </c>
-      <c r="D107" s="5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="E107" s="5" t="inlineStr">
-        <is>
-          <t>Cliente · listado 14/09</t>
-        </is>
-      </c>
-      <c r="F107" s="5" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="G107" s="5" t="inlineStr">
-        <is>
-          <t>F3.1</t>
-        </is>
-      </c>
-      <c r="H107" s="5" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I107" s="5" t="inlineStr">
-        <is>
-          <t>interfaz.md aprobado por el cliente y revisado por el auditor de requisitos.</t>
-        </is>
-      </c>
-      <c r="J107" s="5" t="inlineStr">
-        <is>
-          <t>Cumple</t>
-        </is>
-      </c>
-      <c r="K107" s="5" t="inlineStr">
-        <is>
-          <t>0.2.3</t>
-        </is>
-      </c>
-      <c r="L107" s="5" t="inlineStr">
-        <is>
-          <t>interfaz.md v1.0 · AR-04 · aprobación del cliente el 20/10</t>
-        </is>
-      </c>
-      <c r="M107" s="5" t="inlineStr">
-        <is>
-          <t>Verificado</t>
-        </is>
-      </c>
-      <c r="N107" s="5" t="inlineStr">
-        <is>
-          <t>Auditor de requisitos</t>
-        </is>
-      </c>
-      <c r="O107" s="5" t="inlineStr">
-        <is>
-          <t>docs/interfaz.md v1.0, aprobada por ti el 20/10 tras la auditoría AR-04 (10 hallazgos resueltos). Bocetos al tamaño real de cada pantalla en docs/interfaz/, comprobados por herramientas/capturar-wireframes.js. Los cambios posteriores suben su versión.</t>
         </is>
       </c>
       <c r="P107" s="6" t="n"/>
       <c r="Q107" s="5" t="inlineStr"/>
     </row>
-    <row r="108" ht="120" customHeight="1">
+    <row r="108" ht="93" customHeight="1">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>C-07</t>
+          <t>C-06</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
@@ -8754,17 +8766,17 @@
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>Botón «atrás» del sistema: mientras haya un paso anterior en la sesión, el botón o gesto «atrás» cierra Ajustes o vuelve al área anterior; desde la primera área actúa el sistema. Al abrir la app se entra en Libre.</t>
+          <t>Especificación detallada de la interfaz: estructura de menús, jerarquía de controles y flujos de navegación.</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
+          <t>Cliente · listado 14/09</t>
         </is>
       </c>
       <c r="F108" s="5" t="inlineStr">
@@ -8774,17 +8786,17 @@
       </c>
       <c r="G108" s="5" t="inlineStr">
         <is>
-          <t>F3.2</t>
+          <t>F3.1</t>
         </is>
       </c>
       <c r="H108" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>I</t>
         </is>
       </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>Con un paso anterior en la sesión, «atrás» cierra Ajustes o vuelve al área anterior; desde la primera área actúa el sistema; al abrir o recargar se entra en Libre. Prueba manual en Windows y en el simulador de Android de Chrome.</t>
+          <t>interfaz.md aprobado por el cliente y revisado por el auditor de requisitos.</t>
         </is>
       </c>
       <c r="J108" s="5" t="inlineStr">
@@ -8794,12 +8806,12 @@
       </c>
       <c r="K108" s="5" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="L108" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): historial simulado con popstate (3 pruebas) · Sesión 1: A17</t>
+          <t>interfaz.md v1.0 · AR-04 · aprobación del cliente el 20/10</t>
         </is>
       </c>
       <c r="M108" s="5" t="inlineStr">
@@ -8809,21 +8821,21 @@
       </c>
       <c r="N108" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Auditor de requisitos</t>
         </is>
       </c>
       <c r="O108" s="5" t="inlineStr">
         <is>
-          <t>Hecho en la 0.3.0 con el historial del navegador (history): cada área tiene su dirección (#libre, #adivinar…). Un paso que deja la misma área, como tras recargar, se salta. El banco lo prueba con un historial simulado que avisa como el de verdad. Falta la prueba a mano en Windows y en el simulador de Android (Sesión 1). En el iPhone instalado no hay botón atrás. Validado en la Sesión 1 (20/10, informe V-08): A17.</t>
+          <t>docs/interfaz.md v1.0, aprobada por ti el 20/10 tras la auditoría AR-04 (10 hallazgos resueltos). Bocetos al tamaño real de cada pantalla en docs/interfaz/, comprobados por herramientas/capturar-wireframes.js. Los cambios posteriores suben su versión.</t>
         </is>
       </c>
       <c r="P108" s="6" t="n"/>
       <c r="Q108" s="5" t="inlineStr"/>
     </row>
-    <row r="109" ht="93" customHeight="1">
+    <row r="109" ht="120" customHeight="1">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>C-08</t>
+          <t>C-07</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
@@ -8833,7 +8845,7 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Menú Personalización dentro de Ajustes: estilos de nota en el mástil (círculo de color o solo el nombre, más grande o en negrita), estilo del traste y del mástil, interior claro para «Ver todas las notas» y temas de color de la app.</t>
+          <t>Botón «atrás» del sistema: mientras haya un paso anterior en la sesión, el botón o gesto «atrás» cierra Ajustes o vuelve al área anterior; desde la primera área actúa el sistema. Al abrir la app se entra en Libre.</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
@@ -8843,145 +8855,145 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>F3.2</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>Fuera del alcance actual.</t>
+          <t>Con un paso anterior en la sesión, «atrás» cierra Ajustes o vuelve al área anterior; desde la primera área actúa el sistema; al abrir o recargar se entra en Libre. Prueba manual en Windows y en el simulador de Android de Chrome.</t>
         </is>
       </c>
       <c r="J109" s="5" t="inlineStr">
         <is>
-          <t>No aplica</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K109" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="L109" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): historial simulado con popstate (3 pruebas) · Sesión 1: A17</t>
         </is>
       </c>
       <c r="M109" s="5" t="inlineStr">
         <is>
-          <t>No aplica</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N109" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="O109" s="5" t="inlineStr">
         <is>
-          <t>Tus comentarios de la Sesión 1 (A10, C06 y E06), para una actualización posterior. La paleta por nota de G-05 se mantiene como punto de partida.</t>
+          <t>Hecho en la 0.3.0 con el historial del navegador (history): cada área tiene su dirección (#libre, #adivinar…). Un paso que deja la misma área, como tras recargar, se salta. El banco lo prueba con un historial simulado que avisa como el de verdad. Falta la prueba a mano en Windows y en el simulador de Android (Sesión 1). En el iPhone instalado no hay botón atrás. Validado en la Sesión 1 (20/10, informe V-08): A17.</t>
         </is>
       </c>
       <c r="P109" s="6" t="n"/>
       <c r="Q109" s="5" t="inlineStr"/>
     </row>
-    <row r="110" ht="78" customHeight="1">
+    <row r="110" ht="93" customHeight="1">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>X-01</t>
+          <t>C-08</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>Respaldo y publicación</t>
+          <t>Configuración y navegación</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>El código y la documentación están respaldados en el repositorio remoto (GitHub). Respaldar no es publicar.</t>
+          <t>Menú Personalización dentro de Ajustes: estilos de nota en el mástil (círculo de color o solo el nombre, más grande o en negrita), estilo del traste y del mástil, interior claro para «Ver todas las notas» y temas de color de la app.</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>Desarrollo · v1.1</t>
+          <t>Cliente · listado 14/09</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>Posterior</t>
         </is>
       </c>
       <c r="G110" s="5" t="inlineStr">
         <is>
-          <t>F1.2 · F1.4</t>
+          <t>Posterior</t>
         </is>
       </c>
       <c r="H110" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>GitHub muestra la última versión en main, entrada por pull request aprobado, y la etiqueta de cierre de fase.</t>
+          <t>Fuera del alcance actual.</t>
         </is>
       </c>
       <c r="J110" s="5" t="inlineStr">
         <is>
-          <t>Cumple</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="K110" s="5" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L110" s="5" t="inlineStr">
         <is>
-          <t>PR #1 a #5 fusionados · etiqueta v0.1.5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M110" s="5" t="inlineStr">
         <is>
-          <t>Verificado parcialmente</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="N110" s="5" t="inlineStr">
         <is>
-          <t>Auditor de requisitos</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O110" s="5" t="inlineStr">
         <is>
-          <t>Desde el 15/10 todo el proyecto está en pdigue/guitarra; cada versión entra por pull request aprobado (del #1 al #5) y F1 se cerró con la etiqueta v0.1.5. El repositorio es público.</t>
+          <t>Tus comentarios de la Sesión 1 (A10, C06 y E06), para una actualización posterior. La paleta por nota de G-05 se mantiene como punto de partida.</t>
         </is>
       </c>
       <c r="P110" s="6" t="n"/>
       <c r="Q110" s="5" t="inlineStr"/>
     </row>
-    <row r="111" ht="120" customHeight="1">
+    <row r="111" ht="78" customHeight="1">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>X-02</t>
+          <t>X-01</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
@@ -8991,7 +9003,7 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>La app está publicada en una URL pública (GitHub Pages).</t>
+          <t>El código y la documentación están respaldados en el repositorio remoto (GitHub). Respaldar no es publicar.</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
@@ -9006,61 +9018,61 @@
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>F7</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>F7.1</t>
+          <t>F1.2 · F1.4</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>I</t>
         </is>
       </c>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>La URL pública carga la app desde un dispositivo ajeno al proyecto.</t>
+          <t>GitHub muestra la última versión en main, entrada por pull request aprobado, y la etiqueta de cierre de fase.</t>
         </is>
       </c>
       <c r="J111" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K111" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.1.4</t>
         </is>
       </c>
       <c r="L111" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PR #1 a #5 fusionados · etiqueta v0.1.5</t>
         </is>
       </c>
       <c r="M111" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N111" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Auditor de requisitos</t>
         </is>
       </c>
       <c r="O111" s="5" t="inlineStr">
         <is>
-          <t>Antes en V1; pasa a la última fase por decisión del 15/09: desarrollo local de principio a fin. Despliegue de pruebas (decisión del 15/10): antes de la Sesión 1 se publica una versión de pruebas en GitHub Pages, sin anunciar, para probar en el iPhone con https la instalación, el modo sin conexión y el micrófono. X-02 sigue siendo la publicación oficial.</t>
+          <t>Desde el 15/10 todo el proyecto está en pdigue/guitarra; cada versión entra por pull request aprobado (del #1 al #5) y F1 se cerró con la etiqueta v0.1.5. El repositorio es público.</t>
         </is>
       </c>
       <c r="P111" s="6" t="n"/>
       <c r="Q111" s="5" t="inlineStr"/>
     </row>
-    <row r="112" ht="33" customHeight="1">
+    <row r="112" ht="120" customHeight="1">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>X-03</t>
+          <t>X-02</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
@@ -9070,7 +9082,7 @@
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>La app está verificada en móviles reales, instalada como icono desde la web publicada.</t>
+          <t>La app está publicada en una URL pública (GitHub Pages).</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
@@ -9090,7 +9102,7 @@
       </c>
       <c r="G112" s="5" t="inlineStr">
         <is>
-          <t>F7.2</t>
+          <t>F7.1</t>
         </is>
       </c>
       <c r="H112" s="5" t="inlineStr">
@@ -9100,7 +9112,7 @@
       </c>
       <c r="I112" s="5" t="inlineStr">
         <is>
-          <t>La app instalada desde la web funciona en un Android, un iPhone y un Windows reales.</t>
+          <t>La URL pública carga la app desde un dispositivo ajeno al proyecto.</t>
         </is>
       </c>
       <c r="J112" s="5" t="inlineStr">
@@ -9130,15 +9142,94 @@
       </c>
       <c r="O112" s="5" t="inlineStr">
         <is>
-          <t>Cierra G-04 y PL-01 a PL-03 en su modo web.</t>
+          <t>Antes en V1; pasa a la última fase por decisión del 15/09: desarrollo local de principio a fin. Despliegue de pruebas (decisión del 15/10): antes de la Sesión 1 se publica una versión de pruebas en GitHub Pages, sin anunciar, para probar en el iPhone con https la instalación, el modo sin conexión y el micrófono. X-02 sigue siendo la publicación oficial.</t>
         </is>
       </c>
       <c r="P112" s="6" t="n"/>
       <c r="Q112" s="5" t="inlineStr"/>
     </row>
+    <row r="113" ht="33" customHeight="1">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>X-03</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Respaldo y publicación</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>La app está verificada en móviles reales, instalada como icono desde la web publicada.</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>Desarrollo · v1.1</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>F7.2</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I113" s="5" t="inlineStr">
+        <is>
+          <t>La app instalada desde la web funciona en un Android, un iPhone y un Windows reales.</t>
+        </is>
+      </c>
+      <c r="J113" s="5" t="inlineStr">
+        <is>
+          <t>No cumple</t>
+        </is>
+      </c>
+      <c r="K113" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L113" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M113" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="N113" s="5" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="O113" s="5" t="inlineStr">
+        <is>
+          <t>Cierra G-04 y PL-01 a PL-03 en su modo web.</t>
+        </is>
+      </c>
+      <c r="P113" s="6" t="n"/>
+      <c r="Q113" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q112"/>
-  <conditionalFormatting sqref="J5:J112">
+  <autoFilter ref="A4:Q113"/>
+  <conditionalFormatting sqref="J5:J113">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>J5="Cumple"</formula>
     </cfRule>
@@ -9155,7 +9246,7 @@
       <formula>J5="No aplica"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M112">
+  <conditionalFormatting sqref="M5:M113">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>M5="Cumple"</formula>
     </cfRule>
@@ -9173,13 +9264,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="J5:J112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
+    <dataValidation sqref="J5:J113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
       <formula1>"Cumple,Cumple parcialmente,No cumple,No aplica"</formula1>
     </dataValidation>
-    <dataValidation sqref="M5:M112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
+    <dataValidation sqref="M5:M113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
       <formula1>"Verificado,Verificado parcialmente,Pendiente,No aplica"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
+    <dataValidation sqref="H5:H113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
       <formula1>"I,A,D,T,I+T,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9275,23 +9366,23 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$112,"*F1*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$113,"*F1*")</f>
         <v/>
       </c>
       <c r="C5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F1*",Matriz!$J$5:$J$112,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$J$5:$J$113,"Cumple")</f>
         <v/>
       </c>
       <c r="D5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F1*",Matriz!$J$5:$J$112,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F1*",Matriz!$J$5:$J$112,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$J$5:$J$113,"No cumple")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F1*",Matriz!$J$5:$J$112,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$J$5:$J$113,"No aplica")</f>
         <v/>
       </c>
       <c r="G5" s="8">
@@ -9299,11 +9390,11 @@
         <v/>
       </c>
       <c r="H5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F1*",Matriz!$M$5:$M$112,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$M$5:$M$113,"Verificado")</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F1*",Matriz!$M$5:$M$112,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9314,23 +9405,23 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$112,"*F2*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$113,"*F2*")</f>
         <v/>
       </c>
       <c r="C6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F2*",Matriz!$J$5:$J$112,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$J$5:$J$113,"Cumple")</f>
         <v/>
       </c>
       <c r="D6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F2*",Matriz!$J$5:$J$112,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F2*",Matriz!$J$5:$J$112,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$J$5:$J$113,"No cumple")</f>
         <v/>
       </c>
       <c r="F6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F2*",Matriz!$J$5:$J$112,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$J$5:$J$113,"No aplica")</f>
         <v/>
       </c>
       <c r="G6" s="8">
@@ -9338,11 +9429,11 @@
         <v/>
       </c>
       <c r="H6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F2*",Matriz!$M$5:$M$112,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$M$5:$M$113,"Verificado")</f>
         <v/>
       </c>
       <c r="I6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F2*",Matriz!$M$5:$M$112,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9353,23 +9444,23 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$112,"*F3*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$113,"*F3*")</f>
         <v/>
       </c>
       <c r="C7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F3*",Matriz!$J$5:$J$112,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$J$5:$J$113,"Cumple")</f>
         <v/>
       </c>
       <c r="D7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F3*",Matriz!$J$5:$J$112,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F3*",Matriz!$J$5:$J$112,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$J$5:$J$113,"No cumple")</f>
         <v/>
       </c>
       <c r="F7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F3*",Matriz!$J$5:$J$112,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$J$5:$J$113,"No aplica")</f>
         <v/>
       </c>
       <c r="G7" s="8">
@@ -9377,11 +9468,11 @@
         <v/>
       </c>
       <c r="H7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F3*",Matriz!$M$5:$M$112,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$M$5:$M$113,"Verificado")</f>
         <v/>
       </c>
       <c r="I7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F3*",Matriz!$M$5:$M$112,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9392,23 +9483,23 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$112,"*F4*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$113,"*F4*")</f>
         <v/>
       </c>
       <c r="C8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F4*",Matriz!$J$5:$J$112,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$J$5:$J$113,"Cumple")</f>
         <v/>
       </c>
       <c r="D8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F4*",Matriz!$J$5:$J$112,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F4*",Matriz!$J$5:$J$112,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$J$5:$J$113,"No cumple")</f>
         <v/>
       </c>
       <c r="F8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F4*",Matriz!$J$5:$J$112,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$J$5:$J$113,"No aplica")</f>
         <v/>
       </c>
       <c r="G8" s="8">
@@ -9416,11 +9507,11 @@
         <v/>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F4*",Matriz!$M$5:$M$112,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$M$5:$M$113,"Verificado")</f>
         <v/>
       </c>
       <c r="I8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F4*",Matriz!$M$5:$M$112,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9431,23 +9522,23 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$112,"*F5*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$113,"*F5*")</f>
         <v/>
       </c>
       <c r="C9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F5*",Matriz!$J$5:$J$112,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$J$5:$J$113,"Cumple")</f>
         <v/>
       </c>
       <c r="D9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F5*",Matriz!$J$5:$J$112,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F5*",Matriz!$J$5:$J$112,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$J$5:$J$113,"No cumple")</f>
         <v/>
       </c>
       <c r="F9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F5*",Matriz!$J$5:$J$112,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$J$5:$J$113,"No aplica")</f>
         <v/>
       </c>
       <c r="G9" s="8">
@@ -9455,11 +9546,11 @@
         <v/>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F5*",Matriz!$M$5:$M$112,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$M$5:$M$113,"Verificado")</f>
         <v/>
       </c>
       <c r="I9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F5*",Matriz!$M$5:$M$112,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9470,23 +9561,23 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$112,"*F6*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$113,"*F6*")</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F6*",Matriz!$J$5:$J$112,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$J$5:$J$113,"Cumple")</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F6*",Matriz!$J$5:$J$112,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F6*",Matriz!$J$5:$J$112,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$J$5:$J$113,"No cumple")</f>
         <v/>
       </c>
       <c r="F10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F6*",Matriz!$J$5:$J$112,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$J$5:$J$113,"No aplica")</f>
         <v/>
       </c>
       <c r="G10" s="8">
@@ -9494,11 +9585,11 @@
         <v/>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F6*",Matriz!$M$5:$M$112,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$M$5:$M$113,"Verificado")</f>
         <v/>
       </c>
       <c r="I10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F6*",Matriz!$M$5:$M$112,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9509,23 +9600,23 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$112,"*F7*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$113,"*F7*")</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F7*",Matriz!$J$5:$J$112,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$J$5:$J$113,"Cumple")</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F7*",Matriz!$J$5:$J$112,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F7*",Matriz!$J$5:$J$112,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$J$5:$J$113,"No cumple")</f>
         <v/>
       </c>
       <c r="F11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F7*",Matriz!$J$5:$J$112,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$J$5:$J$113,"No aplica")</f>
         <v/>
       </c>
       <c r="G11" s="8">
@@ -9533,11 +9624,11 @@
         <v/>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F7*",Matriz!$M$5:$M$112,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$M$5:$M$113,"Verificado")</f>
         <v/>
       </c>
       <c r="I11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*F7*",Matriz!$M$5:$M$112,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9548,23 +9639,23 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$112,"*Posterior*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$113,"*Posterior*")</f>
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*Posterior*",Matriz!$J$5:$J$112,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$J$5:$J$113,"Cumple")</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*Posterior*",Matriz!$J$5:$J$112,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*Posterior*",Matriz!$J$5:$J$112,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$J$5:$J$113,"No cumple")</f>
         <v/>
       </c>
       <c r="F12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*Posterior*",Matriz!$J$5:$J$112,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$J$5:$J$113,"No aplica")</f>
         <v/>
       </c>
       <c r="G12" s="8">
@@ -9572,11 +9663,11 @@
         <v/>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*Posterior*",Matriz!$M$5:$M$112,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$M$5:$M$113,"Verificado")</f>
         <v/>
       </c>
       <c r="I12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$112,"*Posterior*",Matriz!$M$5:$M$112,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9587,23 +9678,23 @@
         </is>
       </c>
       <c r="B13" s="9">
-        <f>COUNTA(Matriz!$A$5:$A$112)</f>
+        <f>COUNTA(Matriz!$A$5:$A$113)</f>
         <v/>
       </c>
       <c r="C13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$112,"Cumple")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$113,"Cumple")</f>
         <v/>
       </c>
       <c r="D13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$112,"Cumple parcialmente")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$112,"No cumple")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$113,"No cumple")</f>
         <v/>
       </c>
       <c r="F13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$112,"No aplica")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$113,"No aplica")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -9611,11 +9702,11 @@
         <v/>
       </c>
       <c r="H13" s="9">
-        <f>COUNTIF(Matriz!$M$5:$M$112,"Verificado")</f>
+        <f>COUNTIF(Matriz!$M$5:$M$113,"Verificado")</f>
         <v/>
       </c>
       <c r="I13" s="9">
-        <f>COUNTIF(Matriz!$M$5:$M$112,"Verificado parcialmente")</f>
+        <f>COUNTIF(Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9633,7 +9724,7 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$112,"I")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$113,"I")</f>
         <v/>
       </c>
     </row>
@@ -9644,7 +9735,7 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$112,"A")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$113,"A")</f>
         <v/>
       </c>
     </row>
@@ -9655,7 +9746,7 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$112,"D")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$113,"D")</f>
         <v/>
       </c>
     </row>
@@ -9666,7 +9757,7 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$112,"T")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$113,"T")</f>
         <v/>
       </c>
     </row>
@@ -9677,7 +9768,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$112,"I+T")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$113,"I+T")</f>
         <v/>
       </c>
     </row>
@@ -9688,7 +9779,7 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$112,"N/A")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$113,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -9865,7 +9956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9905,7 +9996,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -9915,24 +10006,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.5.4</t>
+          <t>0.5.5</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
+          <t>AC-01 a AC-05 implementados y verificados por el banco (F5.7); AC-06 nuevo, el buscador; criterios al día con tu guía del listado.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -9942,24 +10033,24 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.5.3</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
+          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -9969,24 +10060,24 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.5.2</t>
+          <t>0.5.3</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
+          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -9996,24 +10087,24 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.5.0</t>
+          <t>0.5.2</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
+          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -10023,24 +10114,24 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.4.2</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
+          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -10050,51 +10141,51 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.4.0</t>
+          <t>0.4.2</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
+          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.3.3</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
+          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -10104,24 +10195,24 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>0.3.2</t>
+          <t>0.3.3</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
+          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -10131,24 +10222,24 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>0.3.1</t>
+          <t>0.3.2</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
+          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -10158,24 +10249,24 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -10185,24 +10276,24 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -10212,7 +10303,7 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -10222,14 +10313,14 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -10239,7 +10330,7 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
@@ -10249,24 +10340,24 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
@@ -10276,14 +10367,14 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -10293,24 +10384,24 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -10320,24 +10411,24 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -10347,51 +10438,51 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -10401,7 +10492,7 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
@@ -10411,32 +10502,59 @@
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="46" customHeight="1">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
0.5.6: correcciones de AT-10 y AR-11, y continuidad entre conversaciones (MT-02 a MT-05, AC-03, AC-06)
- Metrónomo: cambiar de compás sonando no mueve el pulso; golpes atrasados
  que se saltan; figuras según el pulso (3/8, 5/8, 7/8 y compuestos); foco
  del teclado; aviso traducido; parada con aviso si el sistema detiene el audio.
- Acordes: alteraciones del pentagrama en dos columnas; Restablecer limpia
  el buscador.
- Documentos: requisitos v1.23, matriz v1.21, roadmap v3.21, interfaz v1.13,
  compatibilidad, IT-03; informes AR-11 y AT-10.
- Continuidad: docs/ESTADO.md, los generadores de requisitos y matriz en
  herramientas/documentos/, y reglas de ahorro de uso en CLAUDE.md.
- Banco 79 de 79.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNqYPth87waeVp6tJXcZMT
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.20. Base: requisitos.md v1.22 · app 0.5.5 · roadmap 3.20 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.21. Base: requisitos.md v1.23 · app 0.5.6 · roadmap 3.21 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.19</t>
+          <t>Cambio en v1.21</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>La app se organiza en áreas accesibles desde una navegación principal: Libre, Adivinar, Afinador y Escalas. Cada área nueva (Metrónomo y Acordes, en F5) se suma a esa navegación.</t>
+          <t>La app se organiza en áreas accesibles desde una navegación principal: Libre, Adivinar, Afinador, Escalas, Acordes y Metrónomo.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>La barra inferior muestra Libre, Adivinar, Afinador y Escalas; cada destino activo abre su vista y cada área nueva (Metrónomo, Acordes) suma su destino.</t>
+          <t>La navegación muestra las seis áreas (Libre, Adivinar, Afinador, Escalas, Acordes y Metrónomo) y cada destino abre su vista.</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #1 y #14 · Sesión 1 A12 · Sesión 1: A12</t>
+          <t>F1.1 #1 y #14 · 0.5.5: comprobar-disposicion, seis pestañas en todas las pantallas · Sesión 1: A12</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="L83" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): barra con teclado, − y +, «Marcar» (media y reinicio tras 2 s), límites y nombre del tempo · comprobar-disposicion: cinco pantallas</t>
+          <t>Banco (node --test): barra con teclado, − y +, «Marcar» (media y reinicio tras 2 s), límites, nombre del tempo, Empezar y Parar · comprobar-disposicion: cinco pantallas</t>
         </is>
       </c>
       <c r="M83" s="5" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>El metrónomo es un área propia, con su pestaña en la navegación principal. Sigue sonando al pasar a Libre, Adivinar, Escalas o Acordes hasta que lo pares, y su pestaña late con el pulso mientras suena. Recuerda el último tempo, compás, acentos y subdivisión.</t>
+          <t>El metrónomo es un área propia, con su pestaña en la navegación principal. Sigue sonando al pasar a Libre, Adivinar, Escalas o Acordes hasta que lo pares, y su pestaña late con el pulso mientras suena. Recuerda el último tempo, compás, figura y acento en el primer tiempo.</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="L87" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): sigue en Libre, pestaña que late, parada con el micrófono y aviso, datos guardados</t>
+          <t>Banco (node --test): sigue en Libre y en el Afinador hasta escuchar con el micrófono, pestaña que late, parada con el micrófono y aviso, datos guardados</t>
         </is>
       </c>
       <c r="M87" s="5" t="inlineStr">
@@ -7159,7 +7159,11 @@
         </is>
       </c>
       <c r="P87" s="6" t="n"/>
-      <c r="Q87" s="5" t="inlineStr"/>
+      <c r="Q87" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="120" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
@@ -7204,7 +7208,7 @@
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>El listado tiene populares arriba y los 30 acordes debajo; cada digitación suena solo a notas del acorde, con la raíz, la tercera y la séptima (la quinta se puede omitir) y la raíz o el bajo indicado como nota más grave.</t>
+          <t>A un lado el listado (populares arriba, los 30 acordes debajo) y al otro el mástil; cada digitación suena solo a notas del acorde, con la raíz, la nota que define el tipo (la tercera, o la cuarta en sus4) y la séptima si la lleva (la quinta se puede omitir), y con la raíz o el bajo indicado como nota más grave.</t>
         </is>
       </c>
       <c r="J88" s="5" t="inlineStr">
@@ -7219,7 +7223,7 @@
       </c>
       <c r="L88" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): las 30 digitaciones, una a una; populares y listado</t>
+          <t>Banco (node --test): las 30 digitaciones, una a una; populares y listado · comprobar-disposicion: listado y mástil a la vez en seis pantallas</t>
         </is>
       </c>
       <c r="M88" s="5" t="inlineStr">
@@ -7238,11 +7242,7 @@
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
-      <c r="Q88" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q88" s="5" t="inlineStr"/>
     </row>
     <row r="89" ht="120" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
@@ -7321,11 +7321,7 @@
         </is>
       </c>
       <c r="P89" s="6" t="n"/>
-      <c r="Q89" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q89" s="5" t="inlineStr"/>
     </row>
     <row r="90" ht="93" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
@@ -7385,7 +7381,7 @@
       </c>
       <c r="L90" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): cinco notas de La menor; B7 con Re♯ · comprobar-disposicion: seis pantallas</t>
+          <t>Banco (node --test): cinco notas de La menor; B7 con Re♯ · el ajuste de pentagrama de siempre (F1.1) · comprobar-disposicion: seis pantallas</t>
         </is>
       </c>
       <c r="M90" s="5" t="inlineStr">
@@ -7404,11 +7400,7 @@
         </is>
       </c>
       <c r="P90" s="6" t="n"/>
-      <c r="Q90" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q90" s="5" t="inlineStr"/>
     </row>
     <row r="91" ht="48" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
@@ -7448,7 +7440,7 @@
       </c>
       <c r="H91" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T</t>
         </is>
       </c>
       <c r="I91" s="5" t="inlineStr">
@@ -7468,7 +7460,7 @@
       </c>
       <c r="L91" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): orden del rasgueo</t>
+          <t>Banco (node --test): orden del rasgueo · cada casilla suena suelta como en todo el mástil (F1.1 #2)</t>
         </is>
       </c>
       <c r="M91" s="5" t="inlineStr">
@@ -7478,7 +7470,7 @@
       </c>
       <c r="N91" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Banco automático + auditor técnico</t>
         </is>
       </c>
       <c r="O91" s="5" t="inlineStr">
@@ -7487,11 +7479,7 @@
         </is>
       </c>
       <c r="P91" s="6" t="n"/>
-      <c r="Q91" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q91" s="5" t="inlineStr"/>
     </row>
     <row r="92" ht="63" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
@@ -7570,13 +7558,9 @@
         </is>
       </c>
       <c r="P92" s="6" t="n"/>
-      <c r="Q92" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="93" customHeight="1">
+      <c r="Q92" s="5" t="inlineStr"/>
+    </row>
+    <row r="93" ht="78" customHeight="1">
       <c r="A93" s="4" t="inlineStr">
         <is>
           <t>AC-06</t>
@@ -7649,13 +7633,13 @@
       </c>
       <c r="O93" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10. Una sola letra solo se busca en la nomenclatura inglesa, para que «D» no traiga también los Do; # y b valen por ♯ y ♭. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
+          <t>Tu petición del 21/10. Una sola letra solo se busca en la nomenclatura inglesa, para que «D» no traiga también los Do; # y b valen por ♯ y ♭. Hecho en la 0.5.5 y validado por el banco.</t>
         </is>
       </c>
       <c r="P93" s="6" t="n"/>
       <c r="Q93" s="5" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Modificado</t>
         </is>
       </c>
     </row>
@@ -7702,7 +7686,7 @@
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>En horizontal, con un alto útil de 268 px o más, cada cuerda mide al menos 40 px (iPhone en Safari e instalada; simulador de Android). En vertical, en pantallas táctiles de menos de 600 px de ancho y en Libre, Adivinar y Escalas, aparece el aviso para girar; nunca en el Afinador; cerrado, no vuelve y «Restablecer» lo recupera.</t>
+          <t>En horizontal, con un alto útil de 268 px o más, cada cuerda mide al menos 40 px (iPhone en Safari e instalada; simulador de Android). En vertical, en pantallas táctiles de menos de 600 px de ancho y en Libre, Adivinar, Escalas y Acordes, aparece el aviso para girar; nunca en el Afinador ni en el Metrónomo; cerrado, no vuelve y «Restablecer» lo recupera.</t>
         </is>
       </c>
       <c r="J94" s="5" t="inlineStr">
@@ -7732,11 +7716,15 @@
       </c>
       <c r="O94" s="5" t="inlineStr">
         <is>
-          <t>Hecho en la 0.3.0 según interfaz.md §7. En horizontal, raíl, mástil a todo el alto y panel: medido en Chromium, 52,8 px por cuerda en el iPhone con Safari (antes 28,8), 60,8 con la app instalada y 42,5 en un Android de 280 px de alto (V-06). El aviso para girar sale solo con el dedo, en vertical y en pantallas de menos de 600 px de ancho, en Libre y Adivinar (y Escalas desde F5), nunca en el Afinador; cerrado no vuelve y «Restablecer» lo recupera. El bloqueo de orientación tiene mal soporte en iOS, así que no se fuerza. Validado en la Sesión 1 (20/10, informe V-08): C02, C03 y D03.</t>
+          <t>Hecho en la 0.3.0 según interfaz.md §7. En horizontal, raíl, mástil a todo el alto y panel: medido en Chromium, 52,8 px por cuerda en el iPhone con Safari (antes 28,8), 60,8 con la app instalada y 42,5 en un Android de 280 px de alto (V-06). El aviso para girar sale solo con el dedo, en vertical y en pantallas de menos de 600 px de ancho, en Libre y Adivinar (y Escalas desde F5), en Libre, Adivinar, Escalas y Acordes; nunca en el Afinador ni en el Metrónomo; cerrado no vuelve y «Restablecer» lo recupera. El bloqueo de orientación tiene mal soporte en iOS, así que no se fuerza. Validado en la Sesión 1 (20/10, informe V-08): C02, C03 y D03.</t>
         </is>
       </c>
       <c r="P94" s="6" t="n"/>
-      <c r="Q94" s="5" t="inlineStr"/>
+      <c r="Q94" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="33" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
@@ -8649,7 +8637,7 @@
       </c>
       <c r="L106" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14 · Sesión 1: A19</t>
+          <t>F1.1 #14 · 0.5.5: comprobar-disposicion, seis pestañas sin salirse ni pisar el nombre · Sesión 1: A19</t>
         </is>
       </c>
       <c r="M106" s="5" t="inlineStr">
@@ -8668,11 +8656,7 @@
         </is>
       </c>
       <c r="P106" s="6" t="n"/>
-      <c r="Q106" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q106" s="5" t="inlineStr"/>
     </row>
     <row r="107" ht="48" customHeight="1">
       <c r="A107" s="4" t="inlineStr">
@@ -9956,7 +9940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9996,7 +9980,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -10006,24 +9990,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.5.5</t>
+          <t>0.5.6</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>AC-01 a AC-05 implementados y verificados por el banco (F5.7); AC-06 nuevo, el buscador; criterios al día con tu guía del listado.</t>
+          <t>Auditoría AR-11: G-02, C-04 y V-01 con las seis áreas; criterio de AC-01 preciso (sus4 y tríadas); evidencias completadas en MT-01, MT-05, AC-01, AC-03 y AC-04 (método T).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -10033,24 +10017,24 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.5.4</t>
+          <t>0.5.5</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
+          <t>AC-01 a AC-05 implementados y verificados por el banco (F5.7); AC-06 nuevo, el buscador; criterios al día con tu guía del listado.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -10060,24 +10044,24 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.5.3</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
+          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -10087,24 +10071,24 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.5.2</t>
+          <t>0.5.3</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
+          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -10114,24 +10098,24 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.5.0</t>
+          <t>0.5.2</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
+          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -10141,24 +10125,24 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.4.2</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
+          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -10168,51 +10152,51 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.4.0</t>
+          <t>0.4.2</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
+          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>0.3.3</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
+          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -10222,24 +10206,24 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>0.3.2</t>
+          <t>0.3.3</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
+          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -10249,24 +10233,24 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>0.3.1</t>
+          <t>0.3.2</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
+          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -10276,24 +10260,24 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -10303,24 +10287,24 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -10330,7 +10314,7 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
@@ -10340,14 +10324,14 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -10357,7 +10341,7 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
@@ -10367,24 +10351,24 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
@@ -10394,14 +10378,14 @@
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -10411,24 +10395,24 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -10438,24 +10422,24 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -10465,51 +10449,51 @@
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -10519,7 +10503,7 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
@@ -10529,32 +10513,59 @@
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="46" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
CP-5: arranque del metrónomo con el audio en pausa y una sola vara de verificación (0.5.7, MT-04, AR-12, AT-11)
Auditorías a fondo de toda F5 (AR-12 y AT-11), sin críticos:
- AT-11 #1 (alto): startMetro espera a que el audio despierte antes de
  programar golpes; prueba nueva con un resume() lento, como el de Safari.
- AR-12 #1 (alto): MT-01, MT-05, AC-02 y AC-03 pasan a verificados
  parcialmente hasta la Sesión 2, como los de Escalas; F5.2, F5.3, F5.6 y
  F5.7 a 🔨. Requisitos v1.24 (53 validados), matriz v1.22, roadmap v3.22.
- AR-12 #2 (alto): pantalla encendida con el metrónomo, pendiente de Pablo.
- Medios y bajos, anotados en su requisito. F5.8 aparcada (decisión del 22/10).
- CHANGELOG, IT-03 y ESTADO al día. Banco 81 de 81.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AWJcxzncaZFWFnJfpoVV8q
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.21. Base: requisitos.md v1.23 · app 0.5.6 · roadmap 3.21 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.22. Base: requisitos.md v1.24 · app 0.5.7 · roadmap 3.22 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.21</t>
+          <t>Cambio en v1.22</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       <c r="P5" s="6" t="n"/>
       <c r="Q5" s="5" t="inlineStr"/>
     </row>
-    <row r="6" ht="63" customHeight="1">
+    <row r="6" ht="108" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>G-02</t>
@@ -820,7 +820,7 @@
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>Escalas, habilitada desde la 0.5.0. Metrónomo, área propia desde la 0.5.4, y Acordes desde la 0.5.5 (tu decisión del 21/10). Validado en la Sesión 1 (20/10, informe V-08): A12.</t>
+          <t>Escalas, habilitada desde la 0.5.0. Metrónomo, área propia desde la 0.5.4, y Acordes desde la 0.5.5 (tu decisión del 21/10). Validado en la Sesión 1 (20/10, informe V-08): A12. Pendiente (CP-5): un registro de áreas, para que añadir una no obligue a tocar cuatro o cinco sitios (AT-11 #4).</t>
         </is>
       </c>
       <c r="P6" s="6" t="n"/>
@@ -2396,11 +2396,15 @@
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>Tu comentario del 21/10. Hecho en la 0.5.2: Ajustes › Notación › Notas alteradas (Do♯ o Re♭, Re♯ o Mi♭, Fa♯ o Sol♭, Sol♯ o La♭, La♯ o Si♭); se usan los signos ♯ y ♭, también en el pentagrama. Validado por el banco. Desde la 0.5.3, también el pentagrama del Afinador; y en Escalas, el lector grande y el lector de pantalla escriben como la escala (AT-09).</t>
+          <t>Tu comentario del 21/10. Hecho en la 0.5.2: Ajustes › Notación › Notas alteradas (Do♯ o Re♭, Re♯ o Mi♭, Fa♯ o Sol♭, Sol♯ o La♭, La♯ o Si♭); se usan los signos ♯ y ♭, también en el pentagrama. Validado por el banco. Desde la 0.5.3, también el pentagrama del Afinador; y en Escalas, el lector grande y el lector de pantalla escriben como la escala (AT-09). Pendiente (CP-5): quitar LATIN y los campos anglo y latin de noteInfo(), que ya no se usan y se saltarían N-06 (AT-11 #10).</t>
         </is>
       </c>
       <c r="P26" s="6" t="n"/>
-      <c r="Q26" s="5" t="inlineStr"/>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="33" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -3863,7 +3867,7 @@
       </c>
       <c r="M45" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N45" s="5" t="inlineStr">
@@ -4955,11 +4959,15 @@
       </c>
       <c r="O59" s="5" t="inlineStr">
         <is>
-          <t>El fallo rompe la racha siempre. Se iluminan todas las posiciones correctas y se vuelve a oír la nota buscada justo después de la pulsada, para aprender por contraste; luego llega el reto siguiente. Desde la 0.3.3 (Sesión 1, A09), la corrección llega a los 1,2 s (antes 0,65) y el reto siguiente 3 s después, para poder comparar las dos notas; el fallo se rellena en rojo con ✗ y las posiciones correctas en verde con ✓, de modo que no dependa solo del color. Sesión 1 (20/10, informe V-08): lo esencial cumplió en A09; el cambio de la 0.3.3 lo pediste tú y se confirma en la Sesión 2.</t>
+          <t>El fallo rompe la racha siempre. Se iluminan todas las posiciones correctas y se vuelve a oír la nota buscada justo después de la pulsada, para aprender por contraste; luego llega el reto siguiente. Desde la 0.3.3 (Sesión 1, A09), la corrección llega a los 1,2 s (antes 0,65) y el reto siguiente 3 s después, para poder comparar las dos notas; el fallo se rellena en rojo con ✗ y las posiciones correctas en verde con ✓, de modo que no dependa solo del color. Sesión 1 (20/10, informe V-08): lo esencial cumplió en A09; el cambio de la 0.3.3 lo pediste tú y se confirma en la Sesión 2. Pendiente (CP-5): condicionarlo a «Al fallar: Ver la respuesta», que desde la 0.5.3 ya no es lo de fábrica, y describirlo así en interfaz.md A2 (AR-12 #7).</t>
         </is>
       </c>
       <c r="P59" s="6" t="n"/>
-      <c r="Q59" s="5" t="inlineStr"/>
+      <c r="Q59" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="120" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
@@ -5261,7 +5269,7 @@
       </c>
       <c r="M63" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N63" s="5" t="inlineStr">
@@ -5350,11 +5358,15 @@
       </c>
       <c r="O64" s="5" t="inlineStr">
         <is>
-          <t>Alcance acotado. Las demás afinaciones pasan a E-02b. Hecho y validado en la 0.5.0 (banco tests/escalas.test.js): las 48 escalas se escriben como en el círculo de quintas, con siete letras distintas en las mayores y menores y sin mezclar ♯ y ♭. Las casillas salen de la clase de altura de cada nota, así que también funcionan en las demás afinaciones; lo que sigue fuera (E-02b) son las digitaciones.</t>
+          <t>Alcance acotado. Las demás afinaciones pasan a E-02b. Hecho y validado en la 0.5.0 (banco tests/escalas.test.js): las 48 escalas se escriben como en el círculo de quintas, con siete letras distintas en las mayores y menores y sin mezclar ♯ y ♭. Las casillas salen de la clase de altura de cada nota, así que también funcionan en las demás afinaciones; lo que sigue fuera (E-02b) son las digitaciones. Pendiente (CP-5): comparar nota a nota las 48 escalas con una tabla de referencia (hoy, 16 más reglas generales) y comprobar las 48 en el mástil (AR-12 #4, AT-11); que una alteración fuera de ±2 dé error y no «Doundefined» (AT-11 #9). Alcance: funciona en todas las afinaciones aunque el texto diga solo estándar; lo confirmas tú (AR-12 #9).</t>
         </is>
       </c>
       <c r="P64" s="6" t="n"/>
-      <c r="Q64" s="5" t="inlineStr"/>
+      <c r="Q64" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="48" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -5498,7 +5510,7 @@
       </c>
       <c r="M66" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N66" s="5" t="inlineStr">
@@ -5514,7 +5526,7 @@
       <c r="P66" s="6" t="n"/>
       <c r="Q66" s="5" t="inlineStr"/>
     </row>
-    <row r="67" ht="93" customHeight="1">
+    <row r="67" ht="120" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
           <t>E-04</t>
@@ -5577,7 +5589,7 @@
       </c>
       <c r="M67" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N67" s="5" t="inlineStr">
@@ -5587,11 +5599,15 @@
       </c>
       <c r="O67" s="5" t="inlineStr">
         <is>
-          <t>Etiquetas tipo T — T — ST — T — T — T — ST. Hecho en la 0.5.0: encima del paso a paso, «Do T Re T Mi ST Fa…»; en las pentatónicas aparece también T½ (tono y medio). Los intervalos van en esa línea y no en cada casilla, donde no caben. Falta que lo veas.</t>
+          <t>Etiquetas tipo T — T — ST — T — T — T — ST. Hecho en la 0.5.0: encima del paso a paso, «Do T Re T Mi ST Fa…»; en las pentatónicas aparece también T½ (tono y medio). Los intervalos van en esa línea y no en cada casilla, donde no caben. Falta que lo veas. Pendiente (CP-5): T, ST y T½ no se traducen al inglés, y «T½» puede leerse como medio tono (AR-12 #8).</t>
         </is>
       </c>
       <c r="P67" s="6" t="n"/>
-      <c r="Q67" s="5" t="inlineStr"/>
+      <c r="Q67" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="120" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
@@ -5751,7 +5767,7 @@
       <c r="P69" s="6" t="n"/>
       <c r="Q69" s="5" t="inlineStr"/>
     </row>
-    <row r="70" ht="78" customHeight="1">
+    <row r="70" ht="120" customHeight="1">
       <c r="A70" s="4" t="inlineStr">
         <is>
           <t>E-06</t>
@@ -5814,7 +5830,7 @@
       </c>
       <c r="M70" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N70" s="5" t="inlineStr">
@@ -5824,11 +5840,15 @@
       </c>
       <c r="O70" s="5" t="inlineStr">
         <is>
-          <t>Hecho en la 0.5.0: ◀ ▶ recorre la escala desde la tónica más grave del mástil hasta su octava; cada paso suena, se resalta en el mástil y en el pentagrama, y se explica («Mi, un tono sobre Re»). Falta que lo veas.</t>
+          <t>Hecho en la 0.5.0: ◀ ▶ recorre la escala desde la tónica más grave del mástil hasta su octava; cada paso suena, se resalta en el mástil y en el pentagrama, y se explica («Mi, un tono sobre Re»). Falta que lo veas. Pendiente (CP-5): con una afinación muy grave (36 o menos) el pentagrama cambia de octava a mitad de escala; hace falta un solo desplazamiento por pentagrama (AT-09 #10, AT-11 #3).</t>
         </is>
       </c>
       <c r="P70" s="6" t="n"/>
-      <c r="Q70" s="5" t="inlineStr"/>
+      <c r="Q70" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="33" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
@@ -6766,7 +6786,7 @@
       <c r="P82" s="6" t="n"/>
       <c r="Q82" s="5" t="inlineStr"/>
     </row>
-    <row r="83" ht="108" customHeight="1">
+    <row r="83" ht="120" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
         <is>
           <t>MT-01</t>
@@ -6829,7 +6849,7 @@
       </c>
       <c r="M83" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N83" s="5" t="inlineStr">
@@ -6839,11 +6859,15 @@
       </c>
       <c r="O83" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10 y tu guía con la app que nos enseñaste: lo más directo. Se usa igual en vertical y en horizontal: como el Afinador, no pide girar el móvil. La barra se mueve también con las flechas del teclado. Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2).</t>
+          <t>Tu petición del 21/10 y tu guía con la app que nos enseñaste: lo más directo. Se usa igual en vertical y en horizontal: como el Afinador, no pide girar el móvil. La barra se mueve también con las flechas del teclado. Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2). Verificado parcialmente: lo sostiene el banco hasta que lo compruebes tú (Sesión 2), igual que las escalas (CP-5, AR-12 #1). Pendiente (CP-5): mostrar qué figura cuenta el tempo («♩. = 80» en 6/8) y citar en el criterio los tramos de los nombres italianos (AR-12 #11).</t>
         </is>
       </c>
       <c r="P83" s="6" t="n"/>
-      <c r="Q83" s="5" t="inlineStr"/>
+      <c r="Q83" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="108" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
@@ -7003,7 +7027,7 @@
       <c r="P85" s="6" t="n"/>
       <c r="Q85" s="5" t="inlineStr"/>
     </row>
-    <row r="86" ht="93" customHeight="1">
+    <row r="86" ht="120" customHeight="1">
       <c r="A86" s="4" t="inlineStr">
         <is>
           <t>MT-04</t>
@@ -7076,11 +7100,15 @@
       </c>
       <c r="O86" s="5" t="inlineStr">
         <is>
-          <t>Con un temporizador normal el pulso «se arrastra»: el reloj de audio es exacto. Lo de pararse sigue la regla del sonido en segundo plano (Sesión 1, C07). Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2).</t>
+          <t>Con un temporizador normal el pulso «se arrastra»: el reloj de audio es exacto. Lo de pararse sigue la regla del sonido en segundo plano (Sesión 1, C07). Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2). En la 0.5.7 (CP-5, AT-11 #1), arranca aunque el iPhone haya dejado el audio en pausa (tras una llamada o Siri): espera a que despierte. Pendiente (CP-5): medir el pulso en Chromium con audio real, 60 s a 250 ppm cambiando de área (AR-12 #3); al parar pueden sonar los golpes ya programados, hasta 100 ms (AT-11 #2); el dibujo no descuenta la latencia de salida (AT-11 #5); desconectar los osciladores al acabar (AT-11 #6). Decisión tuya pendiente: mantener la pantalla encendida mientras suena (AR-12 #2).</t>
         </is>
       </c>
       <c r="P86" s="6" t="n"/>
-      <c r="Q86" s="5" t="inlineStr"/>
+      <c r="Q86" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="120" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
@@ -7145,7 +7173,7 @@
       </c>
       <c r="M87" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N87" s="5" t="inlineStr">
@@ -7155,7 +7183,7 @@
       </c>
       <c r="O87" s="5" t="inlineStr">
         <is>
-          <t>Tu decisión del 21/10: función propia, no un chip del acceso rápido. Al escuchar con el micrófono en el Afinador, el metrónomo se para y lo dice: su clic confundiría al detector. Distribución: interfaz.md §7b, aprobada el 21/10. Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2).</t>
+          <t>Tu decisión del 21/10: función propia, no un chip del acceso rápido. Al escuchar con el micrófono en el Afinador, el metrónomo se para y lo dice: su clic confundiría al detector. Distribución: interfaz.md §7b, aprobada el 21/10. Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2). Verificado parcialmente: lo sostiene el banco hasta que lo compruebes tú (Sesión 2), igual que las escalas (CP-5, AR-12 #1).</t>
         </is>
       </c>
       <c r="P87" s="6" t="n"/>
@@ -7238,11 +7266,15 @@
       </c>
       <c r="O88" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10 («ya iremos ampliando»). Populares: C, G, D, A, E, Am, Em, Dm y F. Los 30: mayores, menores, 7, m7 y maj7 de uso común, Dsus4, C/G y G/B, en posición abierta o con las cejillas más habituales. En vertical el listado va arriba y el mástil abajo; en horizontal, el listado a la derecha. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
+          <t>Tu petición del 21/10 («ya iremos ampliando»). Populares: C, G, D, A, E, Am, Em, Dm y F. Los 30: mayores, menores, 7, m7 y maj7 de uso común, Dsus4, C/G y G/B, en posición abierta o con las cejillas más habituales. En vertical el listado va arriba y el mástil abajo; en horizontal, el listado a la derecha. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2). Pendiente (CP-5): contrastar los 30 con la tablatura y los dedos de un método citado; probar la cejilla y dibujar los 30 en el mástil (AR-12 #4, AT-11); raíz con alteración para F♯m, B♭ o D/F♯ (AT-11 #8); rasgueo con el reloj de audio (AT-11 #7).</t>
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
-      <c r="Q88" s="5" t="inlineStr"/>
+      <c r="Q88" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="120" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
@@ -7307,7 +7339,7 @@
       </c>
       <c r="M89" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N89" s="5" t="inlineStr">
@@ -7317,13 +7349,17 @@
       </c>
       <c r="O89" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10: número y color a la vez, con el color constante entre acordes. Colores de la paleta Okabe-Ito, que se distinguen también con daltonismo; en Acordes no se ven los colores de nota, así que no se confunden con ellos. Cada círculo contrasta al menos 3:1 con el mástil y su número al menos 4,5:1 con el círculo (G-05). El lector de pantalla dice el dedo de cada casilla. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
+          <t>Tu petición del 21/10: número y color a la vez, con el color constante entre acordes. Colores de la paleta Okabe-Ito, que se distinguen también con daltonismo; en Acordes no se ven los colores de nota, así que no se confunden con ellos. Cada círculo contrasta al menos 3:1 con el mástil y su número al menos 4,5:1 con el círculo (G-05). El lector de pantalla dice el dedo de cada casilla. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2). Verificado parcialmente: lo sostiene el banco hasta que lo compruebes tú (Sesión 2), igual que las escalas (CP-5, AR-12 #1).</t>
         </is>
       </c>
       <c r="P89" s="6" t="n"/>
-      <c r="Q89" s="5" t="inlineStr"/>
-    </row>
-    <row r="90" ht="93" customHeight="1">
+      <c r="Q89" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="120" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
         <is>
           <t>AC-03</t>
@@ -7386,7 +7422,7 @@
       </c>
       <c r="M90" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N90" s="5" t="inlineStr">
@@ -7396,11 +7432,15 @@
       </c>
       <c r="O90" s="5" t="inlineStr">
         <is>
-          <t>En el móvil en vertical el pentagrama se aparta para que el listado y el mástil quepan; se ve al girar el móvil y en pantallas amplias. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
+          <t>En el móvil en vertical el pentagrama se aparta para que el listado y el mástil quepan; se ve al girar el móvil y en pantallas amplias. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2). Verificado parcialmente: lo sostiene el banco hasta que lo compruebes tú (Sesión 2), igual que las escalas (CP-5, AR-12 #1).</t>
         </is>
       </c>
       <c r="P90" s="6" t="n"/>
-      <c r="Q90" s="5" t="inlineStr"/>
+      <c r="Q90" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="48" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
@@ -7637,11 +7677,7 @@
         </is>
       </c>
       <c r="P93" s="6" t="n"/>
-      <c r="Q93" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q93" s="5" t="inlineStr"/>
     </row>
     <row r="94" ht="120" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
@@ -7720,11 +7756,7 @@
         </is>
       </c>
       <c r="P94" s="6" t="n"/>
-      <c r="Q94" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q94" s="5" t="inlineStr"/>
     </row>
     <row r="95" ht="33" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
@@ -9940,7 +9972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9980,34 +10012,34 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.5.6</t>
+          <t>0.5.7</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Auditoría AR-11: G-02, C-04 y V-01 con las seis áreas; criterio de AC-01 preciso (sus4 y tríadas); evidencias completadas en MT-01, MT-05, AC-01, AC-03 y AC-04 (método T).</t>
+          <t>Punto de control CP-5 (AR-12 y AT-11): una sola vara para lo que compruebas tú. E-01, E-03, E-04, E-06, P-03, MT-01, MT-05, AC-02 y AC-03, verificados parcialmente hasta la Sesión 2; MT-04, arranque con el audio en pausa (0.5.7); lo pendiente de CP-5, en el comentario de su requisito.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -10017,24 +10049,24 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.5.5</t>
+          <t>0.5.6</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>AC-01 a AC-05 implementados y verificados por el banco (F5.7); AC-06 nuevo, el buscador; criterios al día con tu guía del listado.</t>
+          <t>Auditoría AR-11: G-02, C-04 y V-01 con las seis áreas; criterio de AC-01 preciso (sus4 y tríadas); evidencias completadas en MT-01, MT-05, AC-01, AC-03 y AC-04 (método T).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -10044,24 +10076,24 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.5.4</t>
+          <t>0.5.5</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
+          <t>AC-01 a AC-05 implementados y verificados por el banco (F5.7); AC-06 nuevo, el buscador; criterios al día con tu guía del listado.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -10071,24 +10103,24 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.5.3</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
+          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -10098,24 +10130,24 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.5.2</t>
+          <t>0.5.3</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
+          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -10125,24 +10157,24 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.5.0</t>
+          <t>0.5.2</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
+          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -10152,24 +10184,24 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.4.2</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
+          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -10179,51 +10211,51 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>0.4.0</t>
+          <t>0.4.2</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
+          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>0.3.3</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
+          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -10233,24 +10265,24 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>0.3.2</t>
+          <t>0.3.3</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
+          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -10260,24 +10292,24 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>0.3.1</t>
+          <t>0.3.2</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
+          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -10287,24 +10319,24 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -10314,24 +10346,24 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -10341,7 +10373,7 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
@@ -10351,14 +10383,14 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -10368,7 +10400,7 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
@@ -10378,24 +10410,24 @@
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
@@ -10405,14 +10437,14 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -10422,24 +10454,24 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -10449,24 +10481,24 @@
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -10476,51 +10508,51 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -10530,7 +10562,7 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
@@ -10540,32 +10572,59 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="46" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="46" customHeight="1">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
CP-5 ronda 2: Escalas en la Sesión 2, E-02 verificado parcialmente y redacción precisa (AR-12, AT-11)
Las dos revisiones ligeras de lo corregido dan «resuelto».
- F5.2 y F5.3 entran en la Sesión 2 (o antes en F5.8): sus requisitos la esperaban.
- E-02: la evidencia ya no dice «las 48 escalas»; queda verificado
  parcialmente hasta tener la tabla de referencia completa (52 validados).
- MT-04 anota los tres detalles de la ronda técnica. Informes con su ronda 2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AWJcxzncaZFWFnJfpoVV8q
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -5343,12 +5343,12 @@
       </c>
       <c r="L64" s="5" t="inlineStr">
         <is>
-          <t>tests/escalas.test.js: las 48 escalas frente al círculo de quintas; casillas por clase de altura</t>
+          <t>tests/escalas.test.js: las 24 mayores y menores con siete letras, sin mezclar ♯ y ♭ ni dobles alteraciones, y 16 de ellas nota a nota frente al libro; pentatónicas dentro de su escala; casillas por clase de altura</t>
         </is>
       </c>
       <c r="M64" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N64" s="5" t="inlineStr">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="O64" s="5" t="inlineStr">
         <is>
-          <t>Alcance acotado. Las demás afinaciones pasan a E-02b. Hecho y validado en la 0.5.0 (banco tests/escalas.test.js): las 48 escalas se escriben como en el círculo de quintas, con siete letras distintas en las mayores y menores y sin mezclar ♯ y ♭. Las casillas salen de la clase de altura de cada nota, así que también funcionan en las demás afinaciones; lo que sigue fuera (E-02b) son las digitaciones. Pendiente (CP-5): comparar nota a nota las 48 escalas con una tabla de referencia (hoy, 16 más reglas generales) y comprobar las 48 en el mástil (AR-12 #4, AT-11); que una alteración fuera de ±2 dé error y no «Doundefined» (AT-11 #9). Alcance: funciona en todas las afinaciones aunque el texto diga solo estándar; lo confirmas tú (AR-12 #9).</t>
+          <t>Alcance acotado. Las demás afinaciones pasan a E-02b. Hecho en la 0.5.0 (banco tests/escalas.test.js): las 24 mayores y menores con siete letras distintas, sin mezclar ♯ y ♭ ni dobles alteraciones, y 16 de ellas comparadas nota a nota con el libro; las pentatónicas, dentro de su escala. Verificado parcialmente hasta tener la tabla de referencia completa (CP-5, AR-12 #4 y ronda 2). Las casillas salen de la clase de altura de cada nota, así que también funcionan en las demás afinaciones; lo que sigue fuera (E-02b) son las digitaciones. Pendiente (CP-5): comparar nota a nota las 48 escalas con una tabla de referencia (hoy, 16 más reglas generales) y comprobar las 48 en el mástil (AR-12 #4, AT-11); que una alteración fuera de ±2 dé error y no «Doundefined» (AT-11 #9). Alcance: funciona en todas las afinaciones aunque el texto diga solo estándar; lo confirmas tú (AR-12 #9).</t>
         </is>
       </c>
       <c r="P64" s="6" t="n"/>
@@ -7100,7 +7100,7 @@
       </c>
       <c r="O86" s="5" t="inlineStr">
         <is>
-          <t>Con un temporizador normal el pulso «se arrastra»: el reloj de audio es exacto. Lo de pararse sigue la regla del sonido en segundo plano (Sesión 1, C07). Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2). En la 0.5.7 (CP-5, AT-11 #1), arranca aunque el iPhone haya dejado el audio en pausa (tras una llamada o Siri): espera a que despierte. Pendiente (CP-5): medir el pulso en Chromium con audio real, 60 s a 250 ppm cambiando de área (AR-12 #3); al parar pueden sonar los golpes ya programados, hasta 100 ms (AT-11 #2); el dibujo no descuenta la latencia de salida (AT-11 #5); desconectar los osciladores al acabar (AT-11 #6). Decisión tuya pendiente: mantener la pantalla encendida mientras suena (AR-12 #2).</t>
+          <t>Con un temporizador normal el pulso «se arrastra»: el reloj de audio es exacto. Lo de pararse sigue la regla del sonido en segundo plano (Sesión 1, C07). Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2). En la 0.5.7 (CP-5, AT-11 #1), arranca aunque el iPhone haya dejado el audio en pausa (tras una llamada o Siri): espera a que despierte. Pendiente (CP-5): medir el pulso en Chromium con audio real, 60 s a 250 ppm cambiando de área (AR-12 #3); al parar pueden sonar los golpes ya programados, hasta 100 ms (AT-11 #2); el dibujo no descuenta la latencia de salida (AT-11 #5); desconectar los osciladores al acabar (AT-11 #6). Ronda 2 de AT-11: tras Siri, si el audio sigue en pausa, «Vuelve a pulsar» se repite sin rehacer el audio (medio); durante la espera el botón no cambia (bajo); Empezar, Parar y Empezar en menos de 400 ms puede anular el tercero (bajo). Decisión tuya pendiente: mantener la pantalla encendida mientras suena (AR-12 #2).</t>
         </is>
       </c>
       <c r="P86" s="6" t="n"/>
@@ -10032,7 +10032,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Punto de control CP-5 (AR-12 y AT-11): una sola vara para lo que compruebas tú. E-01, E-03, E-04, E-06, P-03, MT-01, MT-05, AC-02 y AC-03, verificados parcialmente hasta la Sesión 2; MT-04, arranque con el audio en pausa (0.5.7); lo pendiente de CP-5, en el comentario de su requisito.</t>
+          <t>Punto de control CP-5 (AR-12 y AT-11): una sola vara para lo que compruebas tú. E-01, E-02, E-03, E-04, E-06, P-03, MT-01, MT-05, AC-02 y AC-03, verificados parcialmente hasta la Sesión 2; MT-04, arranque con el audio en pausa (0.5.7); lo pendiente de CP-5, en el comentario de su requisito.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F6.1: documentos de la etapa (G-08; requisitos v1.25, matriz v1.23, roadmap v3.23, IT-04)
- G-08 cumple y queda validado por el banco (53 validados).
- Roadmap: F6.1 hecha, F6 en curso y F5 abierta; «Estás aquí» al día.
- IT-04-F6: código fuente frente a artefacto, proceso de construcción y por
  qué hay que probar el artefacto y no solo el fuente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FozqoEELEJkBunkoec24Nq
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.22. Base: requisitos.md v1.24 · app 0.5.7 · roadmap 3.22 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.23. Base: requisitos.md v1.25 · app 0.6.0 · roadmap 3.23 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.22</t>
+          <t>Cambio en v1.23</t>
         </is>
       </c>
     </row>
@@ -824,11 +824,7 @@
         </is>
       </c>
       <c r="P6" s="6" t="n"/>
-      <c r="Q6" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="108" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -1273,7 +1269,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Cumple parcialmente</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1283,12 +1279,12 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): el autónomo es exactamente la app ensamblada (ensamblar.js) más su audio; la app en js/ se carga archivo a archivo</t>
+          <t>Banco (node --test) en dos pasadas: app de varios archivos (banco.test.js) y archivo autónomo (autonomo.test.js), que además lee de dentro sus 17 grabaciones (huellas sha256) sin descargar nada · el autónomo es exactamente la app ensamblada más su audio · comprobar-autonomo (Chromium, file:// y sin conexión) · comprobar-en-navegador</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>Verificado parcialmente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
@@ -1298,11 +1294,15 @@
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>Desde la 0.2.1 hay dos formas reales: index.html para servir (Live Server y web) y dist/trasteando.html, generado a partir de él con herramientas/generar-autonomo.py. El banco comprueba que el autónomo está al día con index.html. Se vuelve más exigente al pasar a módulos (F4.1); F6.1 generará el archivo autónomo a partir de ellos. Desde la 0.4.0 (F4.1), la app vive en varios archivos (css/ y js/, uno por tema); herramientas/generar-autonomo.py sigue generando el archivo autónomo, y ahora usa herramientas/ensamblar.js para unirlos; el banco comprueba que el resultado es exactamente la app más su audio.</t>
+          <t>Desde la 0.2.1 hay dos formas reales: index.html para servir (Live Server y web) y dist/trasteando.html, generado a partir de él con herramientas/generar-autonomo.py. Desde la 0.4.0 (F4.1), la app vive en varios archivos (css/ y js/, uno por tema), y el generador los une con herramientas/ensamblar.js; el banco comprueba que el resultado es exactamente la app más su audio. Hecho en la 0.6.0 (F6.1) y validado por el banco: el banco entero se pasa dos veces, contra la app de varios archivos (la que sirve la web) y contra el autónomo (tests/autonomo.test.js); el autónomo lee de dentro sus 17 grabaciones, las generadas, sin descargar nada; cada módulo incrustado lleva su nombre (//# sourceURL) y el ensamblador se niega a incrustar uno que cortaría la página. En Chromium, abierto desde el disco y sin conexión, abre en 0,3 s sin ningún intento de conexión. Instalarla como PWA es G-04 (F6.3).</t>
         </is>
       </c>
       <c r="P12" s="6" t="n"/>
-      <c r="Q12" s="5" t="inlineStr"/>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="63" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -2400,11 +2400,7 @@
         </is>
       </c>
       <c r="P26" s="6" t="n"/>
-      <c r="Q26" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q26" s="5" t="inlineStr"/>
     </row>
     <row r="27" ht="33" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -4963,11 +4959,7 @@
         </is>
       </c>
       <c r="P59" s="6" t="n"/>
-      <c r="Q59" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q59" s="5" t="inlineStr"/>
     </row>
     <row r="60" ht="120" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
@@ -5362,11 +5354,7 @@
         </is>
       </c>
       <c r="P64" s="6" t="n"/>
-      <c r="Q64" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q64" s="5" t="inlineStr"/>
     </row>
     <row r="65" ht="48" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -5603,11 +5591,7 @@
         </is>
       </c>
       <c r="P67" s="6" t="n"/>
-      <c r="Q67" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q67" s="5" t="inlineStr"/>
     </row>
     <row r="68" ht="120" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
@@ -5844,11 +5828,7 @@
         </is>
       </c>
       <c r="P70" s="6" t="n"/>
-      <c r="Q70" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q70" s="5" t="inlineStr"/>
     </row>
     <row r="71" ht="33" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
@@ -6863,11 +6843,7 @@
         </is>
       </c>
       <c r="P83" s="6" t="n"/>
-      <c r="Q83" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q83" s="5" t="inlineStr"/>
     </row>
     <row r="84" ht="108" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
@@ -7104,11 +7080,7 @@
         </is>
       </c>
       <c r="P86" s="6" t="n"/>
-      <c r="Q86" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q86" s="5" t="inlineStr"/>
     </row>
     <row r="87" ht="120" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
@@ -7187,11 +7159,7 @@
         </is>
       </c>
       <c r="P87" s="6" t="n"/>
-      <c r="Q87" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q87" s="5" t="inlineStr"/>
     </row>
     <row r="88" ht="120" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
@@ -7270,11 +7238,7 @@
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
-      <c r="Q88" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q88" s="5" t="inlineStr"/>
     </row>
     <row r="89" ht="120" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
@@ -7353,11 +7317,7 @@
         </is>
       </c>
       <c r="P89" s="6" t="n"/>
-      <c r="Q89" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q89" s="5" t="inlineStr"/>
     </row>
     <row r="90" ht="120" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
@@ -7436,11 +7396,7 @@
         </is>
       </c>
       <c r="P90" s="6" t="n"/>
-      <c r="Q90" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q90" s="5" t="inlineStr"/>
     </row>
     <row r="91" ht="48" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
@@ -9972,7 +9928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10012,7 +9968,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -10022,51 +9978,51 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.5.7</t>
+          <t>0.6.0</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>Punto de control CP-5 (AR-12 y AT-11): una sola vara para lo que compruebas tú. E-01, E-02, E-03, E-04, E-06, P-03, MT-01, MT-05, AC-02 y AC-03, verificados parcialmente hasta la Sesión 2; MT-04, arranque con el audio en pausa (0.5.7); lo pendiente de CP-5, en el comentario de su requisito.</t>
+          <t>F6.1: G-08 cumple y queda verificado por el banco, que se pasa entero contra la app de varios archivos y contra el archivo autónomo.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.5.6</t>
+          <t>0.5.7</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Auditoría AR-11: G-02, C-04 y V-01 con las seis áreas; criterio de AC-01 preciso (sus4 y tríadas); evidencias completadas en MT-01, MT-05, AC-01, AC-03 y AC-04 (método T).</t>
+          <t>Punto de control CP-5 (AR-12 y AT-11): una sola vara para lo que compruebas tú. E-01, E-02, E-03, E-04, E-06, P-03, MT-01, MT-05, AC-02 y AC-03, verificados parcialmente hasta la Sesión 2; MT-04, arranque con el audio en pausa (0.5.7); lo pendiente de CP-5, en el comentario de su requisito.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -10076,24 +10032,24 @@
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.5.5</t>
+          <t>0.5.6</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>AC-01 a AC-05 implementados y verificados por el banco (F5.7); AC-06 nuevo, el buscador; criterios al día con tu guía del listado.</t>
+          <t>Auditoría AR-11: G-02, C-04 y V-01 con las seis áreas; criterio de AC-01 preciso (sus4 y tríadas); evidencias completadas en MT-01, MT-05, AC-01, AC-03 y AC-04 (método T).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -10103,24 +10059,24 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.5.4</t>
+          <t>0.5.5</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
+          <t>AC-01 a AC-05 implementados y verificados por el banco (F5.7); AC-06 nuevo, el buscador; criterios al día con tu guía del listado.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -10130,24 +10086,24 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.5.3</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
+          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -10157,24 +10113,24 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.5.2</t>
+          <t>0.5.3</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
+          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -10184,24 +10140,24 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.5.0</t>
+          <t>0.5.2</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
+          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -10211,24 +10167,24 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>0.4.2</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
+          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -10238,51 +10194,51 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>0.4.0</t>
+          <t>0.4.2</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
+          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>0.3.3</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
+          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -10292,24 +10248,24 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>0.3.2</t>
+          <t>0.3.3</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
+          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -10319,24 +10275,24 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>0.3.1</t>
+          <t>0.3.2</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
+          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -10346,24 +10302,24 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -10373,24 +10329,24 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -10400,7 +10356,7 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
@@ -10410,14 +10366,14 @@
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -10427,7 +10383,7 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
@@ -10437,24 +10393,24 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
@@ -10464,14 +10420,14 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -10481,24 +10437,24 @@
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -10508,24 +10464,24 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -10535,51 +10491,51 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="46" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -10589,7 +10545,7 @@
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
@@ -10599,32 +10555,59 @@
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="46" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="46" customHeight="1">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F6.1 ronda 1: correcciones de AR-13 y AT-12 (0.6.0, G-08)
- ensamblar.js: el código va pegado a <script> (el salto contaba como
  línea y el navegador daba cada una con una de más, AT-12 #2); rechaza
  también «<!--» (AT-12 #3).
- comprobar-autonomo.js: comprueba en Chromium que un error del autónomo
  dice el módulo y la línea exactos (falla con el autónomo anterior).
- dom-minimo.js: test y unaVez compartidos, con .skip, .todo y .only
  (AT-12 #4); guardián para que todo archivo de pruebas que arranca la app
  se pase contra el autónomo (AT-12 #1); prueba del ensamblador con
  conSalto y sin «<script>\n» (AT-12 #5); nota en autonomo.test.js (#6).
- Documentos: G-08 con lo anotado de AR-13 (#2, #3) y su evidencia (#5);
  CHANGELOG, IT-04, roadmap (Sesión 2), ESTADO; informes AR-13 y AT-12.
- Banco: 156 de 156.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FozqoEELEJkBunkoec24Nq
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -1279,7 +1279,7 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test) en dos pasadas: app de varios archivos (banco.test.js) y archivo autónomo (autonomo.test.js), que además lee de dentro sus 17 grabaciones (huellas sha256) sin descargar nada · el autónomo es exactamente la app ensamblada más su audio · comprobar-autonomo (Chromium, file:// y sin conexión) · comprobar-en-navegador</t>
+          <t>Banco (node --test) en dos pasadas: banco.test.js y escalas.test.js contra la app de varios archivos y contra el autónomo (autonomo.test.js), que además lee de dentro sus 17 grabaciones (huellas sha256) sin descargar nada; una sola vez, lo que lee el repositorio o compara las formas · el autónomo es exactamente la app ensamblada más su audio · comprobar-autonomo (Chromium, file:// y sin conexión: 0,15 s, ninguna conexión, error con módulo y línea exactos) · comprobar-en-navegador · CHANGELOG 0.6.0 · IT-04 · AR-13 y AT-12</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>Desde la 0.2.1 hay dos formas reales: index.html para servir (Live Server y web) y dist/trasteando.html, generado a partir de él con herramientas/generar-autonomo.py. Desde la 0.4.0 (F4.1), la app vive en varios archivos (css/ y js/, uno por tema), y el generador los une con herramientas/ensamblar.js; el banco comprueba que el resultado es exactamente la app más su audio. Hecho en la 0.6.0 (F6.1) y validado por el banco: el banco entero se pasa dos veces, contra la app de varios archivos (la que sirve la web) y contra el autónomo (tests/autonomo.test.js); el autónomo lee de dentro sus 17 grabaciones, las generadas, sin descargar nada; cada módulo incrustado lleva su nombre (//# sourceURL) y el ensamblador se niega a incrustar uno que cortaría la página. En Chromium, abierto desde el disco y sin conexión, abre en 0,3 s sin ningún intento de conexión. Instalarla como PWA es G-04 (F6.3).</t>
+          <t>Desde la 0.2.1 hay dos formas reales: index.html para servir (Live Server y web) y dist/trasteando.html, generado a partir de él con herramientas/generar-autonomo.py. Desde la 0.4.0 (F4.1), la app vive en varios archivos (css/ y js/, uno por tema), y el generador los une con herramientas/ensamblar.js; el banco comprueba que el resultado es exactamente la app más su audio. Hecho en la 0.6.0 (F6.1) y validado por el banco: las pruebas que arrancan la app (banco.test.js y escalas.test.js) se pasan dos veces, contra la app de varios archivos (la que sirve la web) y contra el autónomo (tests/autonomo.test.js); solo van una vez las que leen el repositorio o comparan las dos formas, y las del detector de tono, que no usan la página. El autónomo lee de dentro sus 17 grabaciones, las generadas, sin descargar nada; cada módulo incrustado lleva su nombre (//# sourceURL), y un error dice el módulo y la línea exactos; el ensamblador se niega a incrustar uno que rompería la página. En Chromium, abierto desde el disco y sin conexión, abre en 0,15 s sin ningún intento de conexión. Instalarla como PWA es G-04 (F6.3). Pendiente (AR-13): se reconfirma contra la web publicada en F7.1, como G-03 (#2), y en la Sesión 2 se abre el autónomo con doble clic en Windows, en modo avión (#3).</t>
         </is>
       </c>
       <c r="P12" s="6" t="n"/>
@@ -9988,7 +9988,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>F6.1: G-08 cumple y queda verificado por el banco, que se pasa entero contra la app de varios archivos y contra el archivo autónomo.</t>
+          <t>F6.1: G-08 cumple y queda verificado por el banco, que pasa las pruebas que arrancan la app contra la app de varios archivos y contra el archivo autónomo (AR-13 y AT-12).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F5.8 #1: documentos del péndulo (MT-06 nuevo; requisitos v1.26, matriz v1.24, interfaz v1.14, roadmap v3.24, IT-03)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FozqoEELEJkBunkoec24Nq
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control de cambios" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz'!$A$4:$Q$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz'!$A$4:$Q$114</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q113"/>
+  <dimension ref="A1:Q114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versión 1.23. Base: requisitos.md v1.25 · app 0.6.0 · roadmap 3.23 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
+          <t>Versión 1.24. Base: requisitos.md v1.26 · app 0.6.1 · roadmap 3.24 · emitida el 15/10/2026. Cliente: Pablo Díaz Guerra. Proveedor: chat de Desarrollo. Verificación independiente: auditores de requisitos y técnico.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Cambio en v1.23</t>
+          <t>Cambio en v1.24</t>
         </is>
       </c>
     </row>
@@ -1298,11 +1298,7 @@
         </is>
       </c>
       <c r="P12" s="6" t="n"/>
-      <c r="Q12" s="5" t="inlineStr">
-        <is>
-          <t>Modificado</t>
-        </is>
-      </c>
+      <c r="Q12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="63" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -7164,27 +7160,27 @@
     <row r="88" ht="120" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>AC-01</t>
+          <t>MT-06</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Acordes</t>
+          <t>Metrónomo</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Librería de acordes, un área propia: a un lado, el listado de nombres, con una sección de populares arriba y debajo los 30 acordes más habituales; al otro, el acorde dibujado en el mástil.</t>
+          <t>La barra del tempo es un péndulo, como la de un metrónomo mecánico: la pesa marca el tempo, arriba más lento y abajo más rápido; mientras suena, la barra oscila sobre su pie y llega a un extremo en cada pulso, alternando los lados, hasta 30° a cada lado sin salirse de la pantalla. Se queda recta parada, mientras se arrastra y con «reducir movimiento».</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>Cliente · 21/10</t>
+          <t>Cliente · 22/10 (F5.8 #1)</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
@@ -7194,17 +7190,17 @@
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>F5.7</t>
+          <t>F5.8</t>
         </is>
       </c>
       <c r="H88" s="5" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>D</t>
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>A un lado el listado (populares arriba, los 30 acordes debajo) y al otro el mástil; cada digitación suena solo a notas del acorde, con la raíz, la nota que define el tipo (la tercera, o la cuarta en sus4) y la séptima si la lleva (la quinta se puede omitir), y con la raíz o el bajo indicado como nota más grave.</t>
+          <t>Pesa arriba, 30 ppm, y abajo, 250. Sonando, la barra llega a un extremo en cada pulso, alternando los lados (hasta 30° a cada lado, sin salirse de la pantalla en ninguna disposición), y pasa por el centro entre dos; la subdivisión no la mueve. Recta parada, al arrastrarla y con «reducir movimiento».</t>
         </is>
       </c>
       <c r="J88" s="5" t="inlineStr">
@@ -7214,36 +7210,40 @@
       </c>
       <c r="K88" s="5" t="inlineStr">
         <is>
-          <t>0.5.5</t>
+          <t>0.6.1</t>
         </is>
       </c>
       <c r="L88" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): las 30 digitaciones, una a una; populares y listado · comprobar-disposicion: listado y mástil a la vez en seis pantallas</t>
+          <t>Banco (node --test): extremos alternos en cada pulso, centro a medio camino, la subdivisión no cuenta, recta al arrastrar, al parar y con «reducir movimiento», pesa arriba = 30 ppm, amplitud que cabe; las tres pruebas fallan con la 0.6.0 · Chromium: ±30° en iPhone vertical y ordenador, ±12,7° en horizontal, nunca fuera de la pantalla · comprobar-disposicion: ocho pantallas del metrónomo</t>
         </is>
       </c>
       <c r="M88" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N88" s="5" t="inlineStr">
         <is>
-          <t>Banco automático + auditor técnico</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="O88" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10 («ya iremos ampliando»). Populares: C, G, D, A, E, Am, Em, Dm y F. Los 30: mayores, menores, 7, m7 y maj7 de uso común, Dsus4, C/G y G/B, en posición abierta o con las cejillas más habituales. En vertical el listado va arriba y el mástil abajo; en horizontal, el listado a la derecha. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2). Pendiente (CP-5): contrastar los 30 con la tablatura y los dedos de un método citado; probar la cejilla y dibujar los 30 en el mástil (AR-12 #4, AT-11); raíz con alteración para F♯m, B♭ o D/F♯ (AT-11 #8); rasgueo con el reloj de audio (AT-11 #7).</t>
+          <t>Tu comentario de uso del 22/10 (F5.8 #1) y tu decisión del mismo día: la pesa arriba va más lenta, como en uno mecánico (antes, arriba era más rápido). El ángulo sale del reloj de audio, el mismo de los golpes, así que va con el sonido aunque el navegador vaya a tirones; sigue un coseno, como un péndulo: rápido en el centro y lento en los extremos. La subdivisión no lo mueve: solo los pulsos. Se abre menos si no cabe: en el iPhone en horizontal, unos 13°. Recto con «reducir movimiento» (G-05). Las flechas del teclado siguen la norma de los deslizadores (↑, más rápido). Hecho en la 0.6.1 y comprobado con el banco y en Chromium; verificado parcialmente hasta que lo pruebes tú (Sesión 2).</t>
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
-      <c r="Q88" s="5" t="inlineStr"/>
+      <c r="Q88" s="5" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="120" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>AC-02</t>
+          <t>AC-01</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -7253,7 +7253,7 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>En el mástil, cada nota del acorde lleva un círculo del color de su dedo (1 índice, 2 medio, 3 anular, 4 meñique; el mismo color en todos los acordes) con el número del dedo dentro. Junto al nombre de cada cuerda, ○ si suena al aire y ✕ si no suena; la cejilla, como una barra que une sus cuerdas.</t>
+          <t>Librería de acordes, un área propia: a un lado, el listado de nombres, con una sección de populares arriba y debajo los 30 acordes más habituales; al otro, el acorde dibujado en el mástil.</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
@@ -7278,12 +7278,12 @@
       </c>
       <c r="H89" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T</t>
         </is>
       </c>
       <c r="I89" s="5" t="inlineStr">
         <is>
-          <t>Cada dedo tiene su número y su color, iguales en todos los acordes (Okabe-Ito); círculo ≥ 3:1 contra el mástil y número ≥ 4,5:1 contra el círculo; ○ y ✕ junto al nombre de la cuerda; cejilla como barra; el lector de pantalla dice el dedo.</t>
+          <t>A un lado el listado (populares arriba, los 30 acordes debajo) y al otro el mástil; cada digitación suena solo a notas del acorde, con la raíz, la nota que define el tipo (la tercera, o la cuarta en sus4) y la séptima si la lleva (la quinta se puede omitir), y con la raíz o el bajo indicado como nota más grave.</t>
         </is>
       </c>
       <c r="J89" s="5" t="inlineStr">
@@ -7298,22 +7298,22 @@
       </c>
       <c r="L89" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): La menor y Fa dibujados, contraste de los cuatro colores · comprobar-accesibilidad: Acordes con Fa</t>
+          <t>Banco (node --test): las 30 digitaciones, una a una; populares y listado · comprobar-disposicion: listado y mástil a la vez en seis pantallas</t>
         </is>
       </c>
       <c r="M89" s="5" t="inlineStr">
         <is>
-          <t>Verificado parcialmente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N89" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Banco automático + auditor técnico</t>
         </is>
       </c>
       <c r="O89" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10: número y color a la vez, con el color constante entre acordes. Colores de la paleta Okabe-Ito, que se distinguen también con daltonismo; en Acordes no se ven los colores de nota, así que no se confunden con ellos. Cada círculo contrasta al menos 3:1 con el mástil y su número al menos 4,5:1 con el círculo (G-05). El lector de pantalla dice el dedo de cada casilla. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2). Verificado parcialmente: lo sostiene el banco hasta que lo compruebes tú (Sesión 2), igual que las escalas (CP-5, AR-12 #1).</t>
+          <t>Tu petición del 21/10 («ya iremos ampliando»). Populares: C, G, D, A, E, Am, Em, Dm y F. Los 30: mayores, menores, 7, m7 y maj7 de uso común, Dsus4, C/G y G/B, en posición abierta o con las cejillas más habituales. En vertical el listado va arriba y el mástil abajo; en horizontal, el listado a la derecha. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2). Pendiente (CP-5): contrastar los 30 con la tablatura y los dedos de un método citado; probar la cejilla y dibujar los 30 en el mástil (AR-12 #4, AT-11); raíz con alteración para F♯m, B♭ o D/F♯ (AT-11 #8); rasgueo con el reloj de audio (AT-11 #7).</t>
         </is>
       </c>
       <c r="P89" s="6" t="n"/>
@@ -7322,7 +7322,7 @@
     <row r="90" ht="120" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>AC-03</t>
+          <t>AC-02</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
@@ -7332,12 +7332,12 @@
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>El pentagrama escribe el acorde con sus notas apiladas, escritas como manda el acorde (B7: Re♯); se oculta con el ajuste de pentagrama de siempre.</t>
+          <t>En el mástil, cada nota del acorde lleva un círculo del color de su dedo (1 índice, 2 medio, 3 anular, 4 meñique; el mismo color en todos los acordes) con el número del dedo dentro. Junto al nombre de cada cuerda, ○ si suena al aire y ✕ si no suena; la cejilla, como una barra que une sus cuerdas.</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -7362,7 +7362,7 @@
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>El pentagrama escribe las notas del acorde apiladas, escritas como manda el acorde, y se oculta con su ajuste; en el móvil en vertical se aparta y vuelve al girarlo.</t>
+          <t>Cada dedo tiene su número y su color, iguales en todos los acordes (Okabe-Ito); círculo ≥ 3:1 contra el mástil y número ≥ 4,5:1 contra el círculo; ○ y ✕ junto al nombre de la cuerda; cejilla como barra; el lector de pantalla dice el dedo.</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr">
@@ -7377,7 +7377,7 @@
       </c>
       <c r="L90" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): cinco notas de La menor; B7 con Re♯ · el ajuste de pentagrama de siempre (F1.1) · comprobar-disposicion: seis pantallas</t>
+          <t>Banco (node --test): La menor y Fa dibujados, contraste de los cuatro colores · comprobar-accesibilidad: Acordes con Fa</t>
         </is>
       </c>
       <c r="M90" s="5" t="inlineStr">
@@ -7392,16 +7392,16 @@
       </c>
       <c r="O90" s="5" t="inlineStr">
         <is>
-          <t>En el móvil en vertical el pentagrama se aparta para que el listado y el mástil quepan; se ve al girar el móvil y en pantallas amplias. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2). Verificado parcialmente: lo sostiene el banco hasta que lo compruebes tú (Sesión 2), igual que las escalas (CP-5, AR-12 #1).</t>
+          <t>Tu petición del 21/10: número y color a la vez, con el color constante entre acordes. Colores de la paleta Okabe-Ito, que se distinguen también con daltonismo; en Acordes no se ven los colores de nota, así que no se confunden con ellos. Cada círculo contrasta al menos 3:1 con el mástil y su número al menos 4,5:1 con el círculo (G-05). El lector de pantalla dice el dedo de cada casilla. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2). Verificado parcialmente: lo sostiene el banco hasta que lo compruebes tú (Sesión 2), igual que las escalas (CP-5, AR-12 #1).</t>
         </is>
       </c>
       <c r="P90" s="6" t="n"/>
       <c r="Q90" s="5" t="inlineStr"/>
     </row>
-    <row r="91" ht="48" customHeight="1">
+    <row r="91" ht="120" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>AC-04</t>
+          <t>AC-03</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -7411,12 +7411,12 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>El acorde suena rasgueado, de grave a agudo, al elegirlo y con «Tocar»; cada cuerda se puede tocar suelta.</t>
+          <t>El pentagrama escribe el acorde con sus notas apiladas, escritas como manda el acorde (B7: Re♯); se oculta con el ajuste de pentagrama de siempre.</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -7436,12 +7436,12 @@
       </c>
       <c r="H91" s="5" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>D</t>
         </is>
       </c>
       <c r="I91" s="5" t="inlineStr">
         <is>
-          <t>El acorde suena rasgueado de grave a agudo al elegirlo y con «Tocar»; cada cuerda se puede tocar suelta.</t>
+          <t>El pentagrama escribe las notas del acorde apiladas, escritas como manda el acorde, y se oculta con su ajuste; en el móvil en vertical se aparta y vuelve al girarlo.</t>
         </is>
       </c>
       <c r="J91" s="5" t="inlineStr">
@@ -7456,31 +7456,31 @@
       </c>
       <c r="L91" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): orden del rasgueo · cada casilla suena suelta como en todo el mástil (F1.1 #2)</t>
+          <t>Banco (node --test): cinco notas de La menor; B7 con Re♯ · el ajuste de pentagrama de siempre (F1.1) · comprobar-disposicion: seis pantallas</t>
         </is>
       </c>
       <c r="M91" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N91" s="5" t="inlineStr">
         <is>
-          <t>Banco automático + auditor técnico</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="O91" s="5" t="inlineStr">
         <is>
-          <t>35 ms entre cuerda y cuerda. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
+          <t>En el móvil en vertical el pentagrama se aparta para que el listado y el mástil quepan; se ve al girar el móvil y en pantallas amplias. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2). Verificado parcialmente: lo sostiene el banco hasta que lo compruebes tú (Sesión 2), igual que las escalas (CP-5, AR-12 #1).</t>
         </is>
       </c>
       <c r="P91" s="6" t="n"/>
       <c r="Q91" s="5" t="inlineStr"/>
     </row>
-    <row r="92" ht="63" customHeight="1">
+    <row r="92" ht="48" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>AC-05</t>
+          <t>AC-04</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Las digitaciones son para la afinación estándar en la primera entrega: con otra afinación activa, Acordes lo avisa, no las dibuja y ofrece pasar a la estándar.</t>
+          <t>El acorde suena rasgueado, de grave a agudo, al elegirlo y con «Tocar»; cada cuerda se puede tocar suelta.</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Con otra afinación, Acordes avisa, no dibuja las digitaciones y «Pasar a estándar» las recupera.</t>
+          <t>El acorde suena rasgueado de grave a agudo al elegirlo y con «Tocar»; cada cuerda se puede tocar suelta.</t>
         </is>
       </c>
       <c r="J92" s="5" t="inlineStr">
@@ -7535,7 +7535,7 @@
       </c>
       <c r="L92" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): Drop D y vuelta a la estándar</t>
+          <t>Banco (node --test): orden del rasgueo · cada casilla suena suelta como en todo el mástil (F1.1 #2)</t>
         </is>
       </c>
       <c r="M92" s="5" t="inlineStr">
@@ -7550,16 +7550,16 @@
       </c>
       <c r="O92" s="5" t="inlineStr">
         <is>
-          <t>Las digitaciones dependen de la afinación; las demás, para después. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
+          <t>35 ms entre cuerda y cuerda. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
         </is>
       </c>
       <c r="P92" s="6" t="n"/>
       <c r="Q92" s="5" t="inlineStr"/>
     </row>
-    <row r="93" ht="78" customHeight="1">
+    <row r="93" ht="63" customHeight="1">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>AC-06</t>
+          <t>AC-05</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -7569,7 +7569,7 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Un buscador filtra el listado por cómo empieza el nombre: «G» deja G, Gm, G7, G/B…; vale en las dos nomenclaturas («Sol» encuentra lo mismo) y sin distinguir mayúsculas.</t>
+          <t>Las digitaciones son para la afinación estándar en la primera entrega: con otra afinación activa, Acordes lo avisa, no las dibuja y ofrece pasar a la estándar.</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
@@ -7599,7 +7599,7 @@
       </c>
       <c r="I93" s="5" t="inlineStr">
         <is>
-          <t>El buscador deja los acordes que empiezan por lo escrito, sin distinguir mayúsculas y en las dos nomenclaturas; una letra sola, solo en la inglesa.</t>
+          <t>Con otra afinación, Acordes avisa, no dibuja las digitaciones y «Pasar a estándar» las recupera.</t>
         </is>
       </c>
       <c r="J93" s="5" t="inlineStr">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="L93" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): G, g, Sol, D, Am, f# y vacío</t>
+          <t>Banco (node --test): Drop D y vuelta a la estándar</t>
         </is>
       </c>
       <c r="M93" s="5" t="inlineStr">
@@ -7629,56 +7629,56 @@
       </c>
       <c r="O93" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10. Una sola letra solo se busca en la nomenclatura inglesa, para que «D» no traiga también los Do; # y b valen por ♯ y ♭. Hecho en la 0.5.5 y validado por el banco.</t>
+          <t>Las digitaciones dependen de la afinación; las demás, para después. Hecho en la 0.5.5 y validado por el banco; falta que lo compares con tu guitarra (Sesión 2).</t>
         </is>
       </c>
       <c r="P93" s="6" t="n"/>
       <c r="Q93" s="5" t="inlineStr"/>
     </row>
-    <row r="94" ht="120" customHeight="1">
+    <row r="94" ht="78" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>V-01</t>
+          <t>AC-06</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>Visualización</t>
+          <t>Acordes</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>En móvil se sugiere la orientación horizontal con un aviso discreto; no se fuerza.</t>
+          <t>Un buscador filtra el listado por cómo empieza el nombre: «G» deja G, Gm, G7, G/B…; vale en las dos nomenclaturas («Sol» encuentra lo mismo) y sin distinguir mayúsculas.</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
+          <t>Cliente · 21/10</t>
         </is>
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
         <is>
-          <t>F3.2</t>
+          <t>F5.7</t>
         </is>
       </c>
       <c r="H94" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T</t>
         </is>
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>En horizontal, con un alto útil de 268 px o más, cada cuerda mide al menos 40 px (iPhone en Safari e instalada; simulador de Android). En vertical, en pantallas táctiles de menos de 600 px de ancho y en Libre, Adivinar, Escalas y Acordes, aparece el aviso para girar; nunca en el Afinador ni en el Metrónomo; cerrado, no vuelve y «Restablecer» lo recupera.</t>
+          <t>El buscador deja los acordes que empiezan por lo escrito, sin distinguir mayúsculas y en las dos nomenclaturas; una letra sola, solo en la inglesa.</t>
         </is>
       </c>
       <c r="J94" s="5" t="inlineStr">
@@ -7688,12 +7688,12 @@
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.5.5</t>
         </is>
       </c>
       <c r="L94" s="5" t="inlineStr">
         <is>
-          <t>V-06: comprobar-disposicion.js en 14 pantallas: 52,8 / 60,8 / 42,5 px · Banco (node --test): aviso para girar · Sesión 1: C02, C03 y D03</t>
+          <t>Banco (node --test): G, g, Sol, D, Am, f# y vacío</t>
         </is>
       </c>
       <c r="M94" s="5" t="inlineStr">
@@ -7703,21 +7703,21 @@
       </c>
       <c r="N94" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Banco automático + auditor técnico</t>
         </is>
       </c>
       <c r="O94" s="5" t="inlineStr">
         <is>
-          <t>Hecho en la 0.3.0 según interfaz.md §7. En horizontal, raíl, mástil a todo el alto y panel: medido en Chromium, 52,8 px por cuerda en el iPhone con Safari (antes 28,8), 60,8 con la app instalada y 42,5 en un Android de 280 px de alto (V-06). El aviso para girar sale solo con el dedo, en vertical y en pantallas de menos de 600 px de ancho, en Libre y Adivinar (y Escalas desde F5), en Libre, Adivinar, Escalas y Acordes; nunca en el Afinador ni en el Metrónomo; cerrado no vuelve y «Restablecer» lo recupera. El bloqueo de orientación tiene mal soporte en iOS, así que no se fuerza. Validado en la Sesión 1 (20/10, informe V-08): C02, C03 y D03.</t>
+          <t>Tu petición del 21/10. Una sola letra solo se busca en la nomenclatura inglesa, para que «D» no traiga también los Do; # y b valen por ♯ y ♭. Hecho en la 0.5.5 y validado por el banco.</t>
         </is>
       </c>
       <c r="P94" s="6" t="n"/>
       <c r="Q94" s="5" t="inlineStr"/>
     </row>
-    <row r="95" ht="33" customHeight="1">
+    <row r="95" ht="120" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>V-02</t>
+          <t>V-01</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -7727,7 +7727,7 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>El afinador funciona en vertical y en horizontal.</t>
+          <t>En móvil se sugiere la orientación horizontal con un aviso discreto; no se fuerza.</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
@@ -7737,17 +7737,17 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>F1.1</t>
+          <t>F3.2</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="I95" s="5" t="inlineStr">
         <is>
-          <t>El afinador se usa con comodidad en vertical y en horizontal.</t>
+          <t>En horizontal, con un alto útil de 268 px o más, cada cuerda mide al menos 40 px (iPhone en Safari e instalada; simulador de Android). En vertical, en pantallas táctiles de menos de 600 px de ancho y en Libre, Adivinar, Escalas y Acordes, aparece el aviso para girar; nunca en el Afinador ni en el Metrónomo; cerrado, no vuelve y «Restablecer» lo recupera.</t>
         </is>
       </c>
       <c r="J95" s="5" t="inlineStr">
@@ -7767,17 +7767,17 @@
       </c>
       <c r="K95" s="5" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="L95" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>V-06: comprobar-disposicion.js en 14 pantallas: 52,8 / 60,8 / 42,5 px · Banco (node --test): aviso para girar · Sesión 1: C02, C03 y D03</t>
         </is>
       </c>
       <c r="M95" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N95" s="5" t="inlineStr">
@@ -7785,14 +7785,18 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O95" s="5" t="inlineStr"/>
+      <c r="O95" s="5" t="inlineStr">
+        <is>
+          <t>Hecho en la 0.3.0 según interfaz.md §7. En horizontal, raíl, mástil a todo el alto y panel: medido en Chromium, 52,8 px por cuerda en el iPhone con Safari (antes 28,8), 60,8 con la app instalada y 42,5 en un Android de 280 px de alto (V-06). El aviso para girar sale solo con el dedo, en vertical y en pantallas de menos de 600 px de ancho, en Libre y Adivinar (y Escalas desde F5), en Libre, Adivinar, Escalas y Acordes; nunca en el Afinador ni en el Metrónomo; cerrado no vuelve y «Restablecer» lo recupera. El bloqueo de orientación tiene mal soporte en iOS, así que no se fuerza. Validado en la Sesión 1 (20/10, informe V-08): C02, C03 y D03.</t>
+        </is>
+      </c>
       <c r="P95" s="6" t="n"/>
       <c r="Q95" s="5" t="inlineStr"/>
     </row>
     <row r="96" ht="33" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>V-03</t>
+          <t>V-02</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
@@ -7802,7 +7806,7 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>En escritorio el mástil aprovecha el ancho disponible.</t>
+          <t>El afinador funciona en vertical y en horizontal.</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
@@ -7832,7 +7836,7 @@
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>En una pantalla de 1280 px se ven los 24 trastes sin desplazarse.</t>
+          <t>El afinador se usa con comodidad en vertical y en horizontal.</t>
         </is>
       </c>
       <c r="J96" s="5" t="inlineStr">
@@ -7860,18 +7864,14 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O96" s="5" t="inlineStr">
-        <is>
-          <t>Arranca mostrando el mástil completo en pantallas anchas.</t>
-        </is>
-      </c>
+      <c r="O96" s="5" t="inlineStr"/>
       <c r="P96" s="6" t="n"/>
       <c r="Q96" s="5" t="inlineStr"/>
     </row>
-    <row r="97" ht="120" customHeight="1">
+    <row r="97" ht="33" customHeight="1">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>V-04</t>
+          <t>V-03</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Control de zoom que determina qué porción del mástil se ve.</t>
+          <t>En escritorio el mástil aprovecha el ancho disponible.</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
@@ -7891,17 +7891,17 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
+          <t>Cliente · listado 14/09</t>
         </is>
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>F1 · F3</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>F1.1 · F3.2</t>
+          <t>F1.1</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="I97" s="5" t="inlineStr">
         <is>
-          <t>El zoom cambia los trastes visibles entre 3 y el máximo que cabe, y la etiqueta dice la cifra real; «+» enseña más trastes y «−» menos. Con pointer: coarse, la vista por defecto usa trastes de al menos 40 px y el usuario puede pedir más trastes, de hasta 28 px; si el zoom guardado pide más de los que caben, se muestran los que caben y lo guardado se conserva (V-08).</t>
+          <t>En una pantalla de 1280 px se ven los 24 trastes sin desplazarse.</t>
         </is>
       </c>
       <c r="J97" s="5" t="inlineStr">
@@ -7926,12 +7926,12 @@
       </c>
       <c r="L97" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7 y #8 · V-06 · Banco (node --test): 40 px por defecto, 28 con «+», orden de los botones · Sesión 1: A07, A08 y C04</t>
+          <t>F1.1 #14</t>
         </is>
       </c>
       <c r="M97" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="N97" s="5" t="inlineStr">
@@ -7941,16 +7941,16 @@
       </c>
       <c r="O97" s="5" t="inlineStr">
         <is>
-          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Desde la 0.3.0, con el dedo la vista por defecto usa trastes de 40 px o más (34 con ratón), y la cejuela mide 40. Desde la 0.3.2 (tu comentario del 20/10), «+» enseña más trastes y «−» menos, y con el dedo puedes pedir trastes de hasta 28 px: en el iPhone con Safari, hasta 11 a la vista en vertical y 15 en horizontal. Si el zoom guardado pide más, se muestran los que caben y la etiqueta lo dice, pero lo guardado se conserva para que al girar vuelva (V-08). Validado en la Sesión 1 (20/10, informe V-08): A07, A08 y C04.</t>
+          <t>Arranca mostrando el mástil completo en pantallas anchas.</t>
         </is>
       </c>
       <c r="P97" s="6" t="n"/>
       <c r="Q97" s="5" t="inlineStr"/>
     </row>
-    <row r="98" ht="33" customHeight="1">
+    <row r="98" ht="120" customHeight="1">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>V-05</t>
+          <t>V-04</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
@@ -7960,7 +7960,7 @@
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>Cuando el mástil no cabe, el usuario se desplaza lateralmente.</t>
+          <t>Control de zoom que determina qué porción del mástil se ve.</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
@@ -7970,17 +7970,17 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F1 · F3</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
         <is>
-          <t>F1.1</t>
+          <t>F1.1 · F3.2</t>
         </is>
       </c>
       <c r="H98" s="5" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="I98" s="5" t="inlineStr">
         <is>
-          <t>Con el mástil más ancho que la pantalla se puede desplazar hasta el traste 24.</t>
+          <t>El zoom cambia los trastes visibles entre 3 y el máximo que cabe, y la etiqueta dice la cifra real; «+» enseña más trastes y «−» menos. Con pointer: coarse, la vista por defecto usa trastes de al menos 40 px y el usuario puede pedir más trastes, de hasta 28 px; si el zoom guardado pide más de los que caben, se muestran los que caben y lo guardado se conserva (V-08).</t>
         </is>
       </c>
       <c r="J98" s="5" t="inlineStr">
@@ -8000,12 +8000,12 @@
       </c>
       <c r="K98" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A08.</t>
+          <t>0.1.0</t>
         </is>
       </c>
       <c r="L98" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14 · Sesión 1: A08</t>
+          <t>F1.1 #7 y #8 · V-06 · Banco (node --test): 40 px por defecto, 28 con «+», orden de los botones · Sesión 1: A07, A08 y C04</t>
         </is>
       </c>
       <c r="M98" s="5" t="inlineStr">
@@ -8018,14 +8018,18 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O98" s="5" t="inlineStr"/>
+      <c r="O98" s="5" t="inlineStr">
+        <is>
+          <t>De 3 a 24 trastes a la vista. Desde 0.1.1 la etiqueta indica los trastes que caben de verdad, y el zoom conserva el tramo que estabas mirando. Desde la 0.3.0, con el dedo la vista por defecto usa trastes de 40 px o más (34 con ratón), y la cejuela mide 40. Desde la 0.3.2 (tu comentario del 20/10), «+» enseña más trastes y «−» menos, y con el dedo puedes pedir trastes de hasta 28 px: en el iPhone con Safari, hasta 11 a la vista en vertical y 15 en horizontal. Si el zoom guardado pide más, se muestran los que caben y la etiqueta lo dice, pero lo guardado se conserva para que al girar vuelva (V-08). Validado en la Sesión 1 (20/10, informe V-08): A07, A08 y C04.</t>
+        </is>
+      </c>
       <c r="P98" s="6" t="n"/>
       <c r="Q98" s="5" t="inlineStr"/>
     </row>
-    <row r="99" ht="48" customHeight="1">
+    <row r="99" ht="33" customHeight="1">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>V-06</t>
+          <t>V-05</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -8035,7 +8039,7 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>El ancho de traste no cambia al desplazarse: el zoom fija el tamaño y el desplazamiento mueve la ventana.</t>
+          <t>Cuando el mástil no cabe, el usuario se desplaza lateralmente.</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
@@ -8065,7 +8069,7 @@
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>Desplazarse no cambia el ancho de los trastes.</t>
+          <t>Con el mástil más ancho que la pantalla se puede desplazar hasta el traste 24.</t>
         </is>
       </c>
       <c r="J99" s="5" t="inlineStr">
@@ -8075,12 +8079,12 @@
       </c>
       <c r="K99" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A07.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A08.</t>
         </is>
       </c>
       <c r="L99" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7 · Sesión 1: A07</t>
+          <t>F1.1 #14 · Sesión 1: A08</t>
         </is>
       </c>
       <c r="M99" s="5" t="inlineStr">
@@ -8097,10 +8101,10 @@
       <c r="P99" s="6" t="n"/>
       <c r="Q99" s="5" t="inlineStr"/>
     </row>
-    <row r="100" ht="33" customHeight="1">
+    <row r="100" ht="48" customHeight="1">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>V-07</t>
+          <t>V-06</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
@@ -8110,7 +8114,7 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>El mástil se readapta al redimensionar la ventana.</t>
+          <t>El ancho de traste no cambia al desplazarse: el zoom fija el tamaño y el desplazamiento mueve la ventana.</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
@@ -8140,7 +8144,7 @@
       </c>
       <c r="I100" s="5" t="inlineStr">
         <is>
-          <t>Al redimensionar la ventana el mástil se reajusta sin perder el tramo visible.</t>
+          <t>Desplazarse no cambia el ancho de los trastes.</t>
         </is>
       </c>
       <c r="J100" s="5" t="inlineStr">
@@ -8150,12 +8154,12 @@
       </c>
       <c r="K100" s="5" t="inlineStr">
         <is>
-          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A08.</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A07.</t>
         </is>
       </c>
       <c r="L100" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #7 · Sesión 1: A08</t>
+          <t>F1.1 #7 · Sesión 1: A07</t>
         </is>
       </c>
       <c r="M100" s="5" t="inlineStr">
@@ -8175,7 +8179,7 @@
     <row r="101" ht="33" customHeight="1">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>V-08</t>
+          <t>V-07</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -8185,12 +8189,12 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>El nivel de zoom persiste entre sesiones.</t>
+          <t>El mástil se readapta al redimensionar la ventana.</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -8215,7 +8219,7 @@
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>El zoom se mantiene tras recargar y tras girar el móvil.</t>
+          <t>Al redimensionar la ventana el mástil se reajusta sin perder el tramo visible.</t>
         </is>
       </c>
       <c r="J101" s="5" t="inlineStr">
@@ -8225,17 +8229,17 @@
       </c>
       <c r="K101" s="5" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>0.1.0 **Validado en la Sesión 1** (20/10, informe `V-08`): A08.</t>
         </is>
       </c>
       <c r="L101" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #13</t>
+          <t>F1.1 #7 · Sesión 1: A08</t>
         </is>
       </c>
       <c r="M101" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N101" s="5" t="inlineStr">
@@ -8243,18 +8247,14 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="O101" s="5" t="inlineStr">
-        <is>
-          <t>Desde 0.1.1 girar el móvil ya no pisa el zoom elegido.</t>
-        </is>
-      </c>
+      <c r="O101" s="5" t="inlineStr"/>
       <c r="P101" s="6" t="n"/>
       <c r="Q101" s="5" t="inlineStr"/>
     </row>
-    <row r="102" ht="63" customHeight="1">
+    <row r="102" ht="33" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>V-09</t>
+          <t>V-08</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
@@ -8264,17 +8264,17 @@
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>Al ocultar la numeración se puede conservar una referencia de tramo: el modo «Guía» deja solo los números de los trastes con marca.</t>
+          <t>El nivel de zoom persiste entre sesiones.</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>AR-01</t>
+          <t>Cliente · listado 14/09</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
@@ -8284,17 +8284,17 @@
       </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
-          <t>F1.3</t>
+          <t>F1.1</t>
         </is>
       </c>
       <c r="H102" s="5" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>D</t>
         </is>
       </c>
       <c r="I102" s="5" t="inlineStr">
         <is>
-          <t>El modo Guía mantiene visibles solo los números de los trastes con marca.</t>
+          <t>El zoom se mantiene tras recargar y tras girar el móvil.</t>
         </is>
       </c>
       <c r="J102" s="5" t="inlineStr">
@@ -8304,56 +8304,56 @@
       </c>
       <c r="K102" s="5" t="inlineStr">
         <is>
-          <t>0.1.2</t>
+          <t>0.1.0</t>
         </is>
       </c>
       <c r="L102" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test) · F1.1 #11 · Sesión 1: A11</t>
+          <t>F1.1 #13</t>
         </is>
       </c>
       <c r="M102" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="N102" s="5" t="inlineStr">
         <is>
-          <t>Banco automático + auditor técnico</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="O102" s="5" t="inlineStr">
         <is>
-          <t>Sin números, los trastes 5 y 17 llevan la misma marca y se confunden. Se descartó el minimapa por desproporcionado. Validado en la Sesión 1 (20/10, informe V-08): A11.</t>
+          <t>Desde 0.1.1 girar el móvil ya no pisa el zoom elegido.</t>
         </is>
       </c>
       <c r="P102" s="6" t="n"/>
       <c r="Q102" s="5" t="inlineStr"/>
     </row>
-    <row r="103" ht="108" customHeight="1">
+    <row r="103" ht="63" customHeight="1">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>C-01</t>
+          <t>V-09</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>Configuración y navegación</t>
+          <t>Visualización</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Menú de configuración accesible desde cualquier pantalla.</t>
+          <t>Al ocultar la numeración se puede conservar una referencia de tramo: el modo «Guía» deja solo los números de los trastes con marca.</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>AR-01</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
@@ -8363,17 +8363,17 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>F1.1</t>
+          <t>F1.3</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T</t>
         </is>
       </c>
       <c r="I103" s="5" t="inlineStr">
         <is>
-          <t>El botón de Ajustes abre el panel desde cualquier pantalla y Escape lo cierra.</t>
+          <t>El modo Guía mantiene visibles solo los números de los trastes con marca.</t>
         </is>
       </c>
       <c r="J103" s="5" t="inlineStr">
@@ -8383,12 +8383,12 @@
       </c>
       <c r="K103" s="5" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>0.1.2</t>
         </is>
       </c>
       <c r="L103" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14 · Sesión 1: A19 y C05</t>
+          <t>Banco (node --test) · F1.1 #11 · Sesión 1: A11</t>
         </is>
       </c>
       <c r="M103" s="5" t="inlineStr">
@@ -8398,21 +8398,21 @@
       </c>
       <c r="N103" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Banco automático + auditor técnico</t>
         </is>
       </c>
       <c r="O103" s="5" t="inlineStr">
         <is>
-          <t>Hoja que sube desde abajo en vertical; panel lateral en horizontal y en pantallas amplias, con un segundo botón en el raíl (0.3.0). Es un diálogo: mientras está abierto, el resto de la página no responde (AT-04). Validado en la Sesión 1 (20/10, informe V-08): A19 y C05.</t>
+          <t>Sin números, los trastes 5 y 17 llevan la misma marca y se confunden. Se descartó el minimapa por desproporcionado. Validado en la Sesión 1 (20/10, informe V-08): A11.</t>
         </is>
       </c>
       <c r="P103" s="6" t="n"/>
       <c r="Q103" s="5" t="inlineStr"/>
     </row>
-    <row r="104" ht="120" customHeight="1">
+    <row r="104" ht="108" customHeight="1">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>C-02</t>
+          <t>C-01</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>El menú contiene nomenclatura, pentagrama, timbre, numeración de trastes (tres modos), ver todas las notas, señalar iguales y afinación activa, y muestra la versión de la app.</t>
+          <t>Menú de configuración accesible desde cualquier pantalla.</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
@@ -8447,12 +8447,12 @@
       </c>
       <c r="H104" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>D</t>
         </is>
       </c>
       <c r="I104" s="5" t="inlineStr">
         <is>
-          <t>El panel contiene todos los ajustes listados, el idioma (0.4.2) y la versión de la app.</t>
+          <t>El botón de Ajustes abre el panel desde cualquier pantalla y Escape lo cierra.</t>
         </is>
       </c>
       <c r="J104" s="5" t="inlineStr">
@@ -8467,31 +8467,31 @@
       </c>
       <c r="L104" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #12 · Banco (node --test): grupo Idioma</t>
+          <t>F1.1 #14 · Sesión 1: A19 y C05</t>
         </is>
       </c>
       <c r="M104" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N104" s="5" t="inlineStr">
         <is>
-          <t>Auditor de requisitos</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="O104" s="5" t="inlineStr">
         <is>
-          <t>Ampliado en 0.1.2 con la numeración en tres modos y la versión (G-10). En F6.4 se añade el grupo «Acerca de», con los créditos (G-06) y la privacidad (G-11) (interfaz.md v1.0, aprobada el 20/10). Desde la 0.4.2, Ajustes empieza con el grupo «Idioma · Language» (G-12). Tiene también «Al fallar» en Adivinar (J-13, 0.5.1) y «Notas alteradas», ♯ o ♭ por tecla negra (N-06, 0.5.2).</t>
+          <t>Hoja que sube desde abajo en vertical; panel lateral en horizontal y en pantallas amplias, con un segundo botón en el raíl (0.3.0). Es un diálogo: mientras está abierto, el resto de la página no responde (AT-04). Validado en la Sesión 1 (20/10, informe V-08): A19 y C05.</t>
         </is>
       </c>
       <c r="P104" s="6" t="n"/>
       <c r="Q104" s="5" t="inlineStr"/>
     </row>
-    <row r="105" ht="78" customHeight="1">
+    <row r="105" ht="120" customHeight="1">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>C-03</t>
+          <t>C-02</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
@@ -8501,7 +8501,7 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Los ajustes frecuentes tienen acceso rápido sin abrir el menú.</t>
+          <t>El menú contiene nomenclatura, pentagrama, timbre, numeración de trastes (tres modos), ver todas las notas, señalar iguales y afinación activa, y muestra la versión de la app.</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
@@ -8526,12 +8526,12 @@
       </c>
       <c r="H105" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>I</t>
         </is>
       </c>
       <c r="I105" s="5" t="inlineStr">
         <is>
-          <t>Nomenclatura, pentagrama y pistas tienen chips de acceso rápido.</t>
+          <t>El panel contiene todos los ajustes listados, el idioma (0.4.2) y la versión de la app.</t>
         </is>
       </c>
       <c r="J105" s="5" t="inlineStr">
@@ -8546,7 +8546,7 @@
       </c>
       <c r="L105" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14</t>
+          <t>F1.1 #12 · Banco (node --test): grupo Idioma</t>
         </is>
       </c>
       <c r="M105" s="5" t="inlineStr">
@@ -8556,21 +8556,21 @@
       </c>
       <c r="N105" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Auditor de requisitos</t>
         </is>
       </c>
       <c r="O105" s="5" t="inlineStr">
         <is>
-          <t>Nomenclatura y pentagrama en chips bajo la cabecera, o en el panel en horizontal, donde el pentagrama se rotula con la clave de sol; las dos pistas del juego, en la tarjeta del reto (0.3.0).</t>
+          <t>Ampliado en 0.1.2 con la numeración en tres modos y la versión (G-10). En F6.4 se añade el grupo «Acerca de», con los créditos (G-06) y la privacidad (G-11) (interfaz.md v1.0, aprobada el 20/10). Desde la 0.4.2, Ajustes empieza con el grupo «Idioma · Language» (G-12). Tiene también «Al fallar» en Adivinar (J-13, 0.5.1) y «Notas alteradas», ♯ o ♭ por tecla negra (N-06, 0.5.2).</t>
         </is>
       </c>
       <c r="P105" s="6" t="n"/>
       <c r="Q105" s="5" t="inlineStr"/>
     </row>
-    <row r="106" ht="120" customHeight="1">
+    <row r="106" ht="78" customHeight="1">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>C-04</t>
+          <t>C-03</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
@@ -8580,7 +8580,7 @@
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>Navegación principal clara entre las áreas de la app.</t>
+          <t>Los ajustes frecuentes tienen acceso rápido sin abrir el menú.</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
@@ -8590,7 +8590,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
+          <t>Cliente · listado 14/09</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="I106" s="5" t="inlineStr">
         <is>
-          <t>La navegación (barra inferior, raíl o pestañas en la cabecera, según la disposición) lleva a cada área con un toque.</t>
+          <t>Nomenclatura, pentagrama y pistas tienen chips de acceso rápido.</t>
         </is>
       </c>
       <c r="J106" s="5" t="inlineStr">
@@ -8625,12 +8625,12 @@
       </c>
       <c r="L106" s="5" t="inlineStr">
         <is>
-          <t>F1.1 #14 · 0.5.5: comprobar-disposicion, seis pestañas sin salirse ni pisar el nombre · Sesión 1: A19</t>
+          <t>F1.1 #14</t>
         </is>
       </c>
       <c r="M106" s="5" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="N106" s="5" t="inlineStr">
@@ -8640,16 +8640,16 @@
       </c>
       <c r="O106" s="5" t="inlineStr">
         <is>
-          <t>Barra inferior con un destino por área en vertical (seis desde la 0.5.5, con Metrónomo y Acordes; en el raíl, pestañas de 44 px; entre 600 y 959 px, las pestañas se alinean a la derecha), raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05). Validado en la Sesión 1 (20/10, informe V-08): A19.</t>
+          <t>Nomenclatura y pentagrama en chips bajo la cabecera, o en el panel en horizontal, donde el pentagrama se rotula con la clave de sol; las dos pistas del juego, en la tarjeta del reto (0.3.0).</t>
         </is>
       </c>
       <c r="P106" s="6" t="n"/>
       <c r="Q106" s="5" t="inlineStr"/>
     </row>
-    <row r="107" ht="48" customHeight="1">
+    <row r="107" ht="120" customHeight="1">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>C-05</t>
+          <t>C-04</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
@@ -8659,17 +8659,17 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Todos los ajustes persisten entre sesiones.</t>
+          <t>Navegación principal clara entre las áreas de la app.</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
       <c r="F107" s="5" t="inlineStr">
@@ -8684,12 +8684,12 @@
       </c>
       <c r="H107" s="5" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>D</t>
         </is>
       </c>
       <c r="I107" s="5" t="inlineStr">
         <is>
-          <t>Todos los ajustes persisten tras recargar, y unos ajustes corruptos o antiguos no rompen la app.</t>
+          <t>La navegación (barra inferior, raíl o pestañas en la cabecera, según la disposición) lleva a cada área con un toque.</t>
         </is>
       </c>
       <c r="J107" s="5" t="inlineStr">
@@ -8704,7 +8704,7 @@
       </c>
       <c r="L107" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): migración · F1.1 #13 · Sesión 1: A14 y A15</t>
+          <t>F1.1 #14 · 0.5.5: comprobar-disposicion, seis pestañas sin salirse ni pisar el nombre · Sesión 1: A19</t>
         </is>
       </c>
       <c r="M107" s="5" t="inlineStr">
@@ -8714,21 +8714,21 @@
       </c>
       <c r="N107" s="5" t="inlineStr">
         <is>
-          <t>Banco automático + auditor técnico</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="O107" s="5" t="inlineStr">
         <is>
-          <t>Un único objeto de estado, validado campo a campo al leerlo (0.1.1). Validado en la Sesión 1 (20/10, informe V-08): A14 y A15.</t>
+          <t>Barra inferior con un destino por área en vertical (seis desde la 0.5.5, con Metrónomo y Acordes; en el raíl, pestañas de 44 px; entre 600 y 959 px, las pestañas se alinean a la derecha), raíl a la izquierda en horizontal y pestañas en la cabecera en pantallas amplias (0.3.0). En pantallas bajas la barra nunca se sale (AR-05). Validado en la Sesión 1 (20/10, informe V-08): A19.</t>
         </is>
       </c>
       <c r="P107" s="6" t="n"/>
       <c r="Q107" s="5" t="inlineStr"/>
     </row>
-    <row r="108" ht="93" customHeight="1">
+    <row r="108" ht="48" customHeight="1">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>C-06</t>
+          <t>C-05</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
@@ -8738,12 +8738,12 @@
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>Especificación detallada de la interfaz: estructura de menús, jerarquía de controles y flujos de navegación.</t>
+          <t>Todos los ajustes persisten entre sesiones.</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -8753,22 +8753,22 @@
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="G108" s="5" t="inlineStr">
         <is>
-          <t>F3.1</t>
+          <t>F1.1</t>
         </is>
       </c>
       <c r="H108" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>T</t>
         </is>
       </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>interfaz.md aprobado por el cliente y revisado por el auditor de requisitos.</t>
+          <t>Todos los ajustes persisten tras recargar, y unos ajustes corruptos o antiguos no rompen la app.</t>
         </is>
       </c>
       <c r="J108" s="5" t="inlineStr">
@@ -8778,12 +8778,12 @@
       </c>
       <c r="K108" s="5" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.1.0</t>
         </is>
       </c>
       <c r="L108" s="5" t="inlineStr">
         <is>
-          <t>interfaz.md v1.0 · AR-04 · aprobación del cliente el 20/10</t>
+          <t>Banco (node --test): migración · F1.1 #13 · Sesión 1: A14 y A15</t>
         </is>
       </c>
       <c r="M108" s="5" t="inlineStr">
@@ -8793,21 +8793,21 @@
       </c>
       <c r="N108" s="5" t="inlineStr">
         <is>
-          <t>Auditor de requisitos</t>
+          <t>Banco automático + auditor técnico</t>
         </is>
       </c>
       <c r="O108" s="5" t="inlineStr">
         <is>
-          <t>docs/interfaz.md v1.0, aprobada por ti el 20/10 tras la auditoría AR-04 (10 hallazgos resueltos). Bocetos al tamaño real de cada pantalla en docs/interfaz/, comprobados por herramientas/capturar-wireframes.js. Los cambios posteriores suben su versión.</t>
+          <t>Un único objeto de estado, validado campo a campo al leerlo (0.1.1). Validado en la Sesión 1 (20/10, informe V-08): A14 y A15.</t>
         </is>
       </c>
       <c r="P108" s="6" t="n"/>
       <c r="Q108" s="5" t="inlineStr"/>
     </row>
-    <row r="109" ht="120" customHeight="1">
+    <row r="109" ht="93" customHeight="1">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>C-07</t>
+          <t>C-06</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
@@ -8817,17 +8817,17 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Botón «atrás» del sistema: mientras haya un paso anterior en la sesión, el botón o gesto «atrás» cierra Ajustes o vuelve al área anterior; desde la primera área actúa el sistema. Al abrir la app se entra en Libre.</t>
+          <t>Especificación detallada de la interfaz: estructura de menús, jerarquía de controles y flujos de navegación.</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
+          <t>Cliente · listado 14/09</t>
         </is>
       </c>
       <c r="F109" s="5" t="inlineStr">
@@ -8837,17 +8837,17 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>F3.2</t>
+          <t>F3.1</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>I</t>
         </is>
       </c>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>Con un paso anterior en la sesión, «atrás» cierra Ajustes o vuelve al área anterior; desde la primera área actúa el sistema; al abrir o recargar se entra en Libre. Prueba manual en Windows y en el simulador de Android de Chrome.</t>
+          <t>interfaz.md aprobado por el cliente y revisado por el auditor de requisitos.</t>
         </is>
       </c>
       <c r="J109" s="5" t="inlineStr">
@@ -8857,12 +8857,12 @@
       </c>
       <c r="K109" s="5" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="L109" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): historial simulado con popstate (3 pruebas) · Sesión 1: A17</t>
+          <t>interfaz.md v1.0 · AR-04 · aprobación del cliente el 20/10</t>
         </is>
       </c>
       <c r="M109" s="5" t="inlineStr">
@@ -8872,21 +8872,21 @@
       </c>
       <c r="N109" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Auditor de requisitos</t>
         </is>
       </c>
       <c r="O109" s="5" t="inlineStr">
         <is>
-          <t>Hecho en la 0.3.0 con el historial del navegador (history): cada área tiene su dirección (#libre, #adivinar…). Un paso que deja la misma área, como tras recargar, se salta. El banco lo prueba con un historial simulado que avisa como el de verdad. Falta la prueba a mano en Windows y en el simulador de Android (Sesión 1). En el iPhone instalado no hay botón atrás. Validado en la Sesión 1 (20/10, informe V-08): A17.</t>
+          <t>docs/interfaz.md v1.0, aprobada por ti el 20/10 tras la auditoría AR-04 (10 hallazgos resueltos). Bocetos al tamaño real de cada pantalla en docs/interfaz/, comprobados por herramientas/capturar-wireframes.js. Los cambios posteriores suben su versión.</t>
         </is>
       </c>
       <c r="P109" s="6" t="n"/>
       <c r="Q109" s="5" t="inlineStr"/>
     </row>
-    <row r="110" ht="93" customHeight="1">
+    <row r="110" ht="120" customHeight="1">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>C-08</t>
+          <t>C-07</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
@@ -8896,7 +8896,7 @@
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>Menú Personalización dentro de Ajustes: estilos de nota en el mástil (círculo de color o solo el nombre, más grande o en negrita), estilo del traste y del mástil, interior claro para «Ver todas las notas» y temas de color de la app.</t>
+          <t>Botón «atrás» del sistema: mientras haya un paso anterior en la sesión, el botón o gesto «atrás» cierra Ajustes o vuelve al área anterior; desde la primera área actúa el sistema. Al abrir la app se entra en Libre.</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
@@ -8906,145 +8906,145 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>Cliente · listado 14/09</t>
+          <t>Cliente · 20/10 (interfaz.md v1.0)</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="G110" s="5" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>F3.2</t>
         </is>
       </c>
       <c r="H110" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>Fuera del alcance actual.</t>
+          <t>Con un paso anterior en la sesión, «atrás» cierra Ajustes o vuelve al área anterior; desde la primera área actúa el sistema; al abrir o recargar se entra en Libre. Prueba manual en Windows y en el simulador de Android de Chrome.</t>
         </is>
       </c>
       <c r="J110" s="5" t="inlineStr">
         <is>
-          <t>No aplica</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K110" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="L110" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Banco (node --test): historial simulado con popstate (3 pruebas) · Sesión 1: A17</t>
         </is>
       </c>
       <c r="M110" s="5" t="inlineStr">
         <is>
-          <t>No aplica</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="N110" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="O110" s="5" t="inlineStr">
         <is>
-          <t>Tus comentarios de la Sesión 1 (A10, C06 y E06), para una actualización posterior. La paleta por nota de G-05 se mantiene como punto de partida.</t>
+          <t>Hecho en la 0.3.0 con el historial del navegador (history): cada área tiene su dirección (#libre, #adivinar…). Un paso que deja la misma área, como tras recargar, se salta. El banco lo prueba con un historial simulado que avisa como el de verdad. Falta la prueba a mano en Windows y en el simulador de Android (Sesión 1). En el iPhone instalado no hay botón atrás. Validado en la Sesión 1 (20/10, informe V-08): A17.</t>
         </is>
       </c>
       <c r="P110" s="6" t="n"/>
       <c r="Q110" s="5" t="inlineStr"/>
     </row>
-    <row r="111" ht="78" customHeight="1">
+    <row r="111" ht="93" customHeight="1">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>X-01</t>
+          <t>C-08</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>Respaldo y publicación</t>
+          <t>Configuración y navegación</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>El código y la documentación están respaldados en el repositorio remoto (GitHub). Respaldar no es publicar.</t>
+          <t>Menú Personalización dentro de Ajustes: estilos de nota en el mástil (círculo de color o solo el nombre, más grande o en negrita), estilo del traste y del mástil, interior claro para «Ver todas las notas» y temas de color de la app.</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>Desarrollo · v1.1</t>
+          <t>Cliente · listado 14/09</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>Posterior</t>
         </is>
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>F1.2 · F1.4</t>
+          <t>Posterior</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>GitHub muestra la última versión en main, entrada por pull request aprobado, y la etiqueta de cierre de fase.</t>
+          <t>Fuera del alcance actual.</t>
         </is>
       </c>
       <c r="J111" s="5" t="inlineStr">
         <is>
-          <t>Cumple</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="K111" s="5" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L111" s="5" t="inlineStr">
         <is>
-          <t>PR #1 a #5 fusionados · etiqueta v0.1.5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M111" s="5" t="inlineStr">
         <is>
-          <t>Verificado parcialmente</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="N111" s="5" t="inlineStr">
         <is>
-          <t>Auditor de requisitos</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O111" s="5" t="inlineStr">
         <is>
-          <t>Desde el 15/10 todo el proyecto está en pdigue/guitarra; cada versión entra por pull request aprobado (del #1 al #5) y F1 se cerró con la etiqueta v0.1.5. El repositorio es público.</t>
+          <t>Tus comentarios de la Sesión 1 (A10, C06 y E06), para una actualización posterior. La paleta por nota de G-05 se mantiene como punto de partida.</t>
         </is>
       </c>
       <c r="P111" s="6" t="n"/>
       <c r="Q111" s="5" t="inlineStr"/>
     </row>
-    <row r="112" ht="120" customHeight="1">
+    <row r="112" ht="78" customHeight="1">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>X-02</t>
+          <t>X-01</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
@@ -9054,7 +9054,7 @@
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>La app está publicada en una URL pública (GitHub Pages).</t>
+          <t>El código y la documentación están respaldados en el repositorio remoto (GitHub). Respaldar no es publicar.</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
@@ -9069,61 +9069,61 @@
       </c>
       <c r="F112" s="5" t="inlineStr">
         <is>
-          <t>F7</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="G112" s="5" t="inlineStr">
         <is>
-          <t>F7.1</t>
+          <t>F1.2 · F1.4</t>
         </is>
       </c>
       <c r="H112" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>I</t>
         </is>
       </c>
       <c r="I112" s="5" t="inlineStr">
         <is>
-          <t>La URL pública carga la app desde un dispositivo ajeno al proyecto.</t>
+          <t>GitHub muestra la última versión en main, entrada por pull request aprobado, y la etiqueta de cierre de fase.</t>
         </is>
       </c>
       <c r="J112" s="5" t="inlineStr">
         <is>
-          <t>No cumple</t>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="K112" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.1.4</t>
         </is>
       </c>
       <c r="L112" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PR #1 a #5 fusionados · etiqueta v0.1.5</t>
         </is>
       </c>
       <c r="M112" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Verificado parcialmente</t>
         </is>
       </c>
       <c r="N112" s="5" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Auditor de requisitos</t>
         </is>
       </c>
       <c r="O112" s="5" t="inlineStr">
         <is>
-          <t>Antes en V1; pasa a la última fase por decisión del 15/09: desarrollo local de principio a fin. Despliegue de pruebas (decisión del 15/10): antes de la Sesión 1 se publica una versión de pruebas en GitHub Pages, sin anunciar, para probar en el iPhone con https la instalación, el modo sin conexión y el micrófono. X-02 sigue siendo la publicación oficial.</t>
+          <t>Desde el 15/10 todo el proyecto está en pdigue/guitarra; cada versión entra por pull request aprobado (del #1 al #5) y F1 se cerró con la etiqueta v0.1.5. El repositorio es público.</t>
         </is>
       </c>
       <c r="P112" s="6" t="n"/>
       <c r="Q112" s="5" t="inlineStr"/>
     </row>
-    <row r="113" ht="33" customHeight="1">
+    <row r="113" ht="120" customHeight="1">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>X-03</t>
+          <t>X-02</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>La app está verificada en móviles reales, instalada como icono desde la web publicada.</t>
+          <t>La app está publicada en una URL pública (GitHub Pages).</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
@@ -9153,7 +9153,7 @@
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>F7.2</t>
+          <t>F7.1</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr">
@@ -9163,7 +9163,7 @@
       </c>
       <c r="I113" s="5" t="inlineStr">
         <is>
-          <t>La app instalada desde la web funciona en un Android, un iPhone y un Windows reales.</t>
+          <t>La URL pública carga la app desde un dispositivo ajeno al proyecto.</t>
         </is>
       </c>
       <c r="J113" s="5" t="inlineStr">
@@ -9193,15 +9193,94 @@
       </c>
       <c r="O113" s="5" t="inlineStr">
         <is>
-          <t>Cierra G-04 y PL-01 a PL-03 en su modo web.</t>
+          <t>Antes en V1; pasa a la última fase por decisión del 15/09: desarrollo local de principio a fin. Despliegue de pruebas (decisión del 15/10): antes de la Sesión 1 se publica una versión de pruebas en GitHub Pages, sin anunciar, para probar en el iPhone con https la instalación, el modo sin conexión y el micrófono. X-02 sigue siendo la publicación oficial.</t>
         </is>
       </c>
       <c r="P113" s="6" t="n"/>
       <c r="Q113" s="5" t="inlineStr"/>
     </row>
+    <row r="114" ht="33" customHeight="1">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>X-03</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>Respaldo y publicación</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>La app está verificada en móviles reales, instalada como icono desde la web publicada.</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>Desarrollo · v1.1</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>F7.2</t>
+        </is>
+      </c>
+      <c r="H114" s="5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I114" s="5" t="inlineStr">
+        <is>
+          <t>La app instalada desde la web funciona en un Android, un iPhone y un Windows reales.</t>
+        </is>
+      </c>
+      <c r="J114" s="5" t="inlineStr">
+        <is>
+          <t>No cumple</t>
+        </is>
+      </c>
+      <c r="K114" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L114" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M114" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="N114" s="5" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="O114" s="5" t="inlineStr">
+        <is>
+          <t>Cierra G-04 y PL-01 a PL-03 en su modo web.</t>
+        </is>
+      </c>
+      <c r="P114" s="6" t="n"/>
+      <c r="Q114" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q113"/>
-  <conditionalFormatting sqref="J5:J113">
+  <autoFilter ref="A4:Q114"/>
+  <conditionalFormatting sqref="J5:J114">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>J5="Cumple"</formula>
     </cfRule>
@@ -9218,7 +9297,7 @@
       <formula>J5="No aplica"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M113">
+  <conditionalFormatting sqref="M5:M114">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>M5="Cumple"</formula>
     </cfRule>
@@ -9236,13 +9315,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="J5:J113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
+    <dataValidation sqref="J5:J114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
       <formula1>"Cumple,Cumple parcialmente,No cumple,No aplica"</formula1>
     </dataValidation>
-    <dataValidation sqref="M5:M113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
+    <dataValidation sqref="M5:M114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
       <formula1>"Verificado,Verificado parcialmente,Pendiente,No aplica"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
+    <dataValidation sqref="H5:H114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor no válido" error="Elige un valor de la lista. Están descritos en la hoja Leyenda." type="list">
       <formula1>"I,A,D,T,I+T,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9338,23 +9417,23 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$113,"*F1*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$114,"*F1*")</f>
         <v/>
       </c>
       <c r="C5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$J$5:$J$113,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F1*",Matriz!$J$5:$J$114,"Cumple")</f>
         <v/>
       </c>
       <c r="D5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F1*",Matriz!$J$5:$J$114,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$J$5:$J$113,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F1*",Matriz!$J$5:$J$114,"No cumple")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$J$5:$J$113,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F1*",Matriz!$J$5:$J$114,"No aplica")</f>
         <v/>
       </c>
       <c r="G5" s="8">
@@ -9362,11 +9441,11 @@
         <v/>
       </c>
       <c r="H5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$M$5:$M$113,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F1*",Matriz!$M$5:$M$114,"Verificado")</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F1*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F1*",Matriz!$M$5:$M$114,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9377,23 +9456,23 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$113,"*F2*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$114,"*F2*")</f>
         <v/>
       </c>
       <c r="C6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$J$5:$J$113,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F2*",Matriz!$J$5:$J$114,"Cumple")</f>
         <v/>
       </c>
       <c r="D6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F2*",Matriz!$J$5:$J$114,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$J$5:$J$113,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F2*",Matriz!$J$5:$J$114,"No cumple")</f>
         <v/>
       </c>
       <c r="F6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$J$5:$J$113,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F2*",Matriz!$J$5:$J$114,"No aplica")</f>
         <v/>
       </c>
       <c r="G6" s="8">
@@ -9401,11 +9480,11 @@
         <v/>
       </c>
       <c r="H6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$M$5:$M$113,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F2*",Matriz!$M$5:$M$114,"Verificado")</f>
         <v/>
       </c>
       <c r="I6" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F2*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F2*",Matriz!$M$5:$M$114,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9416,23 +9495,23 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$113,"*F3*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$114,"*F3*")</f>
         <v/>
       </c>
       <c r="C7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$J$5:$J$113,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F3*",Matriz!$J$5:$J$114,"Cumple")</f>
         <v/>
       </c>
       <c r="D7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F3*",Matriz!$J$5:$J$114,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$J$5:$J$113,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F3*",Matriz!$J$5:$J$114,"No cumple")</f>
         <v/>
       </c>
       <c r="F7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$J$5:$J$113,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F3*",Matriz!$J$5:$J$114,"No aplica")</f>
         <v/>
       </c>
       <c r="G7" s="8">
@@ -9440,11 +9519,11 @@
         <v/>
       </c>
       <c r="H7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$M$5:$M$113,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F3*",Matriz!$M$5:$M$114,"Verificado")</f>
         <v/>
       </c>
       <c r="I7" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F3*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F3*",Matriz!$M$5:$M$114,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9455,23 +9534,23 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$113,"*F4*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$114,"*F4*")</f>
         <v/>
       </c>
       <c r="C8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$J$5:$J$113,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F4*",Matriz!$J$5:$J$114,"Cumple")</f>
         <v/>
       </c>
       <c r="D8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F4*",Matriz!$J$5:$J$114,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$J$5:$J$113,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F4*",Matriz!$J$5:$J$114,"No cumple")</f>
         <v/>
       </c>
       <c r="F8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$J$5:$J$113,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F4*",Matriz!$J$5:$J$114,"No aplica")</f>
         <v/>
       </c>
       <c r="G8" s="8">
@@ -9479,11 +9558,11 @@
         <v/>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$M$5:$M$113,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F4*",Matriz!$M$5:$M$114,"Verificado")</f>
         <v/>
       </c>
       <c r="I8" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F4*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F4*",Matriz!$M$5:$M$114,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9494,23 +9573,23 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$113,"*F5*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$114,"*F5*")</f>
         <v/>
       </c>
       <c r="C9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$J$5:$J$113,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F5*",Matriz!$J$5:$J$114,"Cumple")</f>
         <v/>
       </c>
       <c r="D9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F5*",Matriz!$J$5:$J$114,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$J$5:$J$113,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F5*",Matriz!$J$5:$J$114,"No cumple")</f>
         <v/>
       </c>
       <c r="F9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$J$5:$J$113,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F5*",Matriz!$J$5:$J$114,"No aplica")</f>
         <v/>
       </c>
       <c r="G9" s="8">
@@ -9518,11 +9597,11 @@
         <v/>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$M$5:$M$113,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F5*",Matriz!$M$5:$M$114,"Verificado")</f>
         <v/>
       </c>
       <c r="I9" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F5*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F5*",Matriz!$M$5:$M$114,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9533,23 +9612,23 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$113,"*F6*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$114,"*F6*")</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$J$5:$J$113,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F6*",Matriz!$J$5:$J$114,"Cumple")</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F6*",Matriz!$J$5:$J$114,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$J$5:$J$113,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F6*",Matriz!$J$5:$J$114,"No cumple")</f>
         <v/>
       </c>
       <c r="F10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$J$5:$J$113,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F6*",Matriz!$J$5:$J$114,"No aplica")</f>
         <v/>
       </c>
       <c r="G10" s="8">
@@ -9557,11 +9636,11 @@
         <v/>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$M$5:$M$113,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F6*",Matriz!$M$5:$M$114,"Verificado")</f>
         <v/>
       </c>
       <c r="I10" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F6*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F6*",Matriz!$M$5:$M$114,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9572,23 +9651,23 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$113,"*F7*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$114,"*F7*")</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$J$5:$J$113,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F7*",Matriz!$J$5:$J$114,"Cumple")</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F7*",Matriz!$J$5:$J$114,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$J$5:$J$113,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F7*",Matriz!$J$5:$J$114,"No cumple")</f>
         <v/>
       </c>
       <c r="F11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$J$5:$J$113,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F7*",Matriz!$J$5:$J$114,"No aplica")</f>
         <v/>
       </c>
       <c r="G11" s="8">
@@ -9596,11 +9675,11 @@
         <v/>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$M$5:$M$113,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F7*",Matriz!$M$5:$M$114,"Verificado")</f>
         <v/>
       </c>
       <c r="I11" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*F7*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*F7*",Matriz!$M$5:$M$114,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9611,23 +9690,23 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Matriz!$F$5:$F$113,"*Posterior*")</f>
+        <f>COUNTIF(Matriz!$F$5:$F$114,"*Posterior*")</f>
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$J$5:$J$113,"Cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*Posterior*",Matriz!$J$5:$J$114,"Cumple")</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*Posterior*",Matriz!$J$5:$J$114,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$J$5:$J$113,"No cumple")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*Posterior*",Matriz!$J$5:$J$114,"No cumple")</f>
         <v/>
       </c>
       <c r="F12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$J$5:$J$113,"No aplica")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*Posterior*",Matriz!$J$5:$J$114,"No aplica")</f>
         <v/>
       </c>
       <c r="G12" s="8">
@@ -9635,11 +9714,11 @@
         <v/>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$M$5:$M$113,"Verificado")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*Posterior*",Matriz!$M$5:$M$114,"Verificado")</f>
         <v/>
       </c>
       <c r="I12" s="7">
-        <f>COUNTIFS(Matriz!$F$5:$F$113,"*Posterior*",Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
+        <f>COUNTIFS(Matriz!$F$5:$F$114,"*Posterior*",Matriz!$M$5:$M$114,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9650,23 +9729,23 @@
         </is>
       </c>
       <c r="B13" s="9">
-        <f>COUNTA(Matriz!$A$5:$A$113)</f>
+        <f>COUNTA(Matriz!$A$5:$A$114)</f>
         <v/>
       </c>
       <c r="C13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$113,"Cumple")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$114,"Cumple")</f>
         <v/>
       </c>
       <c r="D13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$113,"Cumple parcialmente")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$114,"Cumple parcialmente")</f>
         <v/>
       </c>
       <c r="E13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$113,"No cumple")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$114,"No cumple")</f>
         <v/>
       </c>
       <c r="F13" s="9">
-        <f>COUNTIF(Matriz!$J$5:$J$113,"No aplica")</f>
+        <f>COUNTIF(Matriz!$J$5:$J$114,"No aplica")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -9674,11 +9753,11 @@
         <v/>
       </c>
       <c r="H13" s="9">
-        <f>COUNTIF(Matriz!$M$5:$M$113,"Verificado")</f>
+        <f>COUNTIF(Matriz!$M$5:$M$114,"Verificado")</f>
         <v/>
       </c>
       <c r="I13" s="9">
-        <f>COUNTIF(Matriz!$M$5:$M$113,"Verificado parcialmente")</f>
+        <f>COUNTIF(Matriz!$M$5:$M$114,"Verificado parcialmente")</f>
         <v/>
       </c>
     </row>
@@ -9696,7 +9775,7 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$113,"I")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$114,"I")</f>
         <v/>
       </c>
     </row>
@@ -9707,7 +9786,7 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$113,"A")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$114,"A")</f>
         <v/>
       </c>
     </row>
@@ -9718,7 +9797,7 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$113,"D")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$114,"D")</f>
         <v/>
       </c>
     </row>
@@ -9729,7 +9808,7 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$113,"T")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$114,"T")</f>
         <v/>
       </c>
     </row>
@@ -9740,7 +9819,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$113,"I+T")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$114,"I+T")</f>
         <v/>
       </c>
     </row>
@@ -9751,7 +9830,7 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>COUNTIF(Matriz!$H$5:$H$113,"N/A")</f>
+        <f>COUNTIF(Matriz!$H$5:$H$114,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -9928,7 +10007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9968,7 +10047,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -9978,24 +10057,24 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>0.6.0</t>
+          <t>0.6.1</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>F6.1: G-08 cumple y queda verificado por el banco, que pasa las pruebas que arrancan la app contra la app de varios archivos y contra el archivo autónomo (AR-13 y AT-12).</t>
+          <t>F5.8, tu comentario #1: MT-06 nuevo, el péndulo del metrónomo (la pesa arriba, más lento). Verificado parcialmente hasta la Sesión 2.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -10005,51 +10084,51 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>0.5.7</t>
+          <t>0.6.0</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>Punto de control CP-5 (AR-12 y AT-11): una sola vara para lo que compruebas tú. E-01, E-02, E-03, E-04, E-06, P-03, MT-01, MT-05, AC-02 y AC-03, verificados parcialmente hasta la Sesión 2; MT-04, arranque con el audio en pausa (0.5.7); lo pendiente de CP-5, en el comentario de su requisito.</t>
+          <t>F6.1: G-08 cumple y queda verificado por el banco, que pasa las pruebas que arrancan la app contra la app de varios archivos y contra el archivo autónomo (AR-13 y AT-12).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>0.5.6</t>
+          <t>0.5.7</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>Auditoría AR-11: G-02, C-04 y V-01 con las seis áreas; criterio de AC-01 preciso (sus4 y tríadas); evidencias completadas en MT-01, MT-05, AC-01, AC-03 y AC-04 (método T).</t>
+          <t>Punto de control CP-5 (AR-12 y AT-11): una sola vara para lo que compruebas tú. E-01, E-02, E-03, E-04, E-06, P-03, MT-01, MT-05, AC-02 y AC-03, verificados parcialmente hasta la Sesión 2; MT-04, arranque con el audio en pausa (0.5.7); lo pendiente de CP-5, en el comentario de su requisito.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -10059,24 +10138,24 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>0.5.5</t>
+          <t>0.5.6</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>AC-01 a AC-05 implementados y verificados por el banco (F5.7); AC-06 nuevo, el buscador; criterios al día con tu guía del listado.</t>
+          <t>Auditoría AR-11: G-02, C-04 y V-01 con las seis áreas; criterio de AC-01 preciso (sus4 y tríadas); evidencias completadas en MT-01, MT-05, AC-01, AC-03 y AC-04 (método T).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -10086,24 +10165,24 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>0.5.4</t>
+          <t>0.5.5</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
+          <t>AC-01 a AC-05 implementados y verificados por el banco (F5.7); AC-06 nuevo, el buscador; criterios al día con tu guía del listado.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -10113,24 +10192,24 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>0.5.3</t>
+          <t>0.5.4</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
+          <t>MT-01 a MT-05 implementados y verificados por el banco (F5.6); criterios del metrónomo al día con tu guía: un solo acento, doce compases, figuras.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -10140,24 +10219,24 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>0.5.2</t>
+          <t>0.5.3</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
+          <t>J-13 por defecto «Reintentar»; MT-05, el metrónomo con su pestaña; criterios de MT-01, AC-02, G-02 y N-06 completados; evidencias nuevas de G-01, P-01, N-06 y J-13 (AR-10 y AT-09); origen de los requisitos del 21/10 corregido.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -10167,24 +10246,24 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>0.5.0</t>
+          <t>0.5.2</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
+          <t>J-13 y N-06 nuevos, verificados por el banco; criterios de MT-01 a MT-05 y AC-01 a AC-05 (planificados).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -10194,24 +10273,24 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>0.4.2</t>
+          <t>0.5.0</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
+          <t>F5: criterios y evidencias de E-01 a E-06 y P-03; E-02 y E-05 verificados por el banco; E-04 con los intervalos en la línea de notas.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -10221,51 +10300,51 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>0.4.0</t>
+          <t>0.4.2</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
+          <t>G-12 nuevo (idioma); J-11 con criterio de banco, verificado; criterios de J-01 (lectura de la nota tocada), J-06 (pistas grandes), J-08 (récords por afinación) y C-02 (idioma).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>20/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>0.3.3</t>
+          <t>0.4.0</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
+          <t>F4.1 a F4.3: evidencias del afinador por micrófono (A-02 a A-05, A-02-CA); A-02-CA y A-04 verificados por el banco; G-10 verificado con las etiquetas de F1 a F3.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -10275,24 +10354,24 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>0.3.2</t>
+          <t>0.3.3</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
+          <t>Sesión 1: 35 requisitos verificados en el iPhone y el PC del cliente (informe V-08), con la prueba que los valida en la evidencia. Criterios nuevos de J-01, J-08, J-10 y S-02 (pendientes de la Sesión 2); evidencia de S-01 (mudo en el iPhone) y PL-04; C-08 y S-09 nuevos, fuera de alcance.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -10302,24 +10381,24 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>0.3.1</t>
+          <t>0.3.2</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
+          <t>Criterios de V-04 y G-05: «+» enseña más trastes y el usuario puede pedir trastes de hasta 28 px con el dedo (comentario del cliente del 20/10).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -10329,24 +10408,24 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>0.3.0</t>
+          <t>0.3.1</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
+          <t>Etapa F3.4: G-05 cumple, verificado parcialmente hasta la Sesión 1. Su criterio añade los umbrales de la paleta (AR-06 #3).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -10356,24 +10435,24 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>0.2.3</t>
+          <t>0.3.0</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
+          <t>Etapa F3.2: V-01 y C-07 cumplen, verificados parcialmente hasta la Sesión 1. Criterios revisados: V-04 (lo guardado se conserva) y G-05 (excepción en vertical por debajo de 660 px de alto).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -10383,7 +10462,7 @@
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
@@ -10393,14 +10472,14 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
+          <t>Interfaz aprobada: C-06 verificado; C-07 nuevo; criterios revisados de V-01 (40 px con alto útil ≥ 268 px y aviso para girar), V-04 (trastes ≥ 40 px en pantallas táctiles), G-05 (controles de 40 × 40 px) y C-04 (navegación según la disposición).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -10410,7 +10489,7 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
@@ -10420,24 +10499,24 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
+          <t>S-07 cumple y queda verificado: licencia CC BY de los 161 sonidos del pack de nylon.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
@@ -10447,14 +10526,14 @@
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
+          <t>Evidencia de S-07: licencia de nylon comprobada en tres sonidos. Criterios sin cambios.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -10464,24 +10543,24 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>0.2.2</t>
+          <t>0.2.3</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
+          <t>CP-2: criterio de G-07 con los límites revisados y solo Windows y Android; X-01 cumple; evidencia de S-01 con la escucha del cliente (V-05).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -10491,24 +10570,24 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>v1.6</t>
+          <t>v1.7</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>0.2.1</t>
+          <t>0.2.2</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
+          <t>Criterio de S-08 según su nueva redacción: nota resultante a ±5 cents tras la corrección.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -10518,51 +10597,51 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>v1.5</t>
+          <t>v1.6</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>0.2.1</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
+          <t>G-07 y G-08 verificados parcialmente con el archivo autónomo (V-03 y banco); falta la prueba en cada plataforma (F2.5).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="46" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>v1.4</t>
+          <t>v1.5</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>0.1.4</t>
+          <t>0.2.0</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
+          <t>S-08 verificado: la app usa sus grabaciones medidas (F2.2). Evidencias nuevas en S-01, S-07 y S-08: banco con todas las notas y grabación en el navegador (V-02).</t>
         </is>
       </c>
     </row>
     <row r="24" ht="46" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -10572,7 +10651,7 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>v1.3</t>
+          <t>v1.4</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
@@ -10582,32 +10661,59 @@
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+          <t>Nuevo PL-04: adaptabilidad entre sistemas, con docs/compatibilidad.md como evidencia. PL-02 sin Android de pruebas por ahora; X-02 con despliegue de pruebas previo.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>0.1.4</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Nuevo S-08: afinación medida de cada muestra, verificado parcialmente hasta F2.2. Criterios revisados en CP-1: S-01, S-08, G-03, G-06 y A-02-CA. S-07 y G-06 pasan a «Cumple parcialmente» con CREDITOS.md y samples/. Las evidencias del banco apuntan a tests/ (node --test, 12 pruebas). Nueva comprobación F1.1 #15 para oír la corrección del registro agudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="46" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>0.1.2</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>Primera emisión. 90 requisitos con origen, método de verificación, criterio de aceptación, declaración del proveedor, evidencia y estado de verificación.</t>
         </is>

</xml_diff>

<commit_message>
F5.8 #1 ronda 1: correcciones de AR-14 y AT-13 (0.6.1, MT-06, MT-01, G-10)
- Tocar la pesa inclinada no cambia el tempo: el toque se proyecta sobre la
  varilla (AT-13 #1, AR-14 #3).
- La amplitud solo se mide con el área a la vista; resize la marca para medir
  de nuevo (AR-14 #1, AT-13 #2).
- proximoPulso: sin saltos al cambiar el tempo en marcha; setCompas no hace
  perder pulsos (AT-13 #3). Consulta de reducir movimiento única, capa propia
  y lostpointercapture (AT-13 #4, #6).
- Seis pruebas nuevas que fallan con la versión anterior; banco 168 de 168.
- Documentos: MT-06 con criterio preciso y lo pendiente; MT-01 remite a
  MT-06; G-10 con la regla de una fase reabierta; tabla «Comentarios de
  F5.8» y Sesión 2 en el roadmap; IT-03, interfaz, CHANGELOG, ESTADO;
  informes AR-14 y AT-13.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FozqoEELEJkBunkoec24Nq
</commit_message>
<xml_diff>
--- a/docs/matriz-cumplimiento.xlsx
+++ b/docs/matriz-cumplimiento.xlsx
@@ -1452,11 +1452,15 @@
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>Vincula cada versión con su fase del roadmap. Cada fase cerrada se marca además con una etiqueta de Git (F1.4). Validado el 21/10: la Sesión 1 (A02) vio la versión en Ajustes, CHANGELOG tiene cada versión y existen las etiquetas v0.1.5, v0.2.3 y v0.3.3 de los cierres de F1, F2 y F3 (las creaste tú en GitHub).</t>
+          <t>Vincula cada versión con su fase del roadmap. Cada fase cerrada se marca además con una etiqueta de Git (F1.4). Validado el 21/10: la Sesión 1 (A02) vio la versión en Ajustes, CHANGELOG tiene cada versión y existen las etiquetas v0.1.5, v0.2.3 y v0.3.3 de los cierres de F1, F2 y F3 (las creaste tú en GitHub). Fase reabierta (AR-14 #6): su trabajo numera con la fase más alta que ya esté en main (F5.8 sale como 0.6.1), y su etiqueta de cierre (v0.5.x) se pone en el commit que la cierra, aunque la app sea 0.6.n.</t>
         </is>
       </c>
       <c r="P14" s="6" t="n"/>
-      <c r="Q14" s="5" t="inlineStr"/>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="63" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -6835,11 +6839,15 @@
       </c>
       <c r="O83" s="5" t="inlineStr">
         <is>
-          <t>Tu petición del 21/10 y tu guía con la app que nos enseñaste: lo más directo. Se usa igual en vertical y en horizontal: como el Afinador, no pide girar el móvil. La barra se mueve también con las flechas del teclado. Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2). Verificado parcialmente: lo sostiene el banco hasta que lo compruebes tú (Sesión 2), igual que las escalas (CP-5, AR-12 #1). Pendiente (CP-5): mostrar qué figura cuenta el tempo («♩. = 80» en 6/8) y citar en el criterio los tramos de los nombres italianos (AR-12 #11).</t>
+          <t>Tu petición del 21/10 y tu guía con la app que nos enseñaste: lo más directo. Se usa igual en vertical y en horizontal: como el Afinador, no pide girar el móvil. La barra se mueve también con las flechas del teclado. Hecho en la 0.5.4 y validado por el banco; falta que lo uses con la guitarra (Sesión 2). Verificado parcialmente: lo sostiene el banco hasta que lo compruebes tú (Sesión 2), igual que las escalas (CP-5, AR-12 #1). Pendiente (CP-5): mostrar qué figura cuenta el tempo («♩. = 80» en 6/8) y citar en el criterio los tramos de los nombres italianos (AR-12 #11). Desde la 0.6.1 la barra es un péndulo y la pesa arriba va más lenta (antes, más rápida): ver MT-06.</t>
         </is>
       </c>
       <c r="P83" s="6" t="n"/>
-      <c r="Q83" s="5" t="inlineStr"/>
+      <c r="Q83" s="5" t="inlineStr">
+        <is>
+          <t>Modificado</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="108" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
@@ -7170,7 +7178,7 @@
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>La barra del tempo es un péndulo, como la de un metrónomo mecánico: la pesa marca el tempo, arriba más lento y abajo más rápido; mientras suena, la barra oscila sobre su pie y llega a un extremo en cada pulso, alternando los lados, hasta 30° a cada lado sin salirse de la pantalla. Se queda recta parada, mientras se arrastra y con «reducir movimiento».</t>
+          <t>La barra del tempo es un péndulo, como la de un metrónomo mecánico: la pesa marca el tempo, arriba más lento y abajo más rápido; mientras suena, la barra oscila sobre su pie y llega a un extremo en cada pulso, alternando los lados, hasta 30° a cada lado sin salirse de la pantalla. Se queda recta parada, mientras se arrastra y con «reducir movimiento». Tocar la pesa donde se ve, aunque esté inclinada, no cambia el tempo; solo arrastrarla.</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
@@ -7200,7 +7208,7 @@
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>Pesa arriba, 30 ppm, y abajo, 250. Sonando, la barra llega a un extremo en cada pulso, alternando los lados (hasta 30° a cada lado, sin salirse de la pantalla en ninguna disposición), y pasa por el centro entre dos; la subdivisión no la mueve. Recta parada, al arrastrarla y con «reducir movimiento».</t>
+          <t>Pesa arriba, 30 ppm, y abajo, 250. Sonando, la barra llega a un extremo en cada pulso, alternando los lados (hasta 30° a cada lado, sin salirse de la pantalla en ninguna disposición), y pasa por el centro entre dos; la subdivisión no la mueve. Recta parada, al arrastrarla y con «reducir movimiento». En el instante de cada pulso está en su extremo (±0,2° en el banco). Tocar la pesa donde se ve, aunque esté inclinada, no cambia el tempo. Con el teclado, ↑ sube el tempo.</t>
         </is>
       </c>
       <c r="J88" s="5" t="inlineStr">
@@ -7215,7 +7223,7 @@
       </c>
       <c r="L88" s="5" t="inlineStr">
         <is>
-          <t>Banco (node --test): extremos alternos en cada pulso, centro a medio camino, la subdivisión no cuenta, recta al arrastrar, al parar y con «reducir movimiento», pesa arriba = 30 ppm, amplitud que cabe; las tres pruebas fallan con la 0.6.0 · Chromium: ±30° en iPhone vertical y ordenador, ±12,7° en horizontal, nunca fuera de la pantalla · comprobar-disposicion: ocho pantallas del metrónomo</t>
+          <t>Banco (node --test): extremos alternos en cada pulso, centro a medio camino, la subdivisión no cuenta (4/4 en corcheas y 6/8), recta al arrastrar, al parar, al perder el dedo y con «reducir movimiento», pesa arriba = 30 ppm y abajo = 250, tocar la pesa inclinada no la mueve, amplitud que cabe y que se mide de nuevo tras girar en otra área, sin salto al cambiar de tempo en marcha, cambiar de compás no pierde pulsos; las pruebas fallan con la versión anterior · Chromium: ±30° en iPhone vertical y ordenador, ±12,7° en horizontal, y 12,7° al volver tras girar en otra área, nunca fuera de la pantalla · comprobar-disposicion: ocho pantallas del metrónomo · AR-14 y AT-13</t>
         </is>
       </c>
       <c r="M88" s="5" t="inlineStr">
@@ -7230,7 +7238,7 @@
       </c>
       <c r="O88" s="5" t="inlineStr">
         <is>
-          <t>Tu comentario de uso del 22/10 (F5.8 #1) y tu decisión del mismo día: la pesa arriba va más lenta, como en uno mecánico (antes, arriba era más rápido). El ángulo sale del reloj de audio, el mismo de los golpes, así que va con el sonido aunque el navegador vaya a tirones; sigue un coseno, como un péndulo: rápido en el centro y lento en los extremos. La subdivisión no lo mueve: solo los pulsos. Se abre menos si no cabe: en el iPhone en horizontal, unos 13°. Recto con «reducir movimiento» (G-05). Las flechas del teclado siguen la norma de los deslizadores (↑, más rápido). Hecho en la 0.6.1 y comprobado con el banco y en Chromium; verificado parcialmente hasta que lo pruebes tú (Sesión 2).</t>
+          <t>Tu comentario de uso del 22/10 (F5.8 #1) y tu decisión del mismo día: la pesa arriba va más lenta, como en uno mecánico (antes, arriba era más rápido). El ángulo sale del reloj de audio, el mismo de los golpes, así que va con el sonido aunque el navegador vaya a tirones; sigue un coseno, como un péndulo: rápido en el centro y lento en los extremos. La subdivisión no lo mueve: solo los pulsos. Se abre menos si no cabe: en el iPhone en horizontal, unos 13°. Recto con «reducir movimiento» (G-05). Las flechas del teclado siguen la norma de los deslizadores (↑, más rápido). Hecho en la 0.6.1 y comprobado con el banco y en Chromium; verificado parcialmente hasta que lo pruebes tú (Sesión 2). Auditorías AR-14 y AT-13, corregido en la ronda 1: tocar la pesa inclinada no cambia el tempo (el toque se proyecta sobre la varilla); girar el móvil con el metrónomo sonando en otra área ya no deja el péndulo demasiado abierto; un cambio grande de tempo en marcha no lo hace saltar (se mide hasta el pulso siguiente de verdad), y cambiar de compás no le hace perder pulsos. Pendiente de tu decisión (AR-14 #2 y #8): en horizontal, aceptar unos 13° o acortar allí la varilla para acercarse a 30°; y si con el teclado ↑ debe subir el tempo (norma) o subir la pesa. Anotado: le afecta AT-11 #5 (el dibujo no descuenta la latencia de salida; con auriculares Bluetooth el péndulo llegaría al extremo antes que el clic) y, en la Sesión 2, comprobar a 60 ppm en vertical, en horizontal y en el PC que la varilla llega al lado con el clic, que el vaivén parece un metrónomo y que va fluido en el iPhone (AR-14 #4, AT-13 #5).</t>
         </is>
       </c>
       <c r="P88" s="6" t="n"/>
@@ -10067,7 +10075,7 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>F5.8, tu comentario #1: MT-06 nuevo, el péndulo del metrónomo (la pesa arriba, más lento). Verificado parcialmente hasta la Sesión 2.</t>
+          <t>F5.8, tu comentario #1: MT-06 nuevo, el péndulo del metrónomo (la pesa arriba, más lento), con las correcciones de AR-14 y AT-13. Verificado parcialmente hasta la Sesión 2. MT-01 y G-10, anotados.</t>
         </is>
       </c>
     </row>

</xml_diff>